<commit_message>
inactive players run update
</commit_message>
<xml_diff>
--- a/data/playoff_odds.xlsx
+++ b/data/playoff_odds.xlsx
@@ -601,13 +601,13 @@
         <v>1</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.72</v>
+        <v>0.752</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.278</v>
+        <v>0.243</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.002</v>
+        <v>0.005</v>
       </c>
       <c r="G2" s="2" t="n"/>
       <c r="H2" s="2" t="n"/>
@@ -638,13 +638,13 @@
         <v>1</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>0.28</v>
+        <v>0.246</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0.6929999999999999</v>
+        <v>0.726</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>0.027</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="4">
@@ -659,12 +659,14 @@
       <c r="C4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="2" t="n"/>
+      <c r="D4" s="3" t="n">
+        <v>0.002</v>
+      </c>
       <c r="E4" s="3" t="n">
-        <v>0.029</v>
+        <v>0.031</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.971</v>
+        <v>0.967</v>
       </c>
       <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="n"/>
@@ -695,13 +697,13 @@
         <v>1</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.752</v>
+        <v>0.782</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0.242</v>
+        <v>0.215</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>0.006</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="6">
@@ -720,18 +722,20 @@
       <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="n"/>
       <c r="G6" s="3" t="n">
-        <v>0.244</v>
+        <v>0.216</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.72</v>
+        <v>0.748</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.033</v>
+        <v>0.034</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.003</v>
-      </c>
-      <c r="K6" s="2" t="n"/>
+        <v>0.001</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>0.001</v>
+      </c>
       <c r="L6" s="2" t="n"/>
       <c r="M6" s="2" t="n"/>
       <c r="N6" s="2" t="n"/>
@@ -756,34 +760,34 @@
         <v>1</v>
       </c>
       <c r="G7" s="4" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>0.556</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>0.259</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="M7" s="4" t="n">
         <v>0.003</v>
       </c>
-      <c r="H7" s="4" t="n">
-        <v>0.023</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>0.516</v>
-      </c>
-      <c r="J7" s="4" t="n">
-        <v>0.283</v>
-      </c>
-      <c r="K7" s="4" t="n">
-        <v>0.145</v>
-      </c>
-      <c r="L7" s="4" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="M7" s="4" t="n">
-        <v>0.004</v>
-      </c>
-      <c r="O7" s="4" t="n">
+      <c r="N7" s="4" t="n">
         <v>0.001</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Антуан Гризманн</t>
+          <t>Котяра</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -797,30 +801,32 @@
       <c r="F8" s="2" t="n"/>
       <c r="G8" s="2" t="n"/>
       <c r="H8" s="3" t="n">
-        <v>0.008</v>
+        <v>0.002</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>0.218</v>
+        <v>0.193</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.343</v>
+        <v>0.328</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>0.333</v>
+        <v>0.334</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>0.078</v>
+        <v>0.103</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>0.015</v>
+        <v>0.022</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>0.004</v>
+        <v>0.011</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="P8" s="2" t="n"/>
+        <v>0.005</v>
+      </c>
+      <c r="P8" s="3" t="n">
+        <v>0.002</v>
+      </c>
       <c r="Q8" s="2" t="n"/>
       <c r="R8" s="2" t="n"/>
       <c r="S8" s="2" t="n"/>
@@ -830,7 +836,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Котяра</t>
+          <t>Драйв</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -839,41 +845,44 @@
       <c r="C9" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="I9" s="4" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>0.116</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>0.287</v>
+      </c>
+      <c r="M9" s="4" t="n">
+        <v>0.154</v>
+      </c>
+      <c r="N9" s="4" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="O9" s="4" t="n">
+        <v>0.121</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="Q9" s="4" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="R9" s="4" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="S9" s="4" t="n">
         <v>0.001</v>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="I9" s="4" t="n">
-        <v>0.217</v>
-      </c>
-      <c r="J9" s="4" t="n">
-        <v>0.309</v>
-      </c>
-      <c r="K9" s="4" t="n">
-        <v>0.337</v>
-      </c>
-      <c r="L9" s="4" t="n">
-        <v>0.082</v>
-      </c>
-      <c r="M9" s="4" t="n">
-        <v>0.029</v>
-      </c>
-      <c r="N9" s="4" t="n">
-        <v>0.011</v>
-      </c>
-      <c r="O9" s="4" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="P9" s="4" t="n">
-        <v>0.002</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Драйв</t>
+          <t>E_ishutkin</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -887,36 +896,28 @@
       <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="n"/>
       <c r="H10" s="2" t="n"/>
-      <c r="I10" s="3" t="n">
-        <v>0.006</v>
-      </c>
-      <c r="J10" s="3" t="n">
-        <v>0.039</v>
-      </c>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="n"/>
       <c r="K10" s="3" t="n">
-        <v>0.103</v>
+        <v>0.003</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0.287</v>
+        <v>0.134</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>0.167</v>
+        <v>0.352</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.138</v>
+        <v>0.326</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>0.129</v>
+        <v>0.155</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>0.083</v>
-      </c>
-      <c r="Q10" s="3" t="n">
-        <v>0.043</v>
-      </c>
-      <c r="R10" s="3" t="n">
-        <v>0.005</v>
-      </c>
+        <v>0.03</v>
+      </c>
+      <c r="Q10" s="2" t="n"/>
+      <c r="R10" s="2" t="n"/>
       <c r="S10" s="2" t="n"/>
       <c r="T10" s="2" t="n"/>
       <c r="U10" s="2" t="n"/>
@@ -924,7 +925,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>E_ishutkin</t>
+          <t>clayzid</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -933,32 +934,47 @@
       <c r="C11" s="4" t="n">
         <v>1</v>
       </c>
+      <c r="I11" s="4" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>0.01</v>
+      </c>
       <c r="K11" s="4" t="n">
-        <v>0.003</v>
+        <v>0.047</v>
       </c>
       <c r="L11" s="4" t="n">
-        <v>0.159</v>
+        <v>0.128</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>0.376</v>
+        <v>0.156</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>0.333</v>
+        <v>0.163</v>
       </c>
       <c r="O11" s="4" t="n">
-        <v>0.102</v>
+        <v>0.179</v>
       </c>
       <c r="P11" s="4" t="n">
-        <v>0.026</v>
+        <v>0.165</v>
       </c>
       <c r="Q11" s="4" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="R11" s="4" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="S11" s="4" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="T11" s="4" t="n">
         <v>0.001</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>clayzid</t>
+          <t>Бэндер</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -972,32 +988,30 @@
       <c r="F12" s="2" t="n"/>
       <c r="G12" s="2" t="n"/>
       <c r="H12" s="2" t="n"/>
-      <c r="I12" s="3" t="n">
-        <v>0.002</v>
-      </c>
+      <c r="I12" s="2" t="n"/>
       <c r="J12" s="3" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0.034</v>
+        <v>0.032</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>0.149</v>
+        <v>0.117</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0.145</v>
+        <v>0.148</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.148</v>
+        <v>0.157</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.189</v>
+        <v>0.174</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>0.173</v>
+        <v>0.178</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>0.111</v>
+        <v>0.146</v>
       </c>
       <c r="R12" s="3" t="n">
         <v>0.039</v>
@@ -1011,7 +1025,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Бэндер</t>
+          <t>Кинзу</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1020,38 +1034,38 @@
       <c r="C13" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I13" s="4" t="n">
+      <c r="J13" s="4" t="n">
         <v>0.001</v>
       </c>
-      <c r="J13" s="4" t="n">
-        <v>0.011</v>
-      </c>
       <c r="K13" s="4" t="n">
-        <v>0.025</v>
+        <v>0.012</v>
       </c>
       <c r="L13" s="4" t="n">
-        <v>0.118</v>
+        <v>0.051</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>0.122</v>
+        <v>0.066</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>0.147</v>
+        <v>0.083</v>
       </c>
       <c r="O13" s="4" t="n">
-        <v>0.204</v>
+        <v>0.177</v>
       </c>
       <c r="P13" s="4" t="n">
-        <v>0.189</v>
+        <v>0.219</v>
       </c>
       <c r="Q13" s="4" t="n">
-        <v>0.137</v>
+        <v>0.292</v>
       </c>
       <c r="R13" s="4" t="n">
-        <v>0.038</v>
+        <v>0.073</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>0.007</v>
+        <v>0.023</v>
+      </c>
+      <c r="T13" s="4" t="n">
+        <v>0.002</v>
       </c>
       <c r="U13" s="4" t="n">
         <v>0.001</v>
@@ -1060,106 +1074,98 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>ksuhony</t>
+          <t>Антуан Гризманн</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
         <v>13</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>1</v>
+        <v>0.9999999999999999</v>
       </c>
       <c r="D14" s="2" t="n"/>
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="2" t="n"/>
       <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
+      <c r="H14" s="3" t="n">
+        <v>0.003</v>
+      </c>
       <c r="I14" s="3" t="n">
+        <v>0.204</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>0.358</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="L14" s="3" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="M14" s="3" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="N14" s="3" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="O14" s="3" t="n">
         <v>0.001</v>
       </c>
-      <c r="J14" s="3" t="n">
-        <v>0.004</v>
-      </c>
-      <c r="K14" s="3" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="L14" s="3" t="n">
-        <v>0.066</v>
-      </c>
-      <c r="M14" s="3" t="n">
-        <v>0.082</v>
-      </c>
-      <c r="N14" s="3" t="n">
-        <v>0.131</v>
-      </c>
-      <c r="O14" s="3" t="n">
-        <v>0.179</v>
-      </c>
       <c r="P14" s="3" t="n">
-        <v>0.228</v>
-      </c>
-      <c r="Q14" s="3" t="n">
-        <v>0.221</v>
-      </c>
-      <c r="R14" s="3" t="n">
-        <v>0.059</v>
-      </c>
-      <c r="S14" s="3" t="n">
-        <v>0.011</v>
-      </c>
-      <c r="T14" s="3" t="n">
         <v>0.001</v>
       </c>
-      <c r="U14" s="3" t="n">
-        <v>0.002</v>
-      </c>
+      <c r="Q14" s="2" t="n"/>
+      <c r="R14" s="2" t="n"/>
+      <c r="S14" s="2" t="n"/>
+      <c r="T14" s="2" t="n"/>
+      <c r="U14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Кинзу</t>
+          <t>ksuhony</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>14</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1</v>
+        <v>0.999</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>0.001</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>0.005</v>
+        <v>0.012</v>
       </c>
       <c r="L15" s="4" t="n">
-        <v>0.035</v>
+        <v>0.067</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>0.057</v>
+        <v>0.077</v>
       </c>
       <c r="N15" s="4" t="n">
-        <v>0.08</v>
+        <v>0.118</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>0.163</v>
+        <v>0.166</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>0.244</v>
+        <v>0.251</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>0.294</v>
+        <v>0.24</v>
       </c>
       <c r="R15" s="4" t="n">
-        <v>0.102</v>
+        <v>0.053</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.012</v>
+        <v>0.008</v>
       </c>
       <c r="T15" s="4" t="n">
-        <v>0.004</v>
-      </c>
-      <c r="U15" s="4" t="n">
         <v>0.002</v>
       </c>
     </row>
@@ -1173,7 +1179,7 @@
         <v>15</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>0.981</v>
+        <v>0.9760000000000001</v>
       </c>
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
@@ -1183,35 +1189,33 @@
       <c r="I16" s="2" t="n"/>
       <c r="J16" s="2" t="n"/>
       <c r="K16" s="2" t="n"/>
-      <c r="L16" s="3" t="n">
-        <v>0.001</v>
-      </c>
+      <c r="L16" s="2" t="n"/>
       <c r="M16" s="3" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0.007</v>
+        <v>0.004</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>0.024</v>
+        <v>0.021</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>0.049</v>
+        <v>0.045</v>
       </c>
       <c r="Q16" s="3" t="n">
-        <v>0.147</v>
+        <v>0.119</v>
       </c>
       <c r="R16" s="3" t="n">
-        <v>0.454</v>
+        <v>0.452</v>
       </c>
       <c r="S16" s="3" t="n">
-        <v>0.195</v>
+        <v>0.2</v>
       </c>
       <c r="T16" s="3" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.093</v>
       </c>
       <c r="U16" s="3" t="n">
-        <v>0.029</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="17">
@@ -1224,31 +1228,31 @@
         <v>16</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>0.7950000000000002</v>
+        <v>0.7889999999999999</v>
       </c>
       <c r="N17" s="4" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="O17" s="4" t="n">
         <v>0.001</v>
       </c>
-      <c r="O17" s="4" t="n">
-        <v>0.002</v>
-      </c>
       <c r="P17" s="4" t="n">
-        <v>0.006</v>
+        <v>0.003</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>0.026</v>
+        <v>0.018</v>
       </c>
       <c r="R17" s="4" t="n">
-        <v>0.132</v>
+        <v>0.129</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.272</v>
+        <v>0.235</v>
       </c>
       <c r="T17" s="4" t="n">
-        <v>0.197</v>
+        <v>0.222</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.159</v>
+        <v>0.179</v>
       </c>
     </row>
     <row r="18">
@@ -1261,7 +1265,7 @@
         <v>17</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>0.734</v>
+        <v>0.73</v>
       </c>
       <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="n"/>
@@ -1274,24 +1278,24 @@
       <c r="L18" s="2" t="n"/>
       <c r="M18" s="2" t="n"/>
       <c r="N18" s="2" t="n"/>
-      <c r="O18" s="3" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="P18" s="2" t="n"/>
+      <c r="O18" s="2" t="n"/>
+      <c r="P18" s="3" t="n">
+        <v>0.006</v>
+      </c>
       <c r="Q18" s="3" t="n">
-        <v>0.012</v>
+        <v>0.014</v>
       </c>
       <c r="R18" s="3" t="n">
-        <v>0.076</v>
+        <v>0.09</v>
       </c>
       <c r="S18" s="3" t="n">
-        <v>0.18</v>
+        <v>0.205</v>
       </c>
       <c r="T18" s="3" t="n">
-        <v>0.253</v>
+        <v>0.213</v>
       </c>
       <c r="U18" s="3" t="n">
-        <v>0.212</v>
+        <v>0.202</v>
       </c>
     </row>
     <row r="19">
@@ -1304,7 +1308,7 @@
         <v>18</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.524</v>
+        <v>0.5529999999999999</v>
       </c>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
@@ -1318,21 +1322,23 @@
       <c r="M19" s="5" t="n"/>
       <c r="N19" s="5" t="n"/>
       <c r="O19" s="5" t="n"/>
-      <c r="P19" s="5" t="n"/>
+      <c r="P19" s="6" t="n">
+        <v>0.001</v>
+      </c>
       <c r="Q19" s="6" t="n">
-        <v>0.001</v>
+        <v>0.004</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>0.04</v>
+        <v>0.055</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>0.105</v>
+        <v>0.134</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>0.191</v>
+        <v>0.161</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>0.187</v>
+        <v>0.198</v>
       </c>
     </row>
     <row r="20">
@@ -1345,7 +1351,7 @@
         <v>19</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>0.457</v>
+        <v>0.468</v>
       </c>
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="n"/>
@@ -1361,19 +1367,19 @@
       <c r="O20" s="2" t="n"/>
       <c r="P20" s="2" t="n"/>
       <c r="Q20" s="3" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>0.026</v>
+        <v>0.035</v>
       </c>
       <c r="S20" s="3" t="n">
-        <v>0.112</v>
+        <v>0.097</v>
       </c>
       <c r="T20" s="3" t="n">
-        <v>0.126</v>
+        <v>0.142</v>
       </c>
       <c r="U20" s="3" t="n">
-        <v>0.189</v>
+        <v>0.191</v>
       </c>
     </row>
     <row r="21">
@@ -1386,22 +1392,28 @@
         <v>20</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>0.426</v>
+        <v>0.415</v>
+      </c>
+      <c r="M21" s="4" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="P21" s="4" t="n">
+        <v>0.001</v>
       </c>
       <c r="Q21" s="4" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="R21" s="4" t="n">
-        <v>0.027</v>
+        <v>0.038</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.096</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="T21" s="4" t="n">
-        <v>0.13</v>
+        <v>0.138</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.17</v>
+        <v>0.148</v>
       </c>
     </row>
     <row r="22">
@@ -1414,7 +1426,7 @@
         <v>21</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>0.07400000000000001</v>
+        <v>0.062</v>
       </c>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
@@ -1434,38 +1446,38 @@
         <v>0.002</v>
       </c>
       <c r="S22" s="3" t="n">
-        <v>0.006</v>
+        <v>0.001</v>
       </c>
       <c r="T22" s="3" t="n">
         <v>0.025</v>
       </c>
       <c r="U22" s="3" t="n">
-        <v>0.041</v>
+        <v>0.034</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Amaney</t>
+          <t>Mihmbox</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>22</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>0.006</v>
+        <v>0.003</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.001</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.005</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Сокол</t>
+          <t>sl1dbygad</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1498,29 +1510,31 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>sl1dbygad</t>
+          <t>Amaney</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>24</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Mihmbox</t>
+          <t>Сокол</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="C26" s="2" t="n"/>
+      <c r="C26" s="3" t="n">
+        <v>0.001</v>
+      </c>
       <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="n"/>
       <c r="F26" s="2" t="n"/>
@@ -1538,7 +1552,9 @@
       <c r="R26" s="2" t="n"/>
       <c r="S26" s="2" t="n"/>
       <c r="T26" s="2" t="n"/>
-      <c r="U26" s="2" t="n"/>
+      <c r="U26" s="3" t="n">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1660,7 +1676,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Bushido</t>
+          <t>EliasPavlov</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1670,7 +1686,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>EliasPavlov</t>
+          <t>Bushido</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1787,7 +1803,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>@TryFraiz</t>
+          <t>rusya6996</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -1816,7 +1832,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>rusya6996</t>
+          <t>@TryFraiz</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1865,7 +1881,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>SPQR</t>
+          <t>Chinaski</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -1894,7 +1910,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Chinaski</t>
+          <t>SPQR</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1904,7 +1920,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Комарик</t>
+          <t>nesmotri_v_shelll1</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -1933,7 +1949,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>nesmotri_v_shelll1</t>
+          <t>Дядя Витя</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1972,7 +1988,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Дядя Витя</t>
+          <t>Тихоня</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1982,7 +1998,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Тихоня</t>
+          <t>dialse</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2011,7 +2027,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>dialse</t>
+          <t>ArutunyanArsen</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2021,7 +2037,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>MMM</t>
+          <t>Chesters</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2050,7 +2066,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Chesters</t>
+          <t>MMM</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2060,7 +2076,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>ArutunyanArsen</t>
+          <t>gamma</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2099,7 +2115,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>gamma</t>
+          <t>FISHer</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -2128,7 +2144,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>FISHer</t>
+          <t>lavr</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2138,7 +2154,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>lavr</t>
+          <t>Добряк</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -2167,7 +2183,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Добряк</t>
+          <t>ЛЕНИН</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -2177,7 +2193,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>ЛЕНИН</t>
+          <t>Акоп</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -2206,7 +2222,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Акоп</t>
+          <t>Чейз</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -2216,7 +2232,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Чейз</t>
+          <t>maria_merlot</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -2245,7 +2261,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>maria_merlot</t>
+          <t>Андрюха Пират</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -2284,7 +2300,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Андрюха Пират</t>
+          <t>jieb</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -2294,7 +2310,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>jieb</t>
+          <t>kirienish</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -2323,7 +2339,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>kirienish</t>
+          <t>aisel_gizatova</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -2333,7 +2349,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>egoist</t>
+          <t>ЭтоМойНик</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -2362,7 +2378,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>aisel_gizatova</t>
+          <t>egoist</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -2372,7 +2388,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>ЭтоМойНик</t>
+          <t>Afteromanov</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -2401,7 +2417,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Afteromanov</t>
+          <t>Никитос</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -2440,7 +2456,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Никитос</t>
+          <t>кинчоч</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -2450,7 +2466,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>кинчоч</t>
+          <t>Сан Саныч</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -2489,7 +2505,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Сан Саныч</t>
+          <t>bogdansskii</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -2528,7 +2544,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>bogdansskii</t>
+          <t>Serg</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -2557,7 +2573,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Serg</t>
+          <t>Staryii</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -2567,7 +2583,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Staryii</t>
+          <t>Danila158</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -2596,7 +2612,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Danila158</t>
+          <t>Комарик</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -2635,7 +2651,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ustayonmymind</t>
+          <t>Al</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -2674,7 +2690,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Al</t>
+          <t>sushk0v_aa</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -2684,7 +2700,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>sushk0v_aa</t>
+          <t>ustayonmymind</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -2762,7 +2778,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Абеляр</t>
+          <t>Retbin</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -2791,7 +2807,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Retbin</t>
+          <t>Игорь</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -2801,7 +2817,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Игорь</t>
+          <t>Абеляр</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
@@ -2879,7 +2895,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>desssai</t>
+          <t>Gluckspilz8</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -2908,7 +2924,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>mkrnnv</t>
+          <t>desssai</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -2918,7 +2934,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>xairullah</t>
+          <t>DmitryParf</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -2947,7 +2963,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Gluckspilz8</t>
+          <t>xairullah</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2957,7 +2973,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Владимир</t>
+          <t>Ромчик</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -2986,7 +3002,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>DmitryParf</t>
+          <t>Владимир</t>
         </is>
       </c>
       <c r="B101" t="n">

</xml_diff>

<commit_message>
multiplier and name fix
</commit_message>
<xml_diff>
--- a/data/playoff_odds.xlsx
+++ b/data/playoff_odds.xlsx
@@ -598,59 +598,57 @@
         <v>1</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>1</v>
+        <v>0.298</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.18</v>
+        <v>0.155</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.144</v>
+        <v>0.141</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.105</v>
+        <v>0.121</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>0.092</v>
+        <v>0.095</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>0.079</v>
+        <v>0.081</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0.081</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.064</v>
+        <v>0.077</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>0.048</v>
+        <v>0.073</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>0.052</v>
+        <v>0.057</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>0.06</v>
+        <v>0.037</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>0.037</v>
+        <v>0.03</v>
       </c>
       <c r="O2" s="3" t="n">
-        <v>0.03</v>
+        <v>0.017</v>
       </c>
       <c r="P2" s="3" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="Q2" s="3" t="n">
         <v>0.01</v>
       </c>
-      <c r="Q2" s="3" t="n">
+      <c r="R2" s="3" t="n">
         <v>0.007</v>
       </c>
-      <c r="R2" s="3" t="n">
+      <c r="S2" s="3" t="n">
         <v>0.004</v>
       </c>
-      <c r="S2" s="3" t="n">
-        <v>0.003</v>
-      </c>
-      <c r="T2" s="3" t="n">
-        <v>0.002</v>
-      </c>
+      <c r="T2" s="2" t="n"/>
       <c r="U2" s="2" t="n"/>
     </row>
     <row r="3">
@@ -663,55 +661,61 @@
         <v>2</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1</v>
+        <v>0.298</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>0.164</v>
+        <v>0.141</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0.124</v>
+        <v>0.137</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>0.123</v>
+        <v>0.102</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.093</v>
+        <v>0.098</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>0.078</v>
+        <v>0.097</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>0.068</v>
+        <v>0.073</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.063</v>
       </c>
       <c r="L3" s="4" t="n">
-        <v>0.054</v>
+        <v>0.058</v>
       </c>
       <c r="M3" s="4" t="n">
-        <v>0.043</v>
+        <v>0.059</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>0.033</v>
+        <v>0.037</v>
       </c>
       <c r="O3" s="4" t="n">
-        <v>0.028</v>
+        <v>0.029</v>
       </c>
       <c r="P3" s="4" t="n">
-        <v>0.016</v>
+        <v>0.02</v>
       </c>
       <c r="Q3" s="4" t="n">
-        <v>0.008</v>
+        <v>0.004</v>
       </c>
       <c r="R3" s="4" t="n">
         <v>0.007</v>
       </c>
       <c r="S3" s="4" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="T3" s="4" t="n">
         <v>0.003</v>
+      </c>
+      <c r="U3" s="4" t="n">
+        <v>0.001</v>
       </c>
     </row>
     <row r="4">
@@ -724,46 +728,46 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>1</v>
+        <v>0.298</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.126</v>
+        <v>0.134</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.111</v>
+        <v>0.113</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.106</v>
+        <v>0.097</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0.09</v>
+        <v>0.091</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.098</v>
+        <v>0.081</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.094</v>
+        <v>0.102</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.074</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>0.066</v>
+        <v>0.081</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>0.065</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>0.053</v>
+        <v>0.063</v>
       </c>
       <c r="N4" s="3" t="n">
         <v>0.038</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>0.039</v>
+        <v>0.026</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>0.024</v>
+        <v>0.017</v>
       </c>
       <c r="Q4" s="3" t="n">
         <v>0.007</v>
@@ -772,12 +776,12 @@
         <v>0.004</v>
       </c>
       <c r="S4" s="3" t="n">
-        <v>0.004</v>
-      </c>
-      <c r="T4" s="2" t="n"/>
-      <c r="U4" s="3" t="n">
-        <v>0.001</v>
-      </c>
+        <v>0.003</v>
+      </c>
+      <c r="T4" s="3" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="U4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -789,122 +793,122 @@
         <v>4</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1</v>
+        <v>0.298</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>0.097</v>
+        <v>0.094</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0.097</v>
+        <v>0.118</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>0.095</v>
       </c>
       <c r="G5" s="4" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="I5" s="4" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="H5" s="4" t="n">
-        <v>0.096</v>
-      </c>
-      <c r="I5" s="4" t="n">
-        <v>0.095</v>
-      </c>
       <c r="J5" s="4" t="n">
-        <v>0.082</v>
+        <v>0.064</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>0.083</v>
+        <v>0.061</v>
       </c>
       <c r="L5" s="4" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>0.055</v>
+        <v>0.066</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v>0.047</v>
+        <v>0.057</v>
       </c>
       <c r="O5" s="4" t="n">
-        <v>0.039</v>
+        <v>0.037</v>
       </c>
       <c r="P5" s="4" t="n">
-        <v>0.026</v>
+        <v>0.027</v>
       </c>
       <c r="Q5" s="4" t="n">
-        <v>0.018</v>
+        <v>0.017</v>
       </c>
       <c r="R5" s="4" t="n">
-        <v>0.01</v>
+        <v>0.014</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="T5" s="4" t="n">
-        <v>0.003</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Пассажир</t>
+          <t>кинчоч</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>1</v>
+        <v>0.298</v>
       </c>
       <c r="D6" s="3" t="n">
+        <v>0.099</v>
+      </c>
+      <c r="E6" s="3" t="n">
         <v>0.075</v>
       </c>
-      <c r="E6" s="3" t="n">
-        <v>0.092</v>
-      </c>
       <c r="F6" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0.073</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="I6" s="3" t="n">
         <v>0.08599999999999999</v>
       </c>
-      <c r="G6" s="3" t="n">
-        <v>0.097</v>
-      </c>
-      <c r="H6" s="3" t="n">
-        <v>0.08699999999999999</v>
-      </c>
-      <c r="I6" s="3" t="n">
-        <v>0.078</v>
-      </c>
       <c r="J6" s="3" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.082</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.075</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>0.077</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>0.055</v>
+        <v>0.068</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>0.048</v>
+        <v>0.057</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>0.058</v>
+        <v>0.038</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>0.035</v>
+        <v>0.039</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>0.021</v>
+        <v>0.023</v>
       </c>
       <c r="R6" s="3" t="n">
-        <v>0.01</v>
+        <v>0.011</v>
       </c>
       <c r="S6" s="3" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="T6" s="3" t="n">
         <v>0.003</v>
-      </c>
-      <c r="T6" s="3" t="n">
-        <v>0.004</v>
       </c>
       <c r="U6" s="3" t="n">
         <v>0.002</v>
@@ -913,465 +917,470 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>кинчоч</t>
+          <t>Пассажир</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>6</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1</v>
+        <v>0.298</v>
       </c>
       <c r="D7" s="4" t="n">
+        <v>0.077</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>0.073</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>0.083</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>0.079</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>0.068</v>
+      </c>
+      <c r="M7" s="4" t="n">
         <v>0.065</v>
       </c>
-      <c r="E7" s="4" t="n">
-        <v>0.077</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>0.091</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>0.089</v>
-      </c>
-      <c r="H7" s="4" t="n">
-        <v>0.08599999999999999</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>0.076</v>
-      </c>
-      <c r="J7" s="4" t="n">
-        <v>0.08500000000000001</v>
-      </c>
-      <c r="K7" s="4" t="n">
-        <v>0.082</v>
-      </c>
-      <c r="L7" s="4" t="n">
-        <v>0.078</v>
-      </c>
-      <c r="M7" s="4" t="n">
-        <v>0.068</v>
-      </c>
       <c r="N7" s="4" t="n">
-        <v>0.068</v>
+        <v>0.055</v>
       </c>
       <c r="O7" s="4" t="n">
-        <v>0.056</v>
+        <v>0.058</v>
       </c>
       <c r="P7" s="4" t="n">
-        <v>0.036</v>
+        <v>0.035</v>
       </c>
       <c r="Q7" s="4" t="n">
-        <v>0.017</v>
+        <v>0.027</v>
       </c>
       <c r="R7" s="4" t="n">
-        <v>0.016</v>
+        <v>0.014</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.007</v>
+        <v>0.005</v>
       </c>
       <c r="T7" s="4" t="n">
-        <v>0.003</v>
+        <v>0.005</v>
+      </c>
+      <c r="U7" s="4" t="n">
+        <v>0.002</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>dolMy</t>
+          <t>G_rant_999</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
         <v>7</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>1</v>
+        <v>0.298</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0.047</v>
+        <v>0.055</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.065</v>
+        <v>0.057</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0.067</v>
+        <v>0.074</v>
       </c>
       <c r="G8" s="3" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="I8" s="3" t="n">
         <v>0.08</v>
       </c>
-      <c r="H8" s="3" t="n">
-        <v>0.074</v>
-      </c>
-      <c r="I8" s="3" t="n">
+      <c r="J8" s="3" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="K8" s="3" t="n">
         <v>0.077</v>
       </c>
-      <c r="J8" s="3" t="n">
-        <v>0.07199999999999999</v>
-      </c>
-      <c r="K8" s="3" t="n">
-        <v>0.08500000000000001</v>
-      </c>
       <c r="L8" s="3" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>0.08</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>0.076</v>
+        <v>0.063</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>0.068</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>0.041</v>
+        <v>0.039</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>0.035</v>
+        <v>0.025</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>0.021</v>
+        <v>0.02</v>
       </c>
       <c r="S8" s="3" t="n">
-        <v>0.022</v>
+        <v>0.012</v>
       </c>
       <c r="T8" s="3" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="U8" s="3" t="n">
         <v>0.003</v>
-      </c>
-      <c r="U8" s="3" t="n">
-        <v>0.002</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Laches1</t>
+          <t>dolMy</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>8</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>1</v>
+        <v>0.298</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>0.044</v>
+        <v>0.046</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.052</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>0.062</v>
+        <v>0.074</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.083</v>
       </c>
       <c r="H9" s="4" t="n">
+        <v>0.079</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>0.074</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>0.08799999999999999</v>
+      </c>
+      <c r="K9" s="4" t="n">
         <v>0.073</v>
       </c>
-      <c r="I9" s="4" t="n">
+      <c r="L9" s="4" t="n">
         <v>0.075</v>
       </c>
-      <c r="J9" s="4" t="n">
-        <v>0.063</v>
-      </c>
-      <c r="K9" s="4" t="n">
-        <v>0.067</v>
-      </c>
-      <c r="L9" s="4" t="n">
-        <v>0.09</v>
-      </c>
       <c r="M9" s="4" t="n">
-        <v>0.101</v>
+        <v>0.079</v>
       </c>
       <c r="N9" s="4" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="O9" s="4" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.055</v>
       </c>
       <c r="P9" s="4" t="n">
-        <v>0.057</v>
+        <v>0.047</v>
       </c>
       <c r="Q9" s="4" t="n">
         <v>0.035</v>
       </c>
       <c r="R9" s="4" t="n">
-        <v>0.03</v>
+        <v>0.017</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.008</v>
+        <v>0.01</v>
       </c>
       <c r="T9" s="4" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.007</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>G_rant_999</t>
+          <t>Сокол</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
         <v>9</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.9990000000000001</v>
+        <v>0.298</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.055</v>
+        <v>0.051</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.057</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.056</v>
+        <v>0.067</v>
       </c>
       <c r="G10" s="3" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>0.083</v>
+      </c>
+      <c r="I10" s="3" t="n">
         <v>0.089</v>
       </c>
-      <c r="H10" s="3" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="I10" s="3" t="n">
+      <c r="J10" s="3" t="n">
+        <v>0.081</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>0.073</v>
+      </c>
+      <c r="M10" s="3" t="n">
         <v>0.077</v>
       </c>
-      <c r="J10" s="3" t="n">
-        <v>0.08599999999999999</v>
-      </c>
-      <c r="K10" s="3" t="n">
-        <v>0.08500000000000001</v>
-      </c>
-      <c r="L10" s="3" t="n">
-        <v>0.077</v>
-      </c>
-      <c r="M10" s="3" t="n">
-        <v>0.07099999999999999</v>
-      </c>
       <c r="N10" s="3" t="n">
-        <v>0.076</v>
+        <v>0.066</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>0.053</v>
+        <v>0.068</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>0.052</v>
+        <v>0.044</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>0.024</v>
+        <v>0.042</v>
       </c>
       <c r="R10" s="3" t="n">
-        <v>0.02</v>
+        <v>0.019</v>
       </c>
       <c r="S10" s="3" t="n">
-        <v>0.011</v>
+        <v>0.018</v>
       </c>
       <c r="T10" s="3" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="U10" s="2" t="n"/>
+        <v>0.01</v>
+      </c>
+      <c r="U10" s="3" t="n">
+        <v>0.002</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Сокол</t>
+          <t>Yanchik_250</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>10</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>0.999</v>
+        <v>0.297702</v>
       </c>
       <c r="D11" s="4" t="n">
         <v>0.048</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0.052</v>
+        <v>0.055</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>0.061</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>0.058</v>
+        <v>0.068</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>0.079</v>
+        <v>0.075</v>
       </c>
       <c r="I11" s="4" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>0.073</v>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>0.081</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="M11" s="4" t="n">
         <v>0.082</v>
       </c>
-      <c r="J11" s="4" t="n">
-        <v>0.099</v>
-      </c>
-      <c r="K11" s="4" t="n">
-        <v>0.08400000000000001</v>
-      </c>
-      <c r="L11" s="4" t="n">
-        <v>0.08799999999999999</v>
-      </c>
-      <c r="M11" s="4" t="n">
-        <v>0.07000000000000001</v>
-      </c>
       <c r="N11" s="4" t="n">
-        <v>0.09</v>
+        <v>0.062</v>
       </c>
       <c r="O11" s="4" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="P11" s="4" t="n">
         <v>0.07099999999999999</v>
       </c>
-      <c r="P11" s="4" t="n">
-        <v>0.042</v>
-      </c>
       <c r="Q11" s="4" t="n">
-        <v>0.033</v>
+        <v>0.038</v>
       </c>
       <c r="R11" s="4" t="n">
-        <v>0.013</v>
+        <v>0.02</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.018</v>
+        <v>0.02</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.005</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.004</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Yanchik_250</t>
+          <t>terzzzzzzzzz</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
         <v>11</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>0.9980000000000001</v>
+        <v>0.2974040000000001</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0.044</v>
+        <v>0.041</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.061</v>
+        <v>0.046</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.054</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0.068</v>
+        <v>0.064</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>0.077</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="J12" s="3" t="n">
+        <v>0.092</v>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>0.081</v>
+      </c>
+      <c r="L12" s="3" t="n">
+        <v>0.097</v>
+      </c>
+      <c r="M12" s="3" t="n">
         <v>0.083</v>
       </c>
-      <c r="K12" s="3" t="n">
-        <v>0.073</v>
-      </c>
-      <c r="L12" s="3" t="n">
-        <v>0.074</v>
-      </c>
-      <c r="M12" s="3" t="n">
-        <v>0.08</v>
-      </c>
       <c r="N12" s="3" t="n">
-        <v>0.079</v>
+        <v>0.097</v>
       </c>
       <c r="O12" s="3" t="n">
         <v>0.075</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>0.075</v>
+        <v>0.048</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>0.039</v>
+        <v>0.031</v>
       </c>
       <c r="R12" s="3" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="S12" s="3" t="n">
         <v>0.015</v>
       </c>
-      <c r="S12" s="3" t="n">
-        <v>0.012</v>
-      </c>
       <c r="T12" s="3" t="n">
-        <v>0.008</v>
+        <v>0.01</v>
       </c>
       <c r="U12" s="3" t="n">
-        <v>0.002</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>terzzzzzzzzz</t>
+          <t>Laches1</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>12</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>0.998</v>
+        <v>0.2971060000000001</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>0.053</v>
+        <v>0.057</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.052</v>
+        <v>0.051</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.058</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.08</v>
+        <v>0.067</v>
       </c>
       <c r="H13" s="4" t="n">
+        <v>0.07199999999999999</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="J13" s="4" t="n">
         <v>0.077</v>
       </c>
-      <c r="I13" s="4" t="n">
-        <v>0.07099999999999999</v>
-      </c>
-      <c r="J13" s="4" t="n">
-        <v>0.079</v>
-      </c>
       <c r="K13" s="4" t="n">
-        <v>0.1</v>
+        <v>0.083</v>
       </c>
       <c r="L13" s="4" t="n">
+        <v>0.078</v>
+      </c>
+      <c r="M13" s="4" t="n">
         <v>0.08599999999999999</v>
       </c>
-      <c r="M13" s="4" t="n">
-        <v>0.08699999999999999</v>
-      </c>
       <c r="N13" s="4" t="n">
-        <v>0.063</v>
+        <v>0.093</v>
       </c>
       <c r="O13" s="4" t="n">
         <v>0.067</v>
       </c>
       <c r="P13" s="4" t="n">
-        <v>0.048</v>
+        <v>0.05</v>
       </c>
       <c r="Q13" s="4" t="n">
-        <v>0.028</v>
+        <v>0.036</v>
       </c>
       <c r="R13" s="4" t="n">
-        <v>0.015</v>
+        <v>0.021</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>0.004</v>
+        <v>0.013</v>
       </c>
       <c r="T13" s="4" t="n">
-        <v>0.008</v>
+        <v>0.01</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.008</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="14">
@@ -1384,59 +1393,61 @@
         <v>13</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>0.9159999999999999</v>
+        <v>0.272372</v>
       </c>
       <c r="D14" s="3" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="E14" s="3" t="n">
         <v>0.002</v>
       </c>
-      <c r="E14" s="2" t="n"/>
       <c r="F14" s="3" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G14" s="3" t="n">
         <v>0.003</v>
-      </c>
-      <c r="G14" s="3" t="n">
-        <v>0.004</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>0.007</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.01</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0.015</v>
+        <v>0.018</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>0.023</v>
+        <v>0.018</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>0.024</v>
+        <v>0.028</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0.049</v>
+        <v>0.028</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>0.06</v>
+        <v>0.055</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.077</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>0.099</v>
+        <v>0.098</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>0.119</v>
+        <v>0.109</v>
       </c>
       <c r="R14" s="3" t="n">
-        <v>0.111</v>
+        <v>0.107</v>
       </c>
       <c r="S14" s="3" t="n">
-        <v>0.097</v>
+        <v>0.094</v>
       </c>
       <c r="T14" s="3" t="n">
-        <v>0.096</v>
+        <v>0.108</v>
       </c>
       <c r="U14" s="3" t="n">
-        <v>0.068</v>
+        <v>0.08799999999999999</v>
       </c>
     </row>
     <row r="15">
@@ -1449,182 +1460,174 @@
         <v>14</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>0.876</v>
+        <v>0.262538</v>
       </c>
       <c r="E15" s="4" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="H15" s="4" t="n">
         <v>0.001</v>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="G15" s="4" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="H15" s="4" t="n">
-        <v>0.004</v>
       </c>
       <c r="I15" s="4" t="n">
         <v>0.004</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>0.013</v>
+        <v>0.007</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>0.012</v>
+        <v>0.02</v>
       </c>
       <c r="L15" s="4" t="n">
-        <v>0.015</v>
+        <v>0.02</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>0.033</v>
+        <v>0.025</v>
       </c>
       <c r="N15" s="4" t="n">
-        <v>0.035</v>
+        <v>0.047</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>0.058</v>
+        <v>0.082</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>0.099</v>
+        <v>0.094</v>
       </c>
       <c r="R15" s="4" t="n">
-        <v>0.108</v>
+        <v>0.103</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.107</v>
+        <v>0.104</v>
       </c>
       <c r="T15" s="4" t="n">
-        <v>0.099</v>
+        <v>0.109</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.109</v>
+        <v>0.094</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Lock</t>
+          <t>Пиковая Дама</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
         <v>15</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>0.8519999999999999</v>
+        <v>0.2577700000000001</v>
       </c>
       <c r="D16" s="2" t="n"/>
-      <c r="E16" s="3" t="n">
-        <v>0.001</v>
-      </c>
+      <c r="E16" s="2" t="n"/>
       <c r="F16" s="3" t="n">
         <v>0.001</v>
       </c>
       <c r="G16" s="2" t="n"/>
       <c r="H16" s="3" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>0.004</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.008</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>0.007</v>
+        <v>0.013</v>
       </c>
       <c r="L16" s="3" t="n">
         <v>0.015</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0.024</v>
+        <v>0.018</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0.041</v>
+        <v>0.034</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>0.044</v>
+        <v>0.037</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>0.066</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="Q16" s="3" t="n">
-        <v>0.105</v>
+        <v>0.107</v>
       </c>
       <c r="R16" s="3" t="n">
-        <v>0.12</v>
+        <v>0.117</v>
       </c>
       <c r="S16" s="3" t="n">
-        <v>0.115</v>
+        <v>0.106</v>
       </c>
       <c r="T16" s="3" t="n">
-        <v>0.105</v>
+        <v>0.109</v>
       </c>
       <c r="U16" s="3" t="n">
-        <v>0.09</v>
+        <v>0.111</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Пиковая Дама</t>
+          <t>Lock</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>16</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>0.833</v>
+        <v>0.255386</v>
       </c>
       <c r="F17" s="4" t="n">
         <v>0.001</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>0.001</v>
+        <v>0.004</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>0.007</v>
+        <v>0.008</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>0.011</v>
+        <v>0.006</v>
       </c>
       <c r="L17" s="4" t="n">
-        <v>0.014</v>
+        <v>0.01</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>0.018</v>
+        <v>0.032</v>
       </c>
       <c r="N17" s="4" t="n">
         <v>0.035</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>0.046</v>
+        <v>0.059</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.077</v>
       </c>
       <c r="Q17" s="4" t="n">
+        <v>0.102</v>
+      </c>
+      <c r="R17" s="4" t="n">
+        <v>0.114</v>
+      </c>
+      <c r="S17" s="4" t="n">
+        <v>0.109</v>
+      </c>
+      <c r="T17" s="4" t="n">
+        <v>0.114</v>
+      </c>
+      <c r="U17" s="4" t="n">
         <v>0.099</v>
-      </c>
-      <c r="R17" s="4" t="n">
-        <v>0.097</v>
-      </c>
-      <c r="S17" s="4" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="T17" s="4" t="n">
-        <v>0.127</v>
-      </c>
-      <c r="U17" s="4" t="n">
-        <v>0.09</v>
       </c>
     </row>
     <row r="18">
@@ -1637,55 +1640,55 @@
         <v>17</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>0.8039999999999999</v>
+        <v>0.246744</v>
       </c>
       <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
-      <c r="G18" s="3" t="n">
+      <c r="F18" s="3" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="3" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="I18" s="3" t="n">
         <v>0.001</v>
       </c>
-      <c r="H18" s="3" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="I18" s="3" t="n">
-        <v>0.004</v>
-      </c>
       <c r="J18" s="3" t="n">
-        <v>0.004</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>0.008</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>0.019</v>
+        <v>0.015</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>0.014</v>
+        <v>0.022</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>0.019</v>
+        <v>0.026</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>0.04</v>
+        <v>0.051</v>
       </c>
       <c r="P18" s="3" t="n">
-        <v>0.076</v>
+        <v>0.056</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>0.098</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="R18" s="3" t="n">
-        <v>0.091</v>
+        <v>0.102</v>
       </c>
       <c r="S18" s="3" t="n">
-        <v>0.105</v>
+        <v>0.125</v>
       </c>
       <c r="T18" s="3" t="n">
-        <v>0.105</v>
+        <v>0.107</v>
       </c>
       <c r="U18" s="3" t="n">
-        <v>0.133</v>
+        <v>0.112</v>
       </c>
     </row>
     <row r="19">
@@ -1698,7 +1701,7 @@
         <v>18</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.799</v>
+        <v>0.22648</v>
       </c>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="6" t="n">
@@ -1707,46 +1710,46 @@
       <c r="F19" s="5" t="n"/>
       <c r="G19" s="5" t="n"/>
       <c r="H19" s="6" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="I19" s="6" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="J19" s="6" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="K19" s="6" t="n">
         <v>0.002</v>
-      </c>
-      <c r="I19" s="6" t="n">
-        <v>0.003</v>
-      </c>
-      <c r="J19" s="6" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="K19" s="6" t="n">
-        <v>0.001</v>
       </c>
       <c r="L19" s="6" t="n">
         <v>0.008</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>0.011</v>
+        <v>0.014</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>0.029</v>
+        <v>0.021</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>0.039</v>
+        <v>0.031</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>0.057</v>
+        <v>0.062</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>0.077</v>
+        <v>0.074</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>0.102</v>
+        <v>0.103</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>0.127</v>
+        <v>0.118</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>0.115</v>
+        <v>0.093</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>0.101</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="20">
@@ -1759,53 +1762,57 @@
         <v>19</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>0.753</v>
-      </c>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
+        <v>0.21903</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>0.001</v>
+      </c>
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="3" t="n">
         <v>0.001</v>
       </c>
       <c r="H20" s="2" t="n"/>
       <c r="I20" s="3" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>0.003</v>
+        <v>0.005</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>0.007</v>
+        <v>0.01</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>0.019</v>
+        <v>0.011</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>0.021</v>
+        <v>0.02</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>0.023</v>
+        <v>0.033</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>0.042</v>
+        <v>0.047</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>0.057</v>
+        <v>0.06</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>0.089</v>
+        <v>0.093</v>
       </c>
       <c r="S20" s="3" t="n">
-        <v>0.099</v>
+        <v>0.09</v>
       </c>
       <c r="T20" s="3" t="n">
-        <v>0.131</v>
+        <v>0.118</v>
       </c>
       <c r="U20" s="3" t="n">
-        <v>0.127</v>
+        <v>0.103</v>
       </c>
     </row>
     <row r="21">
@@ -1818,49 +1825,40 @@
         <v>20</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>0.674</v>
-      </c>
-      <c r="H21" s="4" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="I21" s="4" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="J21" s="4" t="n">
-        <v>0.002</v>
+        <v>0.1937</v>
       </c>
       <c r="K21" s="4" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="L21" s="4" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>0.006</v>
+        <v>0.011</v>
       </c>
       <c r="N21" s="4" t="n">
-        <v>0.015</v>
+        <v>0.019</v>
       </c>
       <c r="O21" s="4" t="n">
-        <v>0.018</v>
+        <v>0.026</v>
       </c>
       <c r="P21" s="4" t="n">
-        <v>0.036</v>
+        <v>0.032</v>
       </c>
       <c r="Q21" s="4" t="n">
-        <v>0.05</v>
+        <v>0.057</v>
       </c>
       <c r="R21" s="4" t="n">
-        <v>0.079</v>
+        <v>0.057</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.082</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="T21" s="4" t="n">
-        <v>0.115</v>
+        <v>0.111</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.131</v>
+        <v>0.121</v>
       </c>
     </row>
     <row r="22">
@@ -1873,7 +1871,7 @@
         <v>21</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>0.398</v>
+        <v>0.118902</v>
       </c>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
@@ -1881,39 +1879,37 @@
       <c r="G22" s="2" t="n"/>
       <c r="H22" s="2" t="n"/>
       <c r="I22" s="2" t="n"/>
-      <c r="J22" s="3" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="K22" s="2" t="n"/>
-      <c r="L22" s="3" t="n">
-        <v>0.001</v>
-      </c>
+      <c r="J22" s="2" t="n"/>
+      <c r="K22" s="3" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="L22" s="2" t="n"/>
       <c r="M22" s="3" t="n">
         <v>0.003</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>0.006</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="P22" s="3" t="n">
         <v>0.008999999999999999</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>0.022</v>
+        <v>0.018</v>
       </c>
       <c r="R22" s="3" t="n">
-        <v>0.034</v>
+        <v>0.033</v>
       </c>
       <c r="S22" s="3" t="n">
-        <v>0.044</v>
+        <v>0.051</v>
       </c>
       <c r="T22" s="3" t="n">
-        <v>0.058</v>
+        <v>0.052</v>
       </c>
       <c r="U22" s="3" t="n">
-        <v>0.1</v>
+        <v>0.08799999999999999</v>
       </c>
     </row>
     <row r="23">
@@ -1926,35 +1922,35 @@
         <v>22</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="Q23" s="4" t="n">
-        <v>0.002</v>
+        <v>0.09917080405271408</v>
+      </c>
+      <c r="P23" s="4" t="n">
+        <v>0.005942641661835695</v>
       </c>
       <c r="R23" s="4" t="n">
-        <v>0.001</v>
+        <v>0.005942641661835695</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.005</v>
+        <v>0.02377056664734278</v>
       </c>
       <c r="T23" s="4" t="n">
-        <v>0.002</v>
+        <v>0.02971320830917848</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.014</v>
+        <v>0.08913962492753542</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>sfv</t>
+          <t>emilian_s</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
         <v>23</v>
       </c>
       <c r="C24" s="3" t="n">
-        <v>0.025</v>
+        <v>0.09652633751593225</v>
       </c>
       <c r="D24" s="2" t="n"/>
       <c r="E24" s="2" t="n"/>
@@ -1968,37 +1964,46 @@
       <c r="M24" s="2" t="n"/>
       <c r="N24" s="2" t="n"/>
       <c r="O24" s="2" t="n"/>
-      <c r="P24" s="2" t="n"/>
+      <c r="P24" s="3" t="n">
+        <v>0.01245822631852507</v>
+      </c>
       <c r="Q24" s="2" t="n"/>
       <c r="R24" s="3" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="S24" s="2" t="n"/>
-      <c r="T24" s="2" t="n"/>
+        <v>0.01245822631852507</v>
+      </c>
+      <c r="S24" s="3" t="n">
+        <v>0.01245822631852507</v>
+      </c>
+      <c r="T24" s="3" t="n">
+        <v>0.0373746789555752</v>
+      </c>
       <c r="U24" s="3" t="n">
-        <v>0.007</v>
+        <v>0.07474935791115041</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>emilian_s</t>
+          <t>sfv</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>24</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>0.023</v>
+        <v>0.09390580362346135</v>
       </c>
       <c r="R25" s="4" t="n">
-        <v>0.002</v>
+        <v>0.01432364301761155</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>0.001</v>
+        <v>0.01432364301761155</v>
+      </c>
+      <c r="T25" s="4" t="n">
+        <v>0.01432364301761155</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.004</v>
+        <v>0.07161821508805777</v>
       </c>
     </row>
     <row r="26">
@@ -2011,7 +2016,7 @@
         <v>25</v>
       </c>
       <c r="C26" s="3" t="n">
-        <v>0.007</v>
+        <v>0.09130942297598842</v>
       </c>
       <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="n"/>
@@ -2029,36 +2034,39 @@
       <c r="Q26" s="2" t="n"/>
       <c r="R26" s="2" t="n"/>
       <c r="S26" s="2" t="n"/>
-      <c r="T26" s="3" t="n">
-        <v>0.001</v>
-      </c>
+      <c r="T26" s="2" t="n"/>
       <c r="U26" s="3" t="n">
-        <v>0.003</v>
+        <v>0.1021358198836559</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TryFraiz</t>
+          <t>1С</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>26</v>
       </c>
       <c r="C27" s="4" t="n">
-        <v>0.001</v>
+        <v>0.08873742238943043</v>
+      </c>
+      <c r="U27" s="4" t="n">
+        <v>0.1488882925997155</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>1С</t>
+          <t>TryFraiz</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="C28" s="2" t="n"/>
+      <c r="C28" s="3" t="n">
+        <v>0.08619003519239145</v>
+      </c>
       <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="n"/>
       <c r="F28" s="2" t="n"/>
@@ -2076,7 +2084,9 @@
       <c r="R28" s="2" t="n"/>
       <c r="S28" s="2" t="n"/>
       <c r="T28" s="2" t="n"/>
-      <c r="U28" s="2" t="n"/>
+      <c r="U28" s="3" t="n">
+        <v>0.1446141530073682</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2087,6 +2097,9 @@
       <c r="B29" t="n">
         <v>28</v>
       </c>
+      <c r="C29" s="4" t="n">
+        <v>0.08366750154394066</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2097,7 +2110,9 @@
       <c r="B30" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="C30" s="2" t="n"/>
+      <c r="C30" s="3" t="n">
+        <v>0.08117006877353256</v>
+      </c>
       <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="n"/>
@@ -2126,6 +2141,9 @@
       <c r="B31" t="n">
         <v>30</v>
       </c>
+      <c r="C31" s="4" t="n">
+        <v>0.07869799174509248</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2136,7 +2154,9 @@
       <c r="B32" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="C32" s="2" t="n"/>
+      <c r="C32" s="3" t="n">
+        <v>0.07625153324752322</v>
+      </c>
       <c r="D32" s="2" t="n"/>
       <c r="E32" s="2" t="n"/>
       <c r="F32" s="2" t="n"/>
@@ -2165,6 +2185,9 @@
       <c r="B33" t="n">
         <v>32</v>
       </c>
+      <c r="C33" s="4" t="n">
+        <v>0.0738309644141493</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2175,7 +2198,9 @@
       <c r="B34" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="C34" s="2" t="n"/>
+      <c r="C34" s="3" t="n">
+        <v>0.07143656517391686</v>
+      </c>
       <c r="D34" s="2" t="n"/>
       <c r="E34" s="2" t="n"/>
       <c r="F34" s="2" t="n"/>
@@ -2204,17 +2229,22 @@
       <c r="B35" t="n">
         <v>34</v>
       </c>
+      <c r="C35" s="4" t="n">
+        <v>0.06906862473750806</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Suruchik</t>
+          <t>Yars</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="C36" s="2" t="n"/>
+      <c r="C36" s="3" t="n">
+        <v>0.06672744212192308</v>
+      </c>
       <c r="D36" s="2" t="n"/>
       <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="n"/>
@@ -2237,23 +2267,28 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Настя дай стек</t>
+          <t>Suruchik</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>36</v>
       </c>
+      <c r="C37" s="4" t="n">
+        <v>0.06441332671753436</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Retbin</t>
+          <t>Настя дай стек</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="C38" s="2" t="n"/>
+      <c r="C38" s="3" t="n">
+        <v>0.06212659890213935</v>
+      </c>
       <c r="D38" s="2" t="n"/>
       <c r="E38" s="2" t="n"/>
       <c r="F38" s="2" t="n"/>
@@ -2282,17 +2317,22 @@
       <c r="B39" t="n">
         <v>38</v>
       </c>
+      <c r="C39" s="4" t="n">
+        <v>0.05986759070714237</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Yars</t>
+          <t>Retbin</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="C40" s="2" t="n"/>
+      <c r="C40" s="3" t="n">
+        <v>0.05763664654169758</v>
+      </c>
       <c r="D40" s="2" t="n"/>
       <c r="E40" s="2" t="n"/>
       <c r="F40" s="2" t="n"/>
@@ -2315,23 +2355,28 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>springbulk</t>
+          <t>БОЛЬШОЙ МИХА</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>40</v>
       </c>
+      <c r="C41" s="4" t="n">
+        <v>0.05543412398146273</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>БОЛЬШОЙ МИХА</t>
+          <t>springbulk</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="C42" s="2" t="n"/>
+      <c r="C42" s="3" t="n">
+        <v>0.05326039462957088</v>
+      </c>
       <c r="D42" s="2" t="n"/>
       <c r="E42" s="2" t="n"/>
       <c r="F42" s="2" t="n"/>
@@ -2360,6 +2405,9 @@
       <c r="B43" t="n">
         <v>42</v>
       </c>
+      <c r="C43" s="4" t="n">
+        <v>0.0511158450585511</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2370,7 +2418,9 @@
       <c r="B44" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="C44" s="2" t="n"/>
+      <c r="C44" s="3" t="n">
+        <v>0.04900087784325523</v>
+      </c>
       <c r="D44" s="2" t="n"/>
       <c r="E44" s="2" t="n"/>
       <c r="F44" s="2" t="n"/>
@@ -2399,6 +2449,9 @@
       <c r="B45" t="n">
         <v>44</v>
       </c>
+      <c r="C45" s="4" t="n">
+        <v>0.04691591269641866</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2409,7 +2462,9 @@
       <c r="B46" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="C46" s="2" t="n"/>
+      <c r="C46" s="3" t="n">
+        <v>0.04486138772035221</v>
+      </c>
       <c r="D46" s="2" t="n"/>
       <c r="E46" s="2" t="n"/>
       <c r="F46" s="2" t="n"/>
@@ -2438,6 +2493,9 @@
       <c r="B47" t="n">
         <v>46</v>
       </c>
+      <c r="C47" s="4" t="n">
+        <v>0.04283776079049762</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2448,7 +2506,9 @@
       <c r="B48" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="C48" s="2" t="n"/>
+      <c r="C48" s="3" t="n">
+        <v>0.04084551108926481</v>
+      </c>
       <c r="D48" s="2" t="n"/>
       <c r="E48" s="2" t="n"/>
       <c r="F48" s="2" t="n"/>
@@ -2477,6 +2537,9 @@
       <c r="B49" t="n">
         <v>48</v>
       </c>
+      <c r="C49" s="4" t="n">
+        <v>0.03888514081181586</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2487,7 +2550,9 @@
       <c r="B50" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="C50" s="2" t="n"/>
+      <c r="C50" s="3" t="n">
+        <v>0.03695717706940388</v>
+      </c>
       <c r="D50" s="2" t="n"/>
       <c r="E50" s="2" t="n"/>
       <c r="F50" s="2" t="n"/>
@@ -2516,6 +2581,9 @@
       <c r="B51" t="n">
         <v>50</v>
       </c>
+      <c r="C51" s="4" t="n">
+        <v>0.03506217402069824</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2526,7 +2594,9 @@
       <c r="B52" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="C52" s="2" t="n"/>
+      <c r="C52" s="3" t="n">
+        <v>0.03320071526746089</v>
+      </c>
       <c r="D52" s="2" t="n"/>
       <c r="E52" s="2" t="n"/>
       <c r="F52" s="2" t="n"/>
@@ -2549,23 +2619,28 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Serg</t>
+          <t>DARI</t>
         </is>
       </c>
       <c r="B53" t="n">
         <v>52</v>
       </c>
+      <c r="C53" s="4" t="n">
+        <v>0.03137341655829062</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>DARI</t>
+          <t>Serg</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="C54" s="2" t="n"/>
+      <c r="C54" s="3" t="n">
+        <v>0.02958092885332818</v>
+      </c>
       <c r="D54" s="2" t="n"/>
       <c r="E54" s="2" t="n"/>
       <c r="F54" s="2" t="n"/>
@@ -2594,6 +2669,9 @@
       <c r="B55" t="n">
         <v>54</v>
       </c>
+      <c r="C55" s="4" t="n">
+        <v>0.02782394181435892</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -2604,7 +2682,9 @@
       <c r="B56" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="C56" s="2" t="n"/>
+      <c r="C56" s="3" t="n">
+        <v>0.02610318779939383</v>
+      </c>
       <c r="D56" s="2" t="n"/>
       <c r="E56" s="2" t="n"/>
       <c r="F56" s="2" t="n"/>
@@ -2633,6 +2713,9 @@
       <c r="B57" t="n">
         <v>56</v>
       </c>
+      <c r="C57" s="4" t="n">
+        <v>0.02441944645956044</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -2643,7 +2726,9 @@
       <c r="B58" s="2" t="n">
         <v>57</v>
       </c>
-      <c r="C58" s="2" t="n"/>
+      <c r="C58" s="3" t="n">
+        <v>0.02277355006037658</v>
+      </c>
       <c r="D58" s="2" t="n"/>
       <c r="E58" s="2" t="n"/>
       <c r="F58" s="2" t="n"/>
@@ -2672,6 +2757,9 @@
       <c r="B59" t="n">
         <v>58</v>
       </c>
+      <c r="C59" s="4" t="n">
+        <v>0.02116638968116055</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -2682,7 +2770,9 @@
       <c r="B60" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="C60" s="2" t="n"/>
+      <c r="C60" s="3" t="n">
+        <v>0.01959892248821406</v>
+      </c>
       <c r="D60" s="2" t="n"/>
       <c r="E60" s="2" t="n"/>
       <c r="F60" s="2" t="n"/>
@@ -2711,6 +2801,9 @@
       <c r="B61" t="n">
         <v>60</v>
       </c>
+      <c r="C61" s="4" t="n">
+        <v>0.01807218033349118</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -2721,7 +2814,9 @@
       <c r="B62" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="C62" s="2" t="n"/>
+      <c r="C62" s="3" t="n">
+        <v>0.01658728000659684</v>
+      </c>
       <c r="D62" s="2" t="n"/>
       <c r="E62" s="2" t="n"/>
       <c r="F62" s="2" t="n"/>
@@ -2750,6 +2845,9 @@
       <c r="B63" t="n">
         <v>62</v>
       </c>
+      <c r="C63" s="4" t="n">
+        <v>0.01514543557290403</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -2760,7 +2858,9 @@
       <c r="B64" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="C64" s="2" t="n"/>
+      <c r="C64" s="3" t="n">
+        <v>0.01374797337771438</v>
+      </c>
       <c r="D64" s="2" t="n"/>
       <c r="E64" s="2" t="n"/>
       <c r="F64" s="2" t="n"/>
@@ -2789,6 +2889,9 @@
       <c r="B65" t="n">
         <v>64</v>
       </c>
+      <c r="C65" s="4" t="n">
+        <v>0.01239635050658926</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -2799,7 +2902,9 @@
       <c r="B66" s="2" t="n">
         <v>65</v>
       </c>
-      <c r="C66" s="2" t="n"/>
+      <c r="C66" s="3" t="n">
+        <v>0.0110921777986788</v>
+      </c>
       <c r="D66" s="2" t="n"/>
       <c r="E66" s="2" t="n"/>
       <c r="F66" s="2" t="n"/>
@@ -2828,17 +2933,22 @@
       <c r="B67" t="n">
         <v>66</v>
       </c>
+      <c r="C67" s="4" t="n">
+        <v>0.00983724896813656</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>rus210385</t>
+          <t>Fara</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
         <v>67</v>
       </c>
-      <c r="C68" s="2" t="n"/>
+      <c r="C68" s="3" t="n">
+        <v>0.008633578092188508</v>
+      </c>
       <c r="D68" s="2" t="n"/>
       <c r="E68" s="2" t="n"/>
       <c r="F68" s="2" t="n"/>
@@ -2861,23 +2971,28 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Fara</t>
+          <t>Shuricspinoza</t>
         </is>
       </c>
       <c r="B69" t="n">
         <v>68</v>
       </c>
+      <c r="C69" s="4" t="n">
+        <v>0.007483448838392796</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Schwepp1S</t>
+          <t>katerina_boc</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
         <v>69</v>
       </c>
-      <c r="C70" s="2" t="n"/>
+      <c r="C70" s="3" t="n">
+        <v>0.006389480632318888</v>
+      </c>
       <c r="D70" s="2" t="n"/>
       <c r="E70" s="2" t="n"/>
       <c r="F70" s="2" t="n"/>
@@ -2900,23 +3015,28 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Shuricspinoza</t>
+          <t>frida_hk</t>
         </is>
       </c>
       <c r="B71" t="n">
         <v>70</v>
       </c>
+      <c r="C71" s="4" t="n">
+        <v>0.005354720098812203</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>twewefe</t>
+          <t>Schwepp1S</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
         <v>71</v>
       </c>
-      <c r="C72" s="2" t="n"/>
+      <c r="C72" s="3" t="n">
+        <v>0.00438277175258728</v>
+      </c>
       <c r="D72" s="2" t="n"/>
       <c r="E72" s="2" t="n"/>
       <c r="F72" s="2" t="n"/>
@@ -2939,23 +3059,28 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>katerina_boc</t>
+          <t>rus210385</t>
         </is>
       </c>
       <c r="B73" t="n">
         <v>72</v>
       </c>
+      <c r="C73" s="4" t="n">
+        <v>0.003477992726794865</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>edimerfi</t>
+          <t>nsa</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
         <v>73</v>
       </c>
-      <c r="C74" s="2" t="n"/>
+      <c r="C74" s="3" t="n">
+        <v>0.002645798710145069</v>
+      </c>
       <c r="D74" s="2" t="n"/>
       <c r="E74" s="2" t="n"/>
       <c r="F74" s="2" t="n"/>
@@ -2978,23 +3103,28 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>frida_hk</t>
+          <t>alinaadmv</t>
         </is>
       </c>
       <c r="B75" t="n">
         <v>74</v>
       </c>
+      <c r="C75" s="4" t="n">
+        <v>0.001893179446613004</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>alinaadmv</t>
+          <t>twewefe</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="C76" s="2" t="n"/>
+      <c r="C76" s="3" t="n">
+        <v>0.00122965612101707</v>
+      </c>
       <c r="D76" s="2" t="n"/>
       <c r="E76" s="2" t="n"/>
       <c r="F76" s="2" t="n"/>
@@ -3017,17 +3147,20 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>DanilaOdinokov</t>
+          <t>edimerfi</t>
         </is>
       </c>
       <c r="B77" t="n">
         <v>76</v>
       </c>
+      <c r="C77" s="4" t="n">
+        <v>0.0006693400123515253</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>nsa</t>
+          <t>DanilaOdinokov</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">

</xml_diff>

<commit_message>
changed mingamesforful and minmultiplier params after brier search
</commit_message>
<xml_diff>
--- a/data/playoff_odds.xlsx
+++ b/data/playoff_odds.xlsx
@@ -591,597 +591,600 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Noize MC</t>
+          <t>Гризли</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>0.298</v>
+        <v>0.25</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.04708400000000001</v>
+        <v>0.039</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.03963400000000001</v>
+        <v>0.034</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.033376</v>
+        <v>0.02475</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>0.03129000000000001</v>
+        <v>0.0235</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>0.02801200000000001</v>
+        <v>0.0245</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.02473400000000001</v>
+        <v>0.0195</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.021754</v>
+        <v>0.0155</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>0.016986</v>
+        <v>0.01475</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>0.012218</v>
+        <v>0.01725</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>0.015496</v>
+        <v>0.01325</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>0.009834000000000002</v>
+        <v>0.00775</v>
       </c>
       <c r="O2" s="3" t="n">
-        <v>0.007450000000000002</v>
+        <v>0.0065</v>
       </c>
       <c r="P2" s="3" t="n">
-        <v>0.003874</v>
+        <v>0.0055</v>
       </c>
       <c r="Q2" s="3" t="n">
-        <v>0.004172</v>
+        <v>0.00175</v>
       </c>
       <c r="R2" s="3" t="n">
-        <v>0.00149</v>
+        <v>0.001</v>
       </c>
       <c r="S2" s="3" t="n">
-        <v>0.000298</v>
-      </c>
-      <c r="T2" s="3" t="n">
-        <v>0.000298</v>
-      </c>
+        <v>0.0015</v>
+      </c>
+      <c r="T2" s="2" t="n"/>
       <c r="U2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Гризли</t>
+          <t>Драйв</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>0.298</v>
+        <v>0.25</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>0.045594</v>
+        <v>0.03225</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0.038144</v>
+        <v>0.03275</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>0.03278</v>
+        <v>0.02375</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.029204</v>
+        <v>0.02775</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>0.026224</v>
+        <v>0.01925</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>0.021754</v>
+        <v>0.02325</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>0.019966</v>
+        <v>0.01725</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>0.021456</v>
+        <v>0.0155</v>
       </c>
       <c r="L3" s="4" t="n">
-        <v>0.018774</v>
+        <v>0.013</v>
       </c>
       <c r="M3" s="4" t="n">
-        <v>0.013112</v>
+        <v>0.01425</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>0.013708</v>
+        <v>0.011</v>
       </c>
       <c r="O3" s="4" t="n">
-        <v>0.007450000000000002</v>
+        <v>0.01</v>
       </c>
       <c r="P3" s="4" t="n">
-        <v>0.004470000000000001</v>
+        <v>0.005</v>
       </c>
       <c r="Q3" s="4" t="n">
-        <v>0.002086</v>
+        <v>0.0025</v>
       </c>
       <c r="R3" s="4" t="n">
-        <v>0.002384</v>
+        <v>0.00175</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.000298</v>
+        <v>0.00025</v>
       </c>
       <c r="T3" s="4" t="n">
-        <v>0.0005960000000000001</v>
+        <v>0.00025</v>
+      </c>
+      <c r="U3" s="4" t="n">
+        <v>0.00025</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Драйв</t>
+          <t>Yanchik_250</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.298</v>
+        <v>0.25</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.04678600000000001</v>
+        <v>0.00775</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.03456800000000001</v>
+        <v>0.0125</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.029502</v>
+        <v>0.0185</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0.02503200000000001</v>
+        <v>0.0165</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.021158</v>
+        <v>0.02325</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.027118</v>
+        <v>0.01775</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.027118</v>
+        <v>0.02275</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>0.021456</v>
+        <v>0.021</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>0.018774</v>
+        <v>0.02</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>0.015496</v>
+        <v>0.0215</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>0.011622</v>
+        <v>0.019</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>0.007152000000000001</v>
+        <v>0.01975</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>0.004172</v>
+        <v>0.008750000000000001</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>0.002682</v>
+        <v>0.00975</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>0.003576000000000001</v>
+        <v>0.007</v>
       </c>
       <c r="S4" s="3" t="n">
-        <v>0.0005960000000000001</v>
-      </c>
-      <c r="T4" s="2" t="n"/>
+        <v>0.00125</v>
+      </c>
+      <c r="T4" s="3" t="n">
+        <v>0.00225</v>
+      </c>
       <c r="U4" s="3" t="n">
-        <v>0.001192</v>
+        <v>0.00075</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>long_2203</t>
+          <t>Пассажир</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>0.298</v>
+        <v>0.24975</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>0.03009800000000001</v>
+        <v>0.0195</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0.03009800000000001</v>
+        <v>0.0195</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>0.03278</v>
+        <v>0.0245</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.027416</v>
+        <v>0.01875</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0.026522</v>
+        <v>0.022</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>0.022648</v>
+        <v>0.0195</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>0.02235</v>
+        <v>0.019</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>0.016688</v>
+        <v>0.02425</v>
       </c>
       <c r="L5" s="4" t="n">
-        <v>0.022946</v>
+        <v>0.0215</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>0.017582</v>
+        <v>0.01725</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v>0.01639</v>
+        <v>0.0145</v>
       </c>
       <c r="O5" s="4" t="n">
-        <v>0.012516</v>
+        <v>0.0105</v>
       </c>
       <c r="P5" s="4" t="n">
-        <v>0.010132</v>
+        <v>0.00975</v>
       </c>
       <c r="Q5" s="4" t="n">
-        <v>0.003278</v>
+        <v>0.0045</v>
       </c>
       <c r="R5" s="4" t="n">
-        <v>0.003278</v>
+        <v>0.0035</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>0.002086</v>
+        <v>0.00075</v>
       </c>
       <c r="T5" s="4" t="n">
-        <v>0.0005960000000000001</v>
+        <v>0.00025</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>0.000298</v>
+        <v>0.00025</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Пассажир</t>
+          <t>G_rant_999</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0.298</v>
+        <v>0.24975</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0.02235</v>
+        <v>0.0165</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.023542</v>
+        <v>0.016</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0.029502</v>
+        <v>0.01625</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0.02384</v>
+        <v>0.01925</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.029204</v>
+        <v>0.02025</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.02831000000000001</v>
+        <v>0.01825</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.021158</v>
+        <v>0.02075</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>0.018774</v>
+        <v>0.02025</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>0.019966</v>
+        <v>0.01825</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>0.021158</v>
+        <v>0.018</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>0.020562</v>
+        <v>0.01725</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>0.016986</v>
+        <v>0.01775</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>0.009238000000000001</v>
+        <v>0.01325</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>0.006556</v>
+        <v>0.01075</v>
       </c>
       <c r="R6" s="3" t="n">
-        <v>0.003576000000000001</v>
+        <v>0.0025</v>
       </c>
       <c r="S6" s="3" t="n">
-        <v>0.00149</v>
+        <v>0.002</v>
       </c>
       <c r="T6" s="3" t="n">
-        <v>0.0005960000000000001</v>
+        <v>0.0015</v>
       </c>
       <c r="U6" s="3" t="n">
-        <v>0.001192</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>terzzzzzzzzz</t>
+          <t>Laches1</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>6</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>0.298</v>
+        <v>0.24975</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>0.01341</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0.015794</v>
+        <v>0.0095</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>0.019966</v>
+        <v>0.01425</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.02086</v>
+        <v>0.019</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0.02682</v>
+        <v>0.02075</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>0.022648</v>
+        <v>0.025</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>0.022946</v>
+        <v>0.0175</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>0.022648</v>
+        <v>0.021</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>0.026522</v>
+        <v>0.022</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>0.023244</v>
+        <v>0.02425</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>0.01788</v>
+        <v>0.0245</v>
       </c>
       <c r="O7" s="4" t="n">
-        <v>0.022052</v>
+        <v>0.0145</v>
       </c>
       <c r="P7" s="4" t="n">
-        <v>0.016986</v>
+        <v>0.01</v>
       </c>
       <c r="Q7" s="4" t="n">
-        <v>0.011622</v>
+        <v>0.006</v>
       </c>
       <c r="R7" s="4" t="n">
-        <v>0.005066000000000001</v>
+        <v>0.0045</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.004172</v>
+        <v>0.004</v>
       </c>
       <c r="T7" s="4" t="n">
-        <v>0.00298</v>
+        <v>0.0025</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.002086</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>G_rant_999</t>
+          <t>Noize MC</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
         <v>7</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>0.2977020000000001</v>
+        <v>0.24975</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0.018774</v>
+        <v>0.04575</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.020264</v>
+        <v>0.0275</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0.020264</v>
+        <v>0.0305</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>0.027118</v>
+        <v>0.02425</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.02235</v>
+        <v>0.01975</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>0.023542</v>
+        <v>0.01875</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.021456</v>
+        <v>0.0195</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>0.022946</v>
+        <v>0.01475</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>0.02682</v>
+        <v>0.0135</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>0.022946</v>
+        <v>0.012</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>0.022052</v>
+        <v>0.008750000000000001</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>0.014006</v>
+        <v>0.00525</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>0.0149</v>
+        <v>0.0045</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>0.008046000000000001</v>
+        <v>0.0025</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>0.004172</v>
+        <v>0.0015</v>
       </c>
       <c r="S8" s="3" t="n">
-        <v>0.003278</v>
+        <v>0.00025</v>
       </c>
       <c r="T8" s="3" t="n">
-        <v>0.002682</v>
+        <v>0.0005</v>
       </c>
       <c r="U8" s="3" t="n">
-        <v>0.002086</v>
+        <v>0.00025</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Сокол</t>
+          <t>long_2203</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>8</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>0.2977020000000001</v>
+        <v>0.24975</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>0.013708</v>
+        <v>0.01825</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.019966</v>
+        <v>0.0275</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>0.01937</v>
+        <v>0.02325</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.021754</v>
+        <v>0.01875</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>0.022946</v>
+        <v>0.0195</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>0.021158</v>
+        <v>0.018</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>0.023244</v>
+        <v>0.0225</v>
       </c>
       <c r="K9" s="4" t="n">
-        <v>0.021158</v>
+        <v>0.024</v>
       </c>
       <c r="L9" s="4" t="n">
-        <v>0.02473400000000001</v>
+        <v>0.019</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>0.027118</v>
+        <v>0.01875</v>
       </c>
       <c r="N9" s="4" t="n">
-        <v>0.021158</v>
+        <v>0.012</v>
       </c>
       <c r="O9" s="4" t="n">
-        <v>0.025628</v>
+        <v>0.00975</v>
       </c>
       <c r="P9" s="4" t="n">
-        <v>0.014602</v>
+        <v>0.008</v>
       </c>
       <c r="Q9" s="4" t="n">
-        <v>0.007152000000000001</v>
+        <v>0.005</v>
       </c>
       <c r="R9" s="4" t="n">
-        <v>0.006854000000000001</v>
+        <v>0.00175</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.004470000000000001</v>
+        <v>0.00075</v>
       </c>
       <c r="T9" s="4" t="n">
-        <v>0.001788</v>
+        <v>0.00125</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>0.0005960000000000001</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Yanchik_250</t>
+          <t>terzzzzzzzzz</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
         <v>9</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.297702</v>
+        <v>0.24975</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.011324</v>
+        <v>0.01375</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.016688</v>
+        <v>0.01425</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.019072</v>
+        <v>0.01525</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>0.021754</v>
+        <v>0.01825</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.024138</v>
+        <v>0.01675</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>0.022052</v>
+        <v>0.019</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.02473400000000001</v>
+        <v>0.01975</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>0.023244</v>
+        <v>0.01875</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0.027714</v>
+        <v>0.02075</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>0.02384</v>
+        <v>0.02125</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.027118</v>
+        <v>0.02075</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>0.019668</v>
+        <v>0.017</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>0.014304</v>
+        <v>0.0145</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>0.011622</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="R10" s="3" t="n">
-        <v>0.004172</v>
+        <v>0.0055</v>
       </c>
       <c r="S10" s="3" t="n">
-        <v>0.003576000000000001</v>
+        <v>0.0025</v>
       </c>
       <c r="T10" s="3" t="n">
-        <v>0.00149</v>
+        <v>0.00125</v>
       </c>
       <c r="U10" s="3" t="n">
-        <v>0.0008940000000000002</v>
+        <v>0.00075</v>
       </c>
     </row>
     <row r="11">
@@ -1194,61 +1197,61 @@
         <v>10</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>0.2974040000000001</v>
+        <v>0.2495</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>0.02235</v>
+        <v>0.02</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0.02384</v>
+        <v>0.025</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>0.025926</v>
+        <v>0.02025</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>0.02384</v>
+        <v>0.023</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>0.022052</v>
+        <v>0.02225</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>0.028608</v>
+        <v>0.0235</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>0.024436</v>
+        <v>0.0195</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>0.031886</v>
+        <v>0.0195</v>
       </c>
       <c r="L11" s="4" t="n">
-        <v>0.021158</v>
+        <v>0.018</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>0.01937</v>
+        <v>0.013</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>0.016092</v>
+        <v>0.0155</v>
       </c>
       <c r="O11" s="4" t="n">
-        <v>0.014304</v>
+        <v>0.01175</v>
       </c>
       <c r="P11" s="4" t="n">
-        <v>0.010132</v>
+        <v>0.00775</v>
       </c>
       <c r="Q11" s="4" t="n">
-        <v>0.005662</v>
+        <v>0.004</v>
       </c>
       <c r="R11" s="4" t="n">
-        <v>0.004172</v>
+        <v>0.00225</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.002682</v>
+        <v>0.002</v>
       </c>
       <c r="T11" s="4" t="n">
-        <v>0.000298</v>
+        <v>0.00175</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.000298</v>
+        <v>0.00025</v>
       </c>
     </row>
     <row r="12">
@@ -1261,128 +1264,128 @@
         <v>11</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>0.2974040000000001</v>
+        <v>0.24925</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0.013708</v>
+        <v>0.01375</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.019966</v>
+        <v>0.01675</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.01788</v>
+        <v>0.019</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0.02473400000000001</v>
+        <v>0.02</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.02086</v>
+        <v>0.02025</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>0.021456</v>
+        <v>0.021</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.028608</v>
+        <v>0.022</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0.031588</v>
+        <v>0.0165</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>0.02235</v>
+        <v>0.01925</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0.023542</v>
+        <v>0.017</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.021158</v>
+        <v>0.01925</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.019966</v>
+        <v>0.01625</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>0.01341</v>
+        <v>0.01225</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>0.005662</v>
+        <v>0.00625</v>
       </c>
       <c r="R12" s="3" t="n">
-        <v>0.005662</v>
+        <v>0.00475</v>
       </c>
       <c r="S12" s="3" t="n">
-        <v>0.003576000000000001</v>
+        <v>0.0025</v>
       </c>
       <c r="T12" s="3" t="n">
-        <v>0.002086</v>
+        <v>0.00125</v>
       </c>
       <c r="U12" s="3" t="n">
-        <v>0.0008940000000000002</v>
+        <v>0.00075</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Laches1</t>
+          <t>Сокол</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>12</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>0.2968080000000001</v>
+        <v>0.24925</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>0.012516</v>
+        <v>0.01425</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.014006</v>
+        <v>0.0135</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0.015198</v>
+        <v>0.01825</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.018178</v>
+        <v>0.0175</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>0.020264</v>
+        <v>0.01825</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>0.025926</v>
+        <v>0.01925</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>0.024138</v>
+        <v>0.02425</v>
       </c>
       <c r="K13" s="4" t="n">
-        <v>0.02831000000000001</v>
+        <v>0.022</v>
       </c>
       <c r="L13" s="4" t="n">
-        <v>0.02473400000000001</v>
+        <v>0.02175</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>0.026522</v>
+        <v>0.02025</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>0.02533000000000001</v>
+        <v>0.01625</v>
       </c>
       <c r="O13" s="4" t="n">
-        <v>0.021456</v>
+        <v>0.013</v>
       </c>
       <c r="P13" s="4" t="n">
-        <v>0.013112</v>
+        <v>0.01225</v>
       </c>
       <c r="Q13" s="4" t="n">
-        <v>0.009536000000000001</v>
+        <v>0.00675</v>
       </c>
       <c r="R13" s="4" t="n">
-        <v>0.006854000000000001</v>
+        <v>0.004</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>0.004470000000000001</v>
+        <v>0.0035</v>
       </c>
       <c r="T13" s="4" t="n">
-        <v>0.003576000000000001</v>
+        <v>0.001</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.0008940000000000002</v>
+        <v>0.00225</v>
       </c>
     </row>
     <row r="14">
@@ -1395,243 +1398,242 @@
         <v>13</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>0.2708820000000001</v>
-      </c>
-      <c r="D14" s="2" t="n"/>
+        <v>0.23125</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>0.00025</v>
+      </c>
       <c r="E14" s="3" t="n">
-        <v>0.000298</v>
+        <v>0.00075</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.001192</v>
+        <v>0.0005</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>0.00149</v>
+        <v>0.00125</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0.00149</v>
+        <v>0.00125</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>0.002384</v>
+        <v>0.00325</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0.005066000000000001</v>
+        <v>0.00375</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>0.004470000000000001</v>
+        <v>0.0025</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>0.006556</v>
+        <v>0.00575</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0.010728</v>
+        <v>0.008750000000000001</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>0.017284</v>
+        <v>0.014</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>0.018476</v>
+        <v>0.021</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>0.033376</v>
+        <v>0.03075</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>0.031886</v>
+        <v>0.02925</v>
       </c>
       <c r="R14" s="3" t="n">
-        <v>0.03576000000000001</v>
+        <v>0.02625</v>
       </c>
       <c r="S14" s="3" t="n">
-        <v>0.03605800000000001</v>
+        <v>0.023</v>
       </c>
       <c r="T14" s="3" t="n">
-        <v>0.027118</v>
+        <v>0.023</v>
       </c>
       <c r="U14" s="3" t="n">
-        <v>0.01937</v>
+        <v>0.021</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Пиковая Дама</t>
+          <t>лучший игрок</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>14</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>0.256876</v>
-      </c>
-      <c r="E15" s="4" t="n">
-        <v>0.000298</v>
+        <v>0.22275</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0.000298</v>
+        <v>0.00025</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.000298</v>
+        <v>0.0005</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>0.00149</v>
+        <v>0.001</v>
       </c>
       <c r="I15" s="4" t="n">
-        <v>0.0005960000000000001</v>
+        <v>0.001</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>0.002086</v>
+        <v>0.00125</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>0.003278</v>
+        <v>0.00325</v>
       </c>
       <c r="L15" s="4" t="n">
-        <v>0.002086</v>
+        <v>0.0065</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>0.007152000000000001</v>
+        <v>0.00725</v>
       </c>
       <c r="N15" s="4" t="n">
-        <v>0.010728</v>
+        <v>0.01175</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>0.014304</v>
+        <v>0.014</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>0.02235</v>
+        <v>0.01975</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>0.02801200000000001</v>
+        <v>0.0295</v>
       </c>
       <c r="R15" s="4" t="n">
-        <v>0.029502</v>
+        <v>0.031</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03963400000000001</v>
+        <v>0.0275</v>
       </c>
       <c r="T15" s="4" t="n">
-        <v>0.029502</v>
+        <v>0.0255</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.035462</v>
+        <v>0.02075</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>лучший игрок</t>
+          <t>Lock</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
         <v>15</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>0.25628</v>
+        <v>0.21575</v>
       </c>
       <c r="D16" s="2" t="n"/>
-      <c r="E16" s="3" t="n">
-        <v>0.000298</v>
-      </c>
+      <c r="E16" s="2" t="n"/>
       <c r="F16" s="3" t="n">
-        <v>0.0005960000000000001</v>
+        <v>0.00025</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>0.0005960000000000001</v>
-      </c>
-      <c r="H16" s="3" t="n">
-        <v>0.00149</v>
-      </c>
-      <c r="I16" s="3" t="n">
-        <v>0.002086</v>
-      </c>
+        <v>0.00075</v>
+      </c>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
       <c r="J16" s="3" t="n">
-        <v>0.002682</v>
+        <v>0.00175</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>0.004470000000000001</v>
+        <v>0.0015</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>0.004172</v>
+        <v>0.00325</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0.009536000000000001</v>
+        <v>0.00375</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0.01341</v>
+        <v>0.011</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>0.021456</v>
+        <v>0.0115</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>0.022946</v>
+        <v>0.0215</v>
       </c>
       <c r="Q16" s="3" t="n">
-        <v>0.033674</v>
+        <v>0.02075</v>
       </c>
       <c r="R16" s="3" t="n">
-        <v>0.032184</v>
+        <v>0.0275</v>
       </c>
       <c r="S16" s="3" t="n">
-        <v>0.028608</v>
+        <v>0.029</v>
       </c>
       <c r="T16" s="3" t="n">
-        <v>0.028906</v>
+        <v>0.031</v>
       </c>
       <c r="U16" s="3" t="n">
-        <v>0.027714</v>
+        <v>0.026</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Lock</t>
+          <t>Пиковая Дама</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>16</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>0.25628</v>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>0.000298</v>
+        <v>0.21375</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>0.0005</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>0.00149</v>
+        <v>0.00125</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>0.001192</v>
+        <v>0.0005</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>0.002681999999999999</v>
+        <v>0.00475</v>
       </c>
       <c r="L17" s="4" t="n">
-        <v>0.00596</v>
+        <v>0.00375</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>0.006854</v>
+        <v>0.0065</v>
       </c>
       <c r="N17" s="4" t="n">
-        <v>0.007152</v>
+        <v>0.00475</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>0.014304</v>
+        <v>0.0135</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>0.022946</v>
+        <v>0.02</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>0.031886</v>
+        <v>0.0245</v>
       </c>
       <c r="R17" s="4" t="n">
-        <v>0.033674</v>
+        <v>0.02575</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.03129</v>
+        <v>0.033</v>
       </c>
       <c r="T17" s="4" t="n">
-        <v>0.03576</v>
+        <v>0.0325</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.03129</v>
+        <v>0.02175</v>
       </c>
     </row>
     <row r="18">
@@ -1644,53 +1646,55 @@
         <v>17</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>0.239294</v>
+        <v>0.19975</v>
       </c>
       <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="3" t="n">
-        <v>0.000298</v>
+        <v>0.00025</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>0.0005960000000000001</v>
-      </c>
-      <c r="I18" s="2" t="n"/>
+        <v>0.0005</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>0.00025</v>
+      </c>
       <c r="J18" s="3" t="n">
-        <v>0.00149</v>
+        <v>0.00125</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>0.0008940000000000002</v>
+        <v>0.00125</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>0.005364000000000001</v>
+        <v>0.00225</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>0.005364000000000001</v>
+        <v>0.0055</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>0.008046000000000001</v>
+        <v>0.00775</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>0.013112</v>
+        <v>0.013</v>
       </c>
       <c r="P18" s="3" t="n">
-        <v>0.018774</v>
+        <v>0.014</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>0.024138</v>
+        <v>0.02275</v>
       </c>
       <c r="R18" s="3" t="n">
-        <v>0.030396</v>
+        <v>0.02425</v>
       </c>
       <c r="S18" s="3" t="n">
-        <v>0.029204</v>
+        <v>0.027</v>
       </c>
       <c r="T18" s="3" t="n">
-        <v>0.03427000000000001</v>
+        <v>0.0235</v>
       </c>
       <c r="U18" s="3" t="n">
-        <v>0.03456800000000001</v>
+        <v>0.03325</v>
       </c>
     </row>
     <row r="19">
@@ -1703,55 +1707,55 @@
         <v>18</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.234228</v>
-      </c>
-      <c r="D19" s="6" t="n">
-        <v>0.000298</v>
-      </c>
+        <v>0.1945</v>
+      </c>
+      <c r="D19" s="5" t="n"/>
       <c r="E19" s="6" t="n">
-        <v>0.000298</v>
-      </c>
-      <c r="F19" s="5" t="n"/>
+        <v>0.0005</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>0.00025</v>
+      </c>
       <c r="G19" s="5" t="n"/>
-      <c r="H19" s="6" t="n">
-        <v>0.001192</v>
-      </c>
-      <c r="I19" s="5" t="n"/>
+      <c r="H19" s="5" t="n"/>
+      <c r="I19" s="6" t="n">
+        <v>0.001</v>
+      </c>
       <c r="J19" s="6" t="n">
-        <v>0.001788</v>
+        <v>0.00075</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>0.002086</v>
+        <v>0.0015</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>0.003576000000000001</v>
+        <v>0.00125</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>0.003576000000000001</v>
+        <v>0.00275</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>0.008940000000000002</v>
+        <v>0.0055</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>0.010728</v>
+        <v>0.00775</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>0.016688</v>
+        <v>0.012</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>0.022946</v>
+        <v>0.01875</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>0.028906</v>
+        <v>0.02325</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>0.031588</v>
+        <v>0.029</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>0.033674</v>
+        <v>0.0315</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>0.035164</v>
+        <v>0.0285</v>
       </c>
     </row>
     <row r="20">
@@ -1764,55 +1768,51 @@
         <v>19</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>0.229758</v>
+        <v>0.18775</v>
       </c>
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="n"/>
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="3" t="n">
-        <v>0.000298</v>
-      </c>
-      <c r="H20" s="3" t="n">
-        <v>0.0008940000000000002</v>
-      </c>
+        <v>0.00025</v>
+      </c>
+      <c r="H20" s="2" t="n"/>
       <c r="I20" s="3" t="n">
-        <v>0.000298</v>
-      </c>
-      <c r="J20" s="3" t="n">
-        <v>0.00149</v>
-      </c>
+        <v>0.00025</v>
+      </c>
+      <c r="J20" s="2" t="n"/>
       <c r="K20" s="3" t="n">
-        <v>0.00149</v>
+        <v>0.00175</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>0.002086</v>
+        <v>0.00175</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>0.003576000000000001</v>
+        <v>0.00275</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>0.006258000000000001</v>
+        <v>0.00475</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>0.009536000000000001</v>
+        <v>0.00925</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>0.017284</v>
+        <v>0.01025</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>0.021754</v>
+        <v>0.01625</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>0.028608</v>
+        <v>0.02175</v>
       </c>
       <c r="S20" s="3" t="n">
-        <v>0.02831000000000001</v>
+        <v>0.02875</v>
       </c>
       <c r="T20" s="3" t="n">
-        <v>0.037548</v>
+        <v>0.02375</v>
       </c>
       <c r="U20" s="3" t="n">
-        <v>0.03695200000000001</v>
+        <v>0.034</v>
       </c>
     </row>
     <row r="21">
@@ -1825,49 +1825,46 @@
         <v>20</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>0.19817</v>
-      </c>
-      <c r="F21" s="4" t="n">
-        <v>0.000298</v>
-      </c>
-      <c r="H21" s="4" t="n">
-        <v>0.000298</v>
+        <v>0.171</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>0.001192</v>
+        <v>0.00025</v>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>0.0005</v>
       </c>
       <c r="K21" s="4" t="n">
-        <v>0.00149</v>
+        <v>0.00125</v>
       </c>
       <c r="L21" s="4" t="n">
-        <v>0.00149</v>
+        <v>0.00125</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>0.00149</v>
+        <v>0.00175</v>
       </c>
       <c r="N21" s="4" t="n">
-        <v>0.002682</v>
+        <v>0.0035</v>
       </c>
       <c r="O21" s="4" t="n">
-        <v>0.006258000000000001</v>
+        <v>0.007</v>
       </c>
       <c r="P21" s="4" t="n">
-        <v>0.01043</v>
+        <v>0.00775</v>
       </c>
       <c r="Q21" s="4" t="n">
-        <v>0.019072</v>
+        <v>0.01375</v>
       </c>
       <c r="R21" s="4" t="n">
-        <v>0.019966</v>
+        <v>0.02125</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.028608</v>
+        <v>0.0205</v>
       </c>
       <c r="T21" s="4" t="n">
-        <v>0.027714</v>
+        <v>0.0275</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.03427000000000001</v>
+        <v>0.0285</v>
       </c>
     </row>
     <row r="22">
@@ -1880,7 +1877,7 @@
         <v>21</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>0.118306</v>
+        <v>0.0925</v>
       </c>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
@@ -1888,37 +1885,35 @@
       <c r="G22" s="2" t="n"/>
       <c r="H22" s="2" t="n"/>
       <c r="I22" s="2" t="n"/>
-      <c r="J22" s="3" t="n">
-        <v>0.000298</v>
-      </c>
+      <c r="J22" s="2" t="n"/>
       <c r="K22" s="2" t="n"/>
       <c r="L22" s="2" t="n"/>
       <c r="M22" s="3" t="n">
-        <v>0.000298</v>
+        <v>0.00025</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>0.0005960000000000001</v>
+        <v>0.0005</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>0.001192</v>
+        <v>0.001</v>
       </c>
       <c r="P22" s="3" t="n">
-        <v>0.003576000000000001</v>
+        <v>0.0025</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>0.006258000000000001</v>
+        <v>0.0055</v>
       </c>
       <c r="R22" s="3" t="n">
-        <v>0.006556</v>
+        <v>0.00825</v>
       </c>
       <c r="S22" s="3" t="n">
-        <v>0.012218</v>
+        <v>0.0095</v>
       </c>
       <c r="T22" s="3" t="n">
-        <v>0.02235</v>
+        <v>0.01575</v>
       </c>
       <c r="U22" s="3" t="n">
-        <v>0.027118</v>
+        <v>0.0215</v>
       </c>
     </row>
     <row r="23">
@@ -1931,38 +1926,35 @@
         <v>22</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>0.09917080405271408</v>
-      </c>
-      <c r="P23" s="4" t="n">
-        <v>0.002023893960259471</v>
+        <v>0.0850229801549332</v>
       </c>
       <c r="Q23" s="4" t="n">
-        <v>0.002023893960259471</v>
+        <v>0.001604207172734589</v>
       </c>
       <c r="R23" s="4" t="n">
-        <v>0.006071681880778414</v>
+        <v>0.003208414345469178</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.006071681880778414</v>
+        <v>0.004812621518203767</v>
       </c>
       <c r="T23" s="4" t="n">
-        <v>0.01214336376155683</v>
+        <v>0.01283365738187671</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.01821504564233524</v>
+        <v>0.02085469324554965</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>emilian_s</t>
+          <t>sfv</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
         <v>23</v>
       </c>
       <c r="C24" s="3" t="n">
-        <v>0.09652633751593225</v>
+        <v>0.08275577633396113</v>
       </c>
       <c r="D24" s="2" t="n"/>
       <c r="E24" s="2" t="n"/>
@@ -1979,38 +1971,35 @@
       <c r="P24" s="2" t="n"/>
       <c r="Q24" s="2" t="n"/>
       <c r="R24" s="3" t="n">
-        <v>0.005362574306440681</v>
+        <v>0.004355567175471638</v>
       </c>
       <c r="S24" s="3" t="n">
-        <v>0.005362574306440681</v>
+        <v>0.004355567175471638</v>
       </c>
       <c r="T24" s="3" t="n">
-        <v>0.01072514861288136</v>
+        <v>0.004355567175471638</v>
       </c>
       <c r="U24" s="3" t="n">
-        <v>0.0268128715322034</v>
+        <v>0.02613340305282983</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>sfv</t>
+          <t>emilian_s</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>24</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>0.09390580362346135</v>
+        <v>0.08050909089802928</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>0.003756232144938454</v>
-      </c>
-      <c r="T25" s="4" t="n">
-        <v>0.01126869643481536</v>
+        <v>0.008945454544225476</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.01126869643481536</v>
+        <v>0.01341818181633821</v>
       </c>
     </row>
     <row r="26">
@@ -2023,7 +2012,7 @@
         <v>25</v>
       </c>
       <c r="C26" s="3" t="n">
-        <v>0.09130942297598842</v>
+        <v>0.07828311297667045</v>
       </c>
       <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="n"/>
@@ -2041,10 +2030,10 @@
       <c r="Q26" s="2" t="n"/>
       <c r="R26" s="2" t="n"/>
       <c r="S26" s="2" t="n"/>
-      <c r="T26" s="3" t="n">
-        <v>0.09130942297598842</v>
-      </c>
-      <c r="U26" s="2" t="n"/>
+      <c r="T26" s="2" t="n"/>
+      <c r="U26" s="3" t="n">
+        <v>0.03914155648833523</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2056,10 +2045,7 @@
         <v>26</v>
       </c>
       <c r="C27" s="4" t="n">
-        <v>0.08873742238943043</v>
-      </c>
-      <c r="U27" s="4" t="n">
-        <v>0.05915828159295362</v>
+        <v>0.07607803702797535</v>
       </c>
     </row>
     <row r="28">
@@ -2072,7 +2058,7 @@
         <v>27</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>0.08619003519239145</v>
+        <v>0.07389406309361407</v>
       </c>
       <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="n"/>
@@ -2103,7 +2089,7 @@
         <v>28</v>
       </c>
       <c r="C29" s="4" t="n">
-        <v>0.08366750154394066</v>
+        <v>0.07173139707127972</v>
       </c>
     </row>
     <row r="30">
@@ -2116,7 +2102,7 @@
         <v>29</v>
       </c>
       <c r="C30" s="3" t="n">
-        <v>0.08117006877353256</v>
+        <v>0.06959025100611502</v>
       </c>
       <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="n"/>
@@ -2147,20 +2133,20 @@
         <v>30</v>
       </c>
       <c r="C31" s="4" t="n">
-        <v>0.07869799174509248</v>
+        <v>0.06747084340285707</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Alina_97</t>
+          <t>Cordell</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
         <v>31</v>
       </c>
       <c r="C32" s="3" t="n">
-        <v>0.07625153324752322</v>
+        <v>0.06537339956063376</v>
       </c>
       <c r="D32" s="2" t="n"/>
       <c r="E32" s="2" t="n"/>
@@ -2184,14 +2170,14 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Cordell</t>
+          <t>Alina_97</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>32</v>
       </c>
       <c r="C33" s="4" t="n">
-        <v>0.0738309644141493</v>
+        <v>0.06329815193256971</v>
       </c>
     </row>
     <row r="34">
@@ -2204,7 +2190,7 @@
         <v>33</v>
       </c>
       <c r="C34" s="3" t="n">
-        <v>0.07143656517391686</v>
+        <v>0.06124534051261734</v>
       </c>
       <c r="D34" s="2" t="n"/>
       <c r="E34" s="2" t="n"/>
@@ -2235,7 +2221,7 @@
         <v>34</v>
       </c>
       <c r="C35" s="4" t="n">
-        <v>0.06906862473750806</v>
+        <v>0.05921521325232173</v>
       </c>
     </row>
     <row r="36">
@@ -2248,7 +2234,7 @@
         <v>35</v>
       </c>
       <c r="C36" s="3" t="n">
-        <v>0.06672744212192308</v>
+        <v>0.05720802651056506</v>
       </c>
       <c r="D36" s="2" t="n"/>
       <c r="E36" s="2" t="n"/>
@@ -2272,27 +2258,27 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Suruchik</t>
+          <t>Ryumon_Hozukimaruu</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>36</v>
       </c>
       <c r="C37" s="4" t="n">
-        <v>0.06441332671753436</v>
+        <v>0.05522404553972425</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Retbin</t>
+          <t>Suruchik</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
         <v>37</v>
       </c>
       <c r="C38" s="3" t="n">
-        <v>0.06212659890213935</v>
+        <v>0.05326354501212222</v>
       </c>
       <c r="D38" s="2" t="n"/>
       <c r="E38" s="2" t="n"/>
@@ -2323,7 +2309,7 @@
         <v>38</v>
       </c>
       <c r="C39" s="4" t="n">
-        <v>0.05986759070714237</v>
+        <v>0.05132680959117145</v>
       </c>
     </row>
     <row r="40">
@@ -2336,7 +2322,7 @@
         <v>39</v>
       </c>
       <c r="C40" s="3" t="n">
-        <v>0.05763664654169758</v>
+        <v>0.04941413455220986</v>
       </c>
       <c r="D40" s="2" t="n"/>
       <c r="E40" s="2" t="n"/>
@@ -2360,27 +2346,27 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Ryumon_Hozukimaruu</t>
+          <t>Retbin</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>40</v>
       </c>
       <c r="C41" s="4" t="n">
-        <v>0.05543412398146273</v>
+        <v>0.04752582645873005</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>БОЛЬШОЙ МИХА</t>
+          <t>Davydovpussy</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
         <v>41</v>
       </c>
       <c r="C42" s="3" t="n">
-        <v>0.05326039462957088</v>
+        <v>0.04566220390052374</v>
       </c>
       <c r="D42" s="2" t="n"/>
       <c r="E42" s="2" t="n"/>
@@ -2404,27 +2390,27 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Rik_dds</t>
+          <t>БОЛЬШОЙ МИХА</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>42</v>
       </c>
       <c r="C43" s="4" t="n">
-        <v>0.0511158450585511</v>
+        <v>0.04382359830122694</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Davydovpussy</t>
+          <t>Rik_dds</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
         <v>43</v>
       </c>
       <c r="C44" s="3" t="n">
-        <v>0.04900087784325523</v>
+        <v>0.04201035480388823</v>
       </c>
       <c r="D44" s="2" t="n"/>
       <c r="E44" s="2" t="n"/>
@@ -2455,7 +2441,7 @@
         <v>44</v>
       </c>
       <c r="C45" s="4" t="n">
-        <v>0.04691591269641866</v>
+        <v>0.04022283324452903</v>
       </c>
     </row>
     <row r="46">
@@ -2468,7 +2454,7 @@
         <v>45</v>
       </c>
       <c r="C46" s="3" t="n">
-        <v>0.04486138772035221</v>
+        <v>0.03846140922526767</v>
       </c>
       <c r="D46" s="2" t="n"/>
       <c r="E46" s="2" t="n"/>
@@ -2492,27 +2478,27 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Qrexi</t>
+          <t>Никита</t>
         </is>
       </c>
       <c r="B47" t="n">
         <v>46</v>
       </c>
       <c r="C47" s="4" t="n">
-        <v>0.04283776079049762</v>
+        <v>0.03672647530049522</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Никита</t>
+          <t>Qrexi</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
         <v>47</v>
       </c>
       <c r="C48" s="3" t="n">
-        <v>0.04084551108926481</v>
+        <v>0.03501844229189371</v>
       </c>
       <c r="D48" s="2" t="n"/>
       <c r="E48" s="2" t="n"/>
@@ -2543,7 +2529,7 @@
         <v>48</v>
       </c>
       <c r="C49" s="4" t="n">
-        <v>0.03888514081181586</v>
+        <v>0.03333774075087094</v>
       </c>
     </row>
     <row r="50">
@@ -2556,7 +2542,7 @@
         <v>49</v>
       </c>
       <c r="C50" s="3" t="n">
-        <v>0.03695717706940388</v>
+        <v>0.03168482259036684</v>
       </c>
       <c r="D50" s="2" t="n"/>
       <c r="E50" s="2" t="n"/>
@@ -2587,7 +2573,7 @@
         <v>50</v>
       </c>
       <c r="C51" s="4" t="n">
-        <v>0.03506217402069824</v>
+        <v>0.03006016291212127</v>
       </c>
     </row>
     <row r="52">
@@ -2600,7 +2586,7 @@
         <v>51</v>
       </c>
       <c r="C52" s="3" t="n">
-        <v>0.03320071526746089</v>
+        <v>0.02846426206058033</v>
       </c>
       <c r="D52" s="2" t="n"/>
       <c r="E52" s="2" t="n"/>
@@ -2631,7 +2617,7 @@
         <v>52</v>
       </c>
       <c r="C53" s="4" t="n">
-        <v>0.03137341655829062</v>
+        <v>0.02689764794092131</v>
       </c>
     </row>
     <row r="54">
@@ -2644,7 +2630,7 @@
         <v>53</v>
       </c>
       <c r="C54" s="3" t="n">
-        <v>0.02958092885332818</v>
+        <v>0.02536087864654337</v>
       </c>
       <c r="D54" s="2" t="n"/>
       <c r="E54" s="2" t="n"/>
@@ -2675,7 +2661,7 @@
         <v>54</v>
       </c>
       <c r="C55" s="4" t="n">
-        <v>0.02782394181435892</v>
+        <v>0.02385454545126794</v>
       </c>
     </row>
     <row r="56">
@@ -2688,7 +2674,7 @@
         <v>55</v>
       </c>
       <c r="C56" s="3" t="n">
-        <v>0.02610318779939383</v>
+        <v>0.0223792762340482</v>
       </c>
       <c r="D56" s="2" t="n"/>
       <c r="E56" s="2" t="n"/>
@@ -2719,7 +2705,7 @@
         <v>56</v>
       </c>
       <c r="C57" s="4" t="n">
-        <v>0.02441944645956044</v>
+        <v>0.02093573942006211</v>
       </c>
     </row>
     <row r="58">
@@ -2732,7 +2718,7 @@
         <v>57</v>
       </c>
       <c r="C58" s="3" t="n">
-        <v>0.02277355006037658</v>
+        <v>0.01952464854284687</v>
       </c>
       <c r="D58" s="2" t="n"/>
       <c r="E58" s="2" t="n"/>
@@ -2763,20 +2749,20 @@
         <v>58</v>
       </c>
       <c r="C59" s="4" t="n">
-        <v>0.02116638968116055</v>
+        <v>0.01814676755929403</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>He3hAy</t>
+          <t>elli</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
         <v>59</v>
       </c>
       <c r="C60" s="3" t="n">
-        <v>0.01959892248821406</v>
+        <v>0.01680291708523153</v>
       </c>
       <c r="D60" s="2" t="n"/>
       <c r="E60" s="2" t="n"/>
@@ -2800,14 +2786,14 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>elli</t>
+          <t>He3hAy</t>
         </is>
       </c>
       <c r="B61" t="n">
         <v>60</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>0.01807218033349118</v>
+        <v>0.01549398176739642</v>
       </c>
     </row>
     <row r="62">
@@ -2820,7 +2806,7 @@
         <v>61</v>
       </c>
       <c r="C62" s="3" t="n">
-        <v>0.01658728000659684</v>
+        <v>0.01422091907287109</v>
       </c>
       <c r="D62" s="2" t="n"/>
       <c r="E62" s="2" t="n"/>
@@ -2844,27 +2830,27 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>repe_kate</t>
+          <t>Mar_u_shka</t>
         </is>
       </c>
       <c r="B63" t="n">
         <v>62</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>0.01514543557290403</v>
+        <v>0.01298476986703021</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Mar_u_shka</t>
+          <t>repe_kate</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
         <v>63</v>
       </c>
       <c r="C64" s="3" t="n">
-        <v>0.01374797337771438</v>
+        <v>0.01178667127718997</v>
       </c>
       <c r="D64" s="2" t="n"/>
       <c r="E64" s="2" t="n"/>
@@ -2895,7 +2881,7 @@
         <v>64</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>0.01239635050658926</v>
+        <v>0.01062787251936665</v>
       </c>
     </row>
     <row r="66">
@@ -2908,7 +2894,7 @@
         <v>65</v>
       </c>
       <c r="C66" s="3" t="n">
-        <v>0.0110921777986788</v>
+        <v>0.009509754628496918</v>
       </c>
       <c r="D66" s="2" t="n"/>
       <c r="E66" s="2" t="n"/>
@@ -2932,27 +2918,27 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Tim19</t>
+          <t>Fara</t>
         </is>
       </c>
       <c r="B67" t="n">
         <v>66</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>0.00983724896813656</v>
+        <v>0.008433855425357134</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>edimerfi</t>
+          <t>Tim19</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
         <v>67</v>
       </c>
       <c r="C68" s="3" t="n">
-        <v>0.008633578092188508</v>
+        <v>0.007401901656540216</v>
       </c>
       <c r="D68" s="2" t="n"/>
       <c r="E68" s="2" t="n"/>
@@ -2976,14 +2962,14 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Fara</t>
+          <t>twewefe</t>
         </is>
       </c>
       <c r="B69" t="n">
         <v>68</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>0.007483448838392796</v>
+        <v>0.006415851198896431</v>
       </c>
     </row>
     <row r="70">
@@ -2996,7 +2982,7 @@
         <v>69</v>
       </c>
       <c r="C70" s="3" t="n">
-        <v>0.006389480632318888</v>
+        <v>0.005477949787653368</v>
       </c>
       <c r="D70" s="2" t="n"/>
       <c r="E70" s="2" t="n"/>
@@ -3020,27 +3006,27 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>katerina_boc</t>
+          <t>Shuricspinoza</t>
         </is>
       </c>
       <c r="B71" t="n">
         <v>70</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>0.005354720098812203</v>
+        <v>0.004590809412561903</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Shuricspinoza</t>
+          <t>nsa</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
         <v>71</v>
       </c>
       <c r="C72" s="3" t="n">
-        <v>0.00438277175258728</v>
+        <v>0.003757520364015158</v>
       </c>
       <c r="D72" s="2" t="n"/>
       <c r="E72" s="2" t="n"/>
@@ -3064,27 +3050,27 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>rus210385</t>
+          <t>katerina_boc</t>
         </is>
       </c>
       <c r="B73" t="n">
         <v>72</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0.003477992726794865</v>
+        <v>0.002981818181408492</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>twewefe</t>
+          <t>rus210385</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
         <v>73</v>
       </c>
       <c r="C74" s="3" t="n">
-        <v>0.002645798710145069</v>
+        <v>0.002268345944911754</v>
       </c>
       <c r="D74" s="2" t="n"/>
       <c r="E74" s="2" t="n"/>
@@ -3115,20 +3101,20 @@
         <v>74</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>0.001893179446613004</v>
+        <v>0.001623096233378776</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>nsa</t>
+          <t>DanilaOdinokov</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
         <v>75</v>
       </c>
       <c r="C76" s="3" t="n">
-        <v>0.00122965612101707</v>
+        <v>0.001054231928169642</v>
       </c>
       <c r="D76" s="2" t="n"/>
       <c r="E76" s="2" t="n"/>
@@ -3159,13 +3145,13 @@
         <v>76</v>
       </c>
       <c r="C77" s="4" t="n">
-        <v>0.0006693400123515253</v>
+        <v>0.0005738511765702378</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>DanilaOdinokov</t>
+          <t>edimerfi</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">

</xml_diff>

<commit_message>
playoff cutoff back to 18
</commit_message>
<xml_diff>
--- a/data/playoff_odds.xlsx
+++ b/data/playoff_odds.xlsx
@@ -591,7 +591,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Гризли</t>
+          <t>Noize MC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -601,60 +601,62 @@
         <v>0.25</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.039</v>
+        <v>0.04175</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.034</v>
+        <v>0.0335</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.02475</v>
+        <v>0.024</v>
       </c>
       <c r="G2" s="3" t="n">
+        <v>0.02525</v>
+      </c>
+      <c r="H2" s="3" t="n">
         <v>0.0235</v>
       </c>
-      <c r="H2" s="3" t="n">
-        <v>0.0245</v>
-      </c>
       <c r="I2" s="3" t="n">
-        <v>0.0195</v>
+        <v>0.0215</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.0155</v>
+        <v>0.016</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>0.01475</v>
+        <v>0.01425</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>0.01725</v>
+        <v>0.01675</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>0.01325</v>
+        <v>0.00975</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>0.00775</v>
+        <v>0.00725</v>
       </c>
       <c r="O2" s="3" t="n">
-        <v>0.0065</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="P2" s="3" t="n">
-        <v>0.0055</v>
+        <v>0.00375</v>
       </c>
       <c r="Q2" s="3" t="n">
-        <v>0.00175</v>
+        <v>0.002</v>
       </c>
       <c r="R2" s="3" t="n">
         <v>0.001</v>
       </c>
       <c r="S2" s="3" t="n">
-        <v>0.0015</v>
-      </c>
-      <c r="T2" s="2" t="n"/>
+        <v>0.00075</v>
+      </c>
+      <c r="T2" s="3" t="n">
+        <v>0.0005</v>
+      </c>
       <c r="U2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Драйв</t>
+          <t>Гризли</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -664,64 +666,58 @@
         <v>0.25</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>0.03225</v>
+        <v>0.03825</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0.03275</v>
+        <v>0.027</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>0.02375</v>
+        <v>0.03025</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.02775</v>
+        <v>0.0235</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>0.01925</v>
+        <v>0.02425</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>0.02325</v>
+        <v>0.02</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>0.01725</v>
+        <v>0.01875</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>0.0155</v>
+        <v>0.01475</v>
       </c>
       <c r="L3" s="4" t="n">
-        <v>0.013</v>
+        <v>0.012</v>
       </c>
       <c r="M3" s="4" t="n">
-        <v>0.01425</v>
+        <v>0.01175</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>0.011</v>
+        <v>0.0115</v>
       </c>
       <c r="O3" s="4" t="n">
-        <v>0.01</v>
+        <v>0.0075</v>
       </c>
       <c r="P3" s="4" t="n">
         <v>0.005</v>
       </c>
       <c r="Q3" s="4" t="n">
-        <v>0.0025</v>
+        <v>0.00325</v>
       </c>
       <c r="R3" s="4" t="n">
         <v>0.00175</v>
       </c>
-      <c r="S3" s="4" t="n">
-        <v>0.00025</v>
-      </c>
       <c r="T3" s="4" t="n">
-        <v>0.00025</v>
-      </c>
-      <c r="U3" s="4" t="n">
-        <v>0.00025</v>
+        <v>0.0005</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Yanchik_250</t>
+          <t>кинчоч</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -731,131 +727,131 @@
         <v>0.25</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.00775</v>
+        <v>0.01975</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.0125</v>
+        <v>0.0205</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.0185</v>
+        <v>0.02325</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0.0165</v>
+        <v>0.018</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.02325</v>
+        <v>0.02175</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.01775</v>
+        <v>0.022</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.02275</v>
+        <v>0.02175</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>0.021</v>
+        <v>0.02</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>0.02</v>
+        <v>0.02175</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>0.0215</v>
+        <v>0.0175</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>0.019</v>
+        <v>0.01475</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>0.01975</v>
+        <v>0.011</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>0.008750000000000001</v>
+        <v>0.00725</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>0.00975</v>
+        <v>0.00475</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>0.007</v>
+        <v>0.004</v>
       </c>
       <c r="S4" s="3" t="n">
         <v>0.00125</v>
       </c>
       <c r="T4" s="3" t="n">
-        <v>0.00225</v>
+        <v>0.0005</v>
       </c>
       <c r="U4" s="3" t="n">
-        <v>0.00075</v>
+        <v>0.00025</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Пассажир</t>
+          <t>G_rant_999</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>0.24975</v>
+        <v>0.25</v>
       </c>
       <c r="D5" s="4" t="n">
+        <v>0.01325</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>0.02025</v>
+      </c>
+      <c r="G5" s="4" t="n">
         <v>0.0195</v>
       </c>
-      <c r="E5" s="4" t="n">
-        <v>0.0195</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>0.0245</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>0.01875</v>
-      </c>
       <c r="H5" s="4" t="n">
-        <v>0.022</v>
+        <v>0.01975</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>0.0195</v>
+        <v>0.0225</v>
       </c>
       <c r="J5" s="4" t="n">
+        <v>0.0185</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>0.0205</v>
+      </c>
+      <c r="L5" s="4" t="n">
         <v>0.019</v>
       </c>
-      <c r="K5" s="4" t="n">
-        <v>0.02425</v>
-      </c>
-      <c r="L5" s="4" t="n">
-        <v>0.0215</v>
-      </c>
       <c r="M5" s="4" t="n">
-        <v>0.01725</v>
+        <v>0.01975</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v>0.0145</v>
+        <v>0.01825</v>
       </c>
       <c r="O5" s="4" t="n">
-        <v>0.0105</v>
+        <v>0.016</v>
       </c>
       <c r="P5" s="4" t="n">
-        <v>0.00975</v>
+        <v>0.01225</v>
       </c>
       <c r="Q5" s="4" t="n">
-        <v>0.0045</v>
+        <v>0.0065</v>
       </c>
       <c r="R5" s="4" t="n">
-        <v>0.0035</v>
+        <v>0.00325</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>0.00075</v>
+        <v>0.00125</v>
       </c>
       <c r="T5" s="4" t="n">
-        <v>0.00025</v>
+        <v>0.0005</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>0.00025</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>G_rant_999</t>
+          <t>terzzzzzzzzz</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -865,122 +861,122 @@
         <v>0.24975</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0.0165</v>
+        <v>0.01125</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.016</v>
+        <v>0.013</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0.01625</v>
+        <v>0.0175</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0.01925</v>
+        <v>0.01525</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>0.02025</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.01825</v>
+        <v>0.01975</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.02075</v>
+        <v>0.01975</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>0.02025</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>0.01825</v>
+        <v>0.02</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>0.018</v>
+        <v>0.024</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>0.01725</v>
+        <v>0.01925</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>0.01775</v>
+        <v>0.016</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>0.01325</v>
+        <v>0.015</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>0.01075</v>
+        <v>0.008</v>
       </c>
       <c r="R6" s="3" t="n">
+        <v>0.0055</v>
+      </c>
+      <c r="S6" s="3" t="n">
         <v>0.0025</v>
       </c>
-      <c r="S6" s="3" t="n">
-        <v>0.002</v>
-      </c>
       <c r="T6" s="3" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="U6" s="3" t="n">
         <v>0.0015</v>
-      </c>
-      <c r="U6" s="3" t="n">
-        <v>0.001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Laches1</t>
+          <t>Сокол</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>6</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>0.24975</v>
+        <v>0.2495</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.01325</v>
       </c>
       <c r="E7" s="4" t="n">
+        <v>0.01375</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>0.02075</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>0.01675</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>0.02075</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>0.0195</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>0.01875</v>
+      </c>
+      <c r="M7" s="4" t="n">
+        <v>0.02025</v>
+      </c>
+      <c r="N7" s="4" t="n">
+        <v>0.02025</v>
+      </c>
+      <c r="O7" s="4" t="n">
+        <v>0.01575</v>
+      </c>
+      <c r="P7" s="4" t="n">
+        <v>0.01375</v>
+      </c>
+      <c r="Q7" s="4" t="n">
         <v>0.0095</v>
       </c>
-      <c r="F7" s="4" t="n">
-        <v>0.01425</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>0.019</v>
-      </c>
-      <c r="H7" s="4" t="n">
-        <v>0.02075</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="J7" s="4" t="n">
-        <v>0.0175</v>
-      </c>
-      <c r="K7" s="4" t="n">
-        <v>0.021</v>
-      </c>
-      <c r="L7" s="4" t="n">
-        <v>0.022</v>
-      </c>
-      <c r="M7" s="4" t="n">
-        <v>0.02425</v>
-      </c>
-      <c r="N7" s="4" t="n">
-        <v>0.0245</v>
-      </c>
-      <c r="O7" s="4" t="n">
-        <v>0.0145</v>
-      </c>
-      <c r="P7" s="4" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="Q7" s="4" t="n">
-        <v>0.006</v>
-      </c>
       <c r="R7" s="4" t="n">
-        <v>0.0045</v>
+        <v>0.0055</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.004</v>
+        <v>0.00225</v>
       </c>
       <c r="T7" s="4" t="n">
-        <v>0.0025</v>
+        <v>0.00325</v>
       </c>
       <c r="U7" s="4" t="n">
         <v>0.001</v>
@@ -989,69 +985,67 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Noize MC</t>
+          <t>Драйв</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
         <v>7</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>0.24975</v>
+        <v>0.2495</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0.04575</v>
+        <v>0.03175</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.0275</v>
+        <v>0.0325</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0.0305</v>
+        <v>0.021</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>0.02425</v>
+        <v>0.02875</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.01975</v>
+        <v>0.02275</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>0.01875</v>
+        <v>0.02175</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.0195</v>
+        <v>0.0175</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>0.01475</v>
+        <v>0.0175</v>
       </c>
       <c r="L8" s="3" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="M8" s="3" t="n">
         <v>0.0135</v>
       </c>
-      <c r="M8" s="3" t="n">
-        <v>0.012</v>
-      </c>
       <c r="N8" s="3" t="n">
-        <v>0.008750000000000001</v>
+        <v>0.0105</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>0.00525</v>
+        <v>0.00475</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>0.0045</v>
+        <v>0.00575</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>0.0025</v>
+        <v>0.00275</v>
       </c>
       <c r="R8" s="3" t="n">
         <v>0.0015</v>
       </c>
       <c r="S8" s="3" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="T8" s="3" t="n">
         <v>0.00025</v>
       </c>
-      <c r="T8" s="3" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="U8" s="3" t="n">
-        <v>0.00025</v>
-      </c>
+      <c r="U8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1063,134 +1057,134 @@
         <v>8</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>0.24975</v>
+        <v>0.2495</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>0.01825</v>
+        <v>0.02275</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.0275</v>
+        <v>0.02875</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>0.02325</v>
+        <v>0.02375</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.01875</v>
+        <v>0.0235</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>0.0195</v>
+        <v>0.02075</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>0.018</v>
+        <v>0.02025</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>0.0225</v>
+        <v>0.022</v>
       </c>
       <c r="K9" s="4" t="n">
-        <v>0.024</v>
+        <v>0.01775</v>
       </c>
       <c r="L9" s="4" t="n">
-        <v>0.019</v>
+        <v>0.0165</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>0.01875</v>
+        <v>0.01675</v>
       </c>
       <c r="N9" s="4" t="n">
         <v>0.012</v>
       </c>
       <c r="O9" s="4" t="n">
-        <v>0.00975</v>
+        <v>0.0095</v>
       </c>
       <c r="P9" s="4" t="n">
-        <v>0.008</v>
+        <v>0.0065</v>
       </c>
       <c r="Q9" s="4" t="n">
-        <v>0.005</v>
+        <v>0.00425</v>
       </c>
       <c r="R9" s="4" t="n">
-        <v>0.00175</v>
+        <v>0.0025</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.00075</v>
+        <v>0.0015</v>
       </c>
       <c r="T9" s="4" t="n">
-        <v>0.00125</v>
+        <v>0.00025</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>0.001</v>
+        <v>0.00025</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>terzzzzzzzzz</t>
+          <t>Пассажир</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
         <v>9</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.24975</v>
+        <v>0.2495</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.01375</v>
+        <v>0.01825</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.01425</v>
+        <v>0.01875</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.01525</v>
+        <v>0.02225</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>0.01825</v>
+        <v>0.02375</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.01675</v>
+        <v>0.022</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>0.019</v>
+        <v>0.0225</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.01975</v>
+        <v>0.0215</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>0.01875</v>
+        <v>0.02175</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0.02075</v>
+        <v>0.01725</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>0.02125</v>
+        <v>0.0155</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.02075</v>
+        <v>0.016</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>0.017</v>
+        <v>0.0125</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>0.0145</v>
+        <v>0.00775</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.0045</v>
       </c>
       <c r="R10" s="3" t="n">
-        <v>0.0055</v>
+        <v>0.0015</v>
       </c>
       <c r="S10" s="3" t="n">
-        <v>0.0025</v>
+        <v>0.00175</v>
       </c>
       <c r="T10" s="3" t="n">
-        <v>0.00125</v>
+        <v>0.001</v>
       </c>
       <c r="U10" s="3" t="n">
-        <v>0.00075</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>кинчоч</t>
+          <t>Yanchik_250</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1200,58 +1194,58 @@
         <v>0.2495</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>0.02</v>
+        <v>0.0115</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0.025</v>
+        <v>0.0155</v>
       </c>
       <c r="F11" s="4" t="n">
+        <v>0.0145</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>0.01425</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>0.01825</v>
+      </c>
+      <c r="I11" s="4" t="n">
         <v>0.02025</v>
       </c>
-      <c r="G11" s="4" t="n">
-        <v>0.023</v>
-      </c>
-      <c r="H11" s="4" t="n">
+      <c r="J11" s="4" t="n">
         <v>0.02225</v>
       </c>
-      <c r="I11" s="4" t="n">
-        <v>0.0235</v>
-      </c>
-      <c r="J11" s="4" t="n">
-        <v>0.0195</v>
-      </c>
       <c r="K11" s="4" t="n">
-        <v>0.0195</v>
+        <v>0.021</v>
       </c>
       <c r="L11" s="4" t="n">
-        <v>0.018</v>
+        <v>0.0215</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>0.013</v>
+        <v>0.0205</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>0.0155</v>
+        <v>0.017</v>
       </c>
       <c r="O11" s="4" t="n">
-        <v>0.01175</v>
+        <v>0.01675</v>
       </c>
       <c r="P11" s="4" t="n">
-        <v>0.00775</v>
+        <v>0.01325</v>
       </c>
       <c r="Q11" s="4" t="n">
-        <v>0.004</v>
+        <v>0.008750000000000001</v>
       </c>
       <c r="R11" s="4" t="n">
-        <v>0.00225</v>
+        <v>0.00625</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.002</v>
+        <v>0.00375</v>
       </c>
       <c r="T11" s="4" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="U11" s="4" t="n">
         <v>0.00175</v>
-      </c>
-      <c r="U11" s="4" t="n">
-        <v>0.00025</v>
       </c>
     </row>
     <row r="12">
@@ -1264,128 +1258,128 @@
         <v>11</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>0.24925</v>
+        <v>0.249</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0.01375</v>
+        <v>0.01325</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.01675</v>
+        <v>0.01475</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.019</v>
+        <v>0.014</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0.02</v>
+        <v>0.0205</v>
       </c>
       <c r="H12" s="3" t="n">
+        <v>0.0215</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>0.02075</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>0.02075</v>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>0.02075</v>
+      </c>
+      <c r="L12" s="3" t="n">
+        <v>0.0235</v>
+      </c>
+      <c r="M12" s="3" t="n">
         <v>0.02025</v>
       </c>
-      <c r="I12" s="3" t="n">
-        <v>0.021</v>
-      </c>
-      <c r="J12" s="3" t="n">
-        <v>0.022</v>
-      </c>
-      <c r="K12" s="3" t="n">
-        <v>0.0165</v>
-      </c>
-      <c r="L12" s="3" t="n">
-        <v>0.01925</v>
-      </c>
-      <c r="M12" s="3" t="n">
-        <v>0.017</v>
-      </c>
       <c r="N12" s="3" t="n">
-        <v>0.01925</v>
+        <v>0.01775</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.01625</v>
+        <v>0.01775</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>0.01225</v>
+        <v>0.00775</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>0.00625</v>
+        <v>0.00475</v>
       </c>
       <c r="R12" s="3" t="n">
-        <v>0.00475</v>
+        <v>0.006</v>
       </c>
       <c r="S12" s="3" t="n">
         <v>0.0025</v>
       </c>
       <c r="T12" s="3" t="n">
-        <v>0.00125</v>
+        <v>0.001</v>
       </c>
       <c r="U12" s="3" t="n">
-        <v>0.00075</v>
+        <v>0.0015</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Сокол</t>
+          <t>Laches1</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>12</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>0.24925</v>
+        <v>0.2485</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>0.01425</v>
+        <v>0.0145</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.0135</v>
+        <v>0.01325</v>
       </c>
       <c r="F13" s="4" t="n">
+        <v>0.01675</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>0.01725</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>0.01575</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>0.0155</v>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="K13" s="4" t="n">
+        <v>0.02275</v>
+      </c>
+      <c r="L13" s="4" t="n">
+        <v>0.02225</v>
+      </c>
+      <c r="M13" s="4" t="n">
         <v>0.01825</v>
       </c>
-      <c r="G13" s="4" t="n">
-        <v>0.0175</v>
-      </c>
-      <c r="H13" s="4" t="n">
-        <v>0.01825</v>
-      </c>
-      <c r="I13" s="4" t="n">
-        <v>0.01925</v>
-      </c>
-      <c r="J13" s="4" t="n">
-        <v>0.02425</v>
-      </c>
-      <c r="K13" s="4" t="n">
-        <v>0.022</v>
-      </c>
-      <c r="L13" s="4" t="n">
-        <v>0.02175</v>
-      </c>
-      <c r="M13" s="4" t="n">
-        <v>0.02025</v>
-      </c>
       <c r="N13" s="4" t="n">
-        <v>0.01625</v>
+        <v>0.0215</v>
       </c>
       <c r="O13" s="4" t="n">
-        <v>0.013</v>
+        <v>0.0165</v>
       </c>
       <c r="P13" s="4" t="n">
-        <v>0.01225</v>
+        <v>0.015</v>
       </c>
       <c r="Q13" s="4" t="n">
-        <v>0.00675</v>
+        <v>0.00625</v>
       </c>
       <c r="R13" s="4" t="n">
+        <v>0.00525</v>
+      </c>
+      <c r="S13" s="4" t="n">
         <v>0.004</v>
       </c>
-      <c r="S13" s="4" t="n">
-        <v>0.0035</v>
-      </c>
       <c r="T13" s="4" t="n">
+        <v>0.00175</v>
+      </c>
+      <c r="U13" s="4" t="n">
         <v>0.001</v>
-      </c>
-      <c r="U13" s="4" t="n">
-        <v>0.00225</v>
       </c>
     </row>
     <row r="14">
@@ -1398,61 +1392,61 @@
         <v>13</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>0.23125</v>
+        <v>0.21525</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>0.00025</v>
       </c>
       <c r="E14" s="3" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="G14" s="3" t="n">
         <v>0.00075</v>
-      </c>
-      <c r="F14" s="3" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="G14" s="3" t="n">
-        <v>0.00125</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>0.00125</v>
       </c>
       <c r="I14" s="3" t="n">
+        <v>0.00175</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>0.00275</v>
+      </c>
+      <c r="K14" s="3" t="n">
         <v>0.00325</v>
       </c>
-      <c r="J14" s="3" t="n">
-        <v>0.00375</v>
-      </c>
-      <c r="K14" s="3" t="n">
-        <v>0.0025</v>
-      </c>
       <c r="L14" s="3" t="n">
-        <v>0.00575</v>
+        <v>0.00675</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0.008750000000000001</v>
+        <v>0.00925</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>0.014</v>
+        <v>0.0115</v>
       </c>
       <c r="O14" s="3" t="n">
         <v>0.021</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>0.03075</v>
+        <v>0.028</v>
       </c>
       <c r="Q14" s="3" t="n">
         <v>0.02925</v>
       </c>
       <c r="R14" s="3" t="n">
-        <v>0.02625</v>
+        <v>0.0295</v>
       </c>
       <c r="S14" s="3" t="n">
-        <v>0.023</v>
+        <v>0.031</v>
       </c>
       <c r="T14" s="3" t="n">
-        <v>0.023</v>
+        <v>0.019</v>
       </c>
       <c r="U14" s="3" t="n">
-        <v>0.021</v>
+        <v>0.0195</v>
       </c>
     </row>
     <row r="15">
@@ -1465,7 +1459,7 @@
         <v>14</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>0.22275</v>
+        <v>0.19825</v>
       </c>
       <c r="F15" s="4" t="n">
         <v>0.00025</v>
@@ -1474,59 +1468,59 @@
         <v>0.0005</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>0.001</v>
+        <v>0.0005</v>
       </c>
       <c r="I15" s="4" t="n">
-        <v>0.001</v>
+        <v>0.00075</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>0.00125</v>
+        <v>0.00225</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>0.00325</v>
+        <v>0.00475</v>
       </c>
       <c r="L15" s="4" t="n">
-        <v>0.0065</v>
+        <v>0.0045</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>0.00725</v>
+        <v>0.0075</v>
       </c>
       <c r="N15" s="4" t="n">
-        <v>0.01175</v>
+        <v>0.014</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>0.014</v>
+        <v>0.01375</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>0.01975</v>
+        <v>0.01475</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>0.0295</v>
+        <v>0.02975</v>
       </c>
       <c r="R15" s="4" t="n">
-        <v>0.031</v>
+        <v>0.03325</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.0275</v>
+        <v>0.02525</v>
       </c>
       <c r="T15" s="4" t="n">
-        <v>0.0255</v>
+        <v>0.02525</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.02075</v>
+        <v>0.02125</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Lock</t>
+          <t>Пиковая Дама</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
         <v>15</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>0.21575</v>
+        <v>0.19025</v>
       </c>
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
@@ -1534,58 +1528,65 @@
         <v>0.00025</v>
       </c>
       <c r="G16" s="3" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="H16" s="3" t="n">
         <v>0.00075</v>
       </c>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
+      <c r="I16" s="3" t="n">
+        <v>0.00175</v>
+      </c>
       <c r="J16" s="3" t="n">
-        <v>0.00175</v>
+        <v>0.0005</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>0.0015</v>
+        <v>0.00225</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>0.00325</v>
+        <v>0.002</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0.00375</v>
+        <v>0.0055</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0.011</v>
+        <v>0.0105</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>0.0115</v>
+        <v>0.013</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>0.0215</v>
+        <v>0.019</v>
       </c>
       <c r="Q16" s="3" t="n">
-        <v>0.02075</v>
+        <v>0.024</v>
       </c>
       <c r="R16" s="3" t="n">
-        <v>0.0275</v>
+        <v>0.02625</v>
       </c>
       <c r="S16" s="3" t="n">
-        <v>0.029</v>
+        <v>0.02775</v>
       </c>
       <c r="T16" s="3" t="n">
-        <v>0.031</v>
+        <v>0.02975</v>
       </c>
       <c r="U16" s="3" t="n">
-        <v>0.026</v>
+        <v>0.02675</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Пиковая Дама</t>
+          <t>Lock</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>16</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>0.21375</v>
+        <v>0.18975</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>0.0005</v>
       </c>
       <c r="F17" s="4" t="n">
         <v>0.00025</v>
@@ -1594,46 +1595,46 @@
         <v>0.0005</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>0.0005</v>
+        <v>0.00025</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>0.00125</v>
+        <v>0.00025</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>0.0005</v>
+        <v>0.00075</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>0.00475</v>
+        <v>0.00325</v>
       </c>
       <c r="L17" s="4" t="n">
-        <v>0.00375</v>
+        <v>0.00425</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>0.0065</v>
+        <v>0.00675</v>
       </c>
       <c r="N17" s="4" t="n">
-        <v>0.00475</v>
+        <v>0.00675</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>0.0135</v>
+        <v>0.0145</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>0.02</v>
+        <v>0.01925</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>0.0245</v>
+        <v>0.02725</v>
       </c>
       <c r="R17" s="4" t="n">
         <v>0.02575</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.033</v>
+        <v>0.02625</v>
       </c>
       <c r="T17" s="4" t="n">
-        <v>0.0325</v>
+        <v>0.0275</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.02175</v>
+        <v>0.02575</v>
       </c>
     </row>
     <row r="18">
@@ -1646,55 +1647,57 @@
         <v>17</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>0.19975</v>
-      </c>
-      <c r="D18" s="2" t="n"/>
+        <v>0.178</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>0.00025</v>
+      </c>
       <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
-      <c r="G18" s="3" t="n">
+      <c r="F18" s="3" t="n">
         <v>0.00025</v>
       </c>
+      <c r="G18" s="2" t="n"/>
       <c r="H18" s="3" t="n">
-        <v>0.0005</v>
+        <v>0.00025</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>0.00025</v>
+        <v>0.00075</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>0.00125</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>0.00125</v>
+        <v>0.00275</v>
       </c>
       <c r="L18" s="3" t="n">
         <v>0.00225</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>0.0055</v>
+        <v>0.0035</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>0.00775</v>
+        <v>0.008</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>0.013</v>
+        <v>0.01</v>
       </c>
       <c r="P18" s="3" t="n">
-        <v>0.014</v>
+        <v>0.0165</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>0.02275</v>
+        <v>0.021</v>
       </c>
       <c r="R18" s="3" t="n">
-        <v>0.02425</v>
+        <v>0.02925</v>
       </c>
       <c r="S18" s="3" t="n">
-        <v>0.027</v>
+        <v>0.02725</v>
       </c>
       <c r="T18" s="3" t="n">
-        <v>0.0235</v>
+        <v>0.02875</v>
       </c>
       <c r="U18" s="3" t="n">
-        <v>0.03325</v>
+        <v>0.026</v>
       </c>
     </row>
     <row r="19">
@@ -1707,19 +1710,19 @@
         <v>18</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.1945</v>
+        <v>0.1685</v>
       </c>
       <c r="D19" s="5" t="n"/>
-      <c r="E19" s="6" t="n">
+      <c r="E19" s="5" t="n"/>
+      <c r="F19" s="6" t="n">
         <v>0.0005</v>
       </c>
-      <c r="F19" s="6" t="n">
+      <c r="G19" s="6" t="n">
         <v>0.00025</v>
       </c>
-      <c r="G19" s="5" t="n"/>
       <c r="H19" s="5" t="n"/>
       <c r="I19" s="6" t="n">
-        <v>0.001</v>
+        <v>0.00075</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>0.00075</v>
@@ -1728,34 +1731,34 @@
         <v>0.0015</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>0.00125</v>
+        <v>0.00175</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>0.00275</v>
+        <v>0.0055</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>0.0055</v>
+        <v>0.00525</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>0.00775</v>
+        <v>0.01</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>0.012</v>
+        <v>0.015</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>0.01875</v>
+        <v>0.01925</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>0.02325</v>
+        <v>0.01775</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>0.029</v>
+        <v>0.0285</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>0.0315</v>
+        <v>0.02875</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>0.0285</v>
+        <v>0.033</v>
       </c>
     </row>
     <row r="20">
@@ -1768,51 +1771,51 @@
         <v>19</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>0.18775</v>
+        <v>0.1495</v>
       </c>
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="n"/>
       <c r="F20" s="2" t="n"/>
-      <c r="G20" s="3" t="n">
-        <v>0.00025</v>
-      </c>
+      <c r="G20" s="2" t="n"/>
       <c r="H20" s="2" t="n"/>
       <c r="I20" s="3" t="n">
         <v>0.00025</v>
       </c>
-      <c r="J20" s="2" t="n"/>
+      <c r="J20" s="3" t="n">
+        <v>0.0005</v>
+      </c>
       <c r="K20" s="3" t="n">
-        <v>0.00175</v>
+        <v>0.0015</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>0.00175</v>
+        <v>0.00225</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>0.00275</v>
+        <v>0.002</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>0.00475</v>
+        <v>0.00425</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>0.00925</v>
+        <v>0.008750000000000001</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>0.01025</v>
+        <v>0.012</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>0.01625</v>
+        <v>0.017</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>0.02175</v>
+        <v>0.02</v>
       </c>
       <c r="S20" s="3" t="n">
+        <v>0.02475</v>
+      </c>
+      <c r="T20" s="3" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="U20" s="3" t="n">
         <v>0.02875</v>
-      </c>
-      <c r="T20" s="3" t="n">
-        <v>0.02375</v>
-      </c>
-      <c r="U20" s="3" t="n">
-        <v>0.034</v>
       </c>
     </row>
     <row r="21">
@@ -1825,7 +1828,10 @@
         <v>20</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>0.171</v>
+        <v>0.134</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>0.00025</v>
       </c>
       <c r="I21" s="4" t="n">
         <v>0.00025</v>
@@ -1833,38 +1839,35 @@
       <c r="J21" s="4" t="n">
         <v>0.0005</v>
       </c>
-      <c r="K21" s="4" t="n">
-        <v>0.00125</v>
-      </c>
       <c r="L21" s="4" t="n">
-        <v>0.00125</v>
+        <v>0.001</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>0.00175</v>
+        <v>0.00225</v>
       </c>
       <c r="N21" s="4" t="n">
-        <v>0.0035</v>
+        <v>0.00275</v>
       </c>
       <c r="O21" s="4" t="n">
-        <v>0.007</v>
+        <v>0.005</v>
       </c>
       <c r="P21" s="4" t="n">
-        <v>0.00775</v>
+        <v>0.01</v>
       </c>
       <c r="Q21" s="4" t="n">
+        <v>0.01275</v>
+      </c>
+      <c r="R21" s="4" t="n">
         <v>0.01375</v>
       </c>
-      <c r="R21" s="4" t="n">
-        <v>0.02125</v>
-      </c>
       <c r="S21" s="4" t="n">
-        <v>0.0205</v>
+        <v>0.02175</v>
       </c>
       <c r="T21" s="4" t="n">
-        <v>0.0275</v>
+        <v>0.0325</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.0285</v>
+        <v>0.03125</v>
       </c>
     </row>
     <row r="22">
@@ -1877,7 +1880,7 @@
         <v>21</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>0.0925</v>
+        <v>0.08271522788301899</v>
       </c>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
@@ -1885,35 +1888,35 @@
       <c r="G22" s="2" t="n"/>
       <c r="H22" s="2" t="n"/>
       <c r="I22" s="2" t="n"/>
-      <c r="J22" s="2" t="n"/>
+      <c r="J22" s="3" t="n">
+        <v>0.0003121329354076188</v>
+      </c>
       <c r="K22" s="2" t="n"/>
       <c r="L22" s="2" t="n"/>
-      <c r="M22" s="3" t="n">
-        <v>0.00025</v>
-      </c>
+      <c r="M22" s="2" t="n"/>
       <c r="N22" s="3" t="n">
-        <v>0.0005</v>
+        <v>0.001248531741630475</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>0.001</v>
+        <v>0.001872797612445713</v>
       </c>
       <c r="P22" s="3" t="n">
-        <v>0.0025</v>
+        <v>0.002809196418668569</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>0.0055</v>
+        <v>0.00530625990192952</v>
       </c>
       <c r="R22" s="3" t="n">
-        <v>0.00825</v>
+        <v>0.0115489186100819</v>
       </c>
       <c r="S22" s="3" t="n">
-        <v>0.0095</v>
+        <v>0.01591877970578856</v>
       </c>
       <c r="T22" s="3" t="n">
-        <v>0.01575</v>
+        <v>0.01841584318904951</v>
       </c>
       <c r="U22" s="3" t="n">
-        <v>0.0215</v>
+        <v>0.02528276776801713</v>
       </c>
     </row>
     <row r="23">
@@ -1926,22 +1929,25 @@
         <v>22</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>0.0850229801549332</v>
+        <v>0.08054808646256829</v>
+      </c>
+      <c r="P23" s="4" t="n">
+        <v>0.002301373898930523</v>
       </c>
       <c r="Q23" s="4" t="n">
-        <v>0.001604207172734589</v>
+        <v>0.002301373898930523</v>
       </c>
       <c r="R23" s="4" t="n">
-        <v>0.003208414345469178</v>
+        <v>0.009205495595722091</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.004812621518203767</v>
+        <v>0.01380824339358314</v>
       </c>
       <c r="T23" s="4" t="n">
-        <v>0.01283365738187671</v>
+        <v>0.01380824339358314</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.02085469324554965</v>
+        <v>0.03912335628181889</v>
       </c>
     </row>
     <row r="24">
@@ -1954,7 +1960,7 @@
         <v>23</v>
       </c>
       <c r="C24" s="3" t="n">
-        <v>0.08275577633396113</v>
+        <v>0.07840020915848948</v>
       </c>
       <c r="D24" s="2" t="n"/>
       <c r="E24" s="2" t="n"/>
@@ -1970,17 +1976,15 @@
       <c r="O24" s="2" t="n"/>
       <c r="P24" s="2" t="n"/>
       <c r="Q24" s="2" t="n"/>
-      <c r="R24" s="3" t="n">
-        <v>0.004355567175471638</v>
-      </c>
+      <c r="R24" s="2" t="n"/>
       <c r="S24" s="3" t="n">
-        <v>0.004355567175471638</v>
+        <v>0.0156800418316979</v>
       </c>
       <c r="T24" s="3" t="n">
-        <v>0.004355567175471638</v>
+        <v>0.02352006274754685</v>
       </c>
       <c r="U24" s="3" t="n">
-        <v>0.02613340305282983</v>
+        <v>0.03920010457924474</v>
       </c>
     </row>
     <row r="25">
@@ -1993,13 +1997,19 @@
         <v>24</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>0.08050909089802928</v>
+        <v>0.07627177032444879</v>
+      </c>
+      <c r="R25" s="4" t="n">
+        <v>0.005867059255726829</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>0.008945454544225476</v>
+        <v>0.005867059255726829</v>
+      </c>
+      <c r="T25" s="4" t="n">
+        <v>0.02346823702290732</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.01341818181633821</v>
+        <v>0.04106941479008781</v>
       </c>
     </row>
     <row r="26">
@@ -2012,7 +2022,7 @@
         <v>25</v>
       </c>
       <c r="C26" s="3" t="n">
-        <v>0.07828311297667045</v>
+        <v>0.07416294913579306</v>
       </c>
       <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="n"/>
@@ -2032,7 +2042,7 @@
       <c r="S26" s="2" t="n"/>
       <c r="T26" s="2" t="n"/>
       <c r="U26" s="3" t="n">
-        <v>0.03914155648833523</v>
+        <v>0.07416294913579306</v>
       </c>
     </row>
     <row r="27">
@@ -2045,7 +2055,10 @@
         <v>26</v>
       </c>
       <c r="C27" s="4" t="n">
-        <v>0.07607803702797535</v>
+        <v>0.07207392981597664</v>
+      </c>
+      <c r="U27" s="4" t="n">
+        <v>0.07207392981597664</v>
       </c>
     </row>
     <row r="28">
@@ -2058,7 +2071,7 @@
         <v>27</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>0.07389406309361407</v>
+        <v>0.07000490187816071</v>
       </c>
       <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="n"/>
@@ -2077,7 +2090,9 @@
       <c r="R28" s="2" t="n"/>
       <c r="S28" s="2" t="n"/>
       <c r="T28" s="2" t="n"/>
-      <c r="U28" s="2" t="n"/>
+      <c r="U28" s="3" t="n">
+        <v>0.07000490187816071</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2089,7 +2104,10 @@
         <v>28</v>
       </c>
       <c r="C29" s="4" t="n">
-        <v>0.07173139707127972</v>
+        <v>0.06795606038331763</v>
+      </c>
+      <c r="U29" s="4" t="n">
+        <v>0.06795606038331763</v>
       </c>
     </row>
     <row r="30">
@@ -2102,7 +2120,7 @@
         <v>29</v>
       </c>
       <c r="C30" s="3" t="n">
-        <v>0.06959025100611502</v>
+        <v>0.06592760621631949</v>
       </c>
       <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="n"/>
@@ -2121,7 +2139,9 @@
       <c r="R30" s="2" t="n"/>
       <c r="S30" s="2" t="n"/>
       <c r="T30" s="2" t="n"/>
-      <c r="U30" s="2" t="n"/>
+      <c r="U30" s="3" t="n">
+        <v>0.06592760621631949</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2133,20 +2153,23 @@
         <v>30</v>
       </c>
       <c r="C31" s="4" t="n">
-        <v>0.06747084340285707</v>
+        <v>0.06391974638165407</v>
+      </c>
+      <c r="U31" s="4" t="n">
+        <v>0.06391974638165407</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Cordell</t>
+          <t>Alina_97</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
         <v>31</v>
       </c>
       <c r="C32" s="3" t="n">
-        <v>0.06537339956063376</v>
+        <v>0.06193269432060041</v>
       </c>
       <c r="D32" s="2" t="n"/>
       <c r="E32" s="2" t="n"/>
@@ -2165,19 +2188,24 @@
       <c r="R32" s="2" t="n"/>
       <c r="S32" s="2" t="n"/>
       <c r="T32" s="2" t="n"/>
-      <c r="U32" s="2" t="n"/>
+      <c r="U32" s="3" t="n">
+        <v>0.06193269432060041</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Alina_97</t>
+          <t>Cordell</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>32</v>
       </c>
       <c r="C33" s="4" t="n">
-        <v>0.06329815193256971</v>
+        <v>0.05996667025190814</v>
+      </c>
+      <c r="U33" s="4" t="n">
+        <v>0.05996667025190814</v>
       </c>
     </row>
     <row r="34">
@@ -2190,7 +2218,7 @@
         <v>33</v>
       </c>
       <c r="C34" s="3" t="n">
-        <v>0.06124534051261734</v>
+        <v>0.05802190153826906</v>
       </c>
       <c r="D34" s="2" t="n"/>
       <c r="E34" s="2" t="n"/>
@@ -2209,7 +2237,9 @@
       <c r="R34" s="2" t="n"/>
       <c r="S34" s="2" t="n"/>
       <c r="T34" s="2" t="n"/>
-      <c r="U34" s="2" t="n"/>
+      <c r="U34" s="3" t="n">
+        <v>0.05802190153826906</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2221,20 +2251,23 @@
         <v>34</v>
       </c>
       <c r="C35" s="4" t="n">
-        <v>0.05921521325232173</v>
+        <v>0.05609862308114691</v>
+      </c>
+      <c r="U35" s="4" t="n">
+        <v>0.05609862308114691</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Настя дай стек</t>
+          <t>Suruchik</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
         <v>35</v>
       </c>
       <c r="C36" s="3" t="n">
-        <v>0.05720802651056506</v>
+        <v>0.05419707774685112</v>
       </c>
       <c r="D36" s="2" t="n"/>
       <c r="E36" s="2" t="n"/>
@@ -2253,32 +2286,37 @@
       <c r="R36" s="2" t="n"/>
       <c r="S36" s="2" t="n"/>
       <c r="T36" s="2" t="n"/>
-      <c r="U36" s="2" t="n"/>
+      <c r="U36" s="3" t="n">
+        <v>0.05419707774685112</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Ryumon_Hozukimaruu</t>
+          <t>Настя дай стек</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>36</v>
       </c>
       <c r="C37" s="4" t="n">
-        <v>0.05522404553972425</v>
+        <v>0.05231751682710718</v>
+      </c>
+      <c r="U37" s="4" t="n">
+        <v>0.05231751682710718</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Suruchik</t>
+          <t>Yars</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
         <v>37</v>
       </c>
       <c r="C38" s="3" t="n">
-        <v>0.05326354501212222</v>
+        <v>0.0504602005378</v>
       </c>
       <c r="D38" s="2" t="n"/>
       <c r="E38" s="2" t="n"/>
@@ -2297,32 +2335,37 @@
       <c r="R38" s="2" t="n"/>
       <c r="S38" s="2" t="n"/>
       <c r="T38" s="2" t="n"/>
-      <c r="U38" s="2" t="n"/>
+      <c r="U38" s="3" t="n">
+        <v>0.0504602005378</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Yars</t>
+          <t>Ryumon_Hozukimaruu</t>
         </is>
       </c>
       <c r="B39" t="n">
         <v>38</v>
       </c>
       <c r="C39" s="4" t="n">
-        <v>0.05132680959117145</v>
+        <v>0.04862539856005715</v>
+      </c>
+      <c r="U39" s="4" t="n">
+        <v>0.04862539856005715</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>springbulk</t>
+          <t>Retbin</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
         <v>39</v>
       </c>
       <c r="C40" s="3" t="n">
-        <v>0.04941413455220986</v>
+        <v>0.04681339062840933</v>
       </c>
       <c r="D40" s="2" t="n"/>
       <c r="E40" s="2" t="n"/>
@@ -2341,32 +2384,37 @@
       <c r="R40" s="2" t="n"/>
       <c r="S40" s="2" t="n"/>
       <c r="T40" s="2" t="n"/>
-      <c r="U40" s="2" t="n"/>
+      <c r="U40" s="3" t="n">
+        <v>0.04681339062840933</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Retbin</t>
+          <t>springbulk</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>40</v>
       </c>
       <c r="C41" s="4" t="n">
-        <v>0.04752582645873005</v>
+        <v>0.04502446717142847</v>
+      </c>
+      <c r="U41" s="4" t="n">
+        <v>0.04502446717142847</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Davydovpussy</t>
+          <t>БОЛЬШОЙ МИХА</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
         <v>41</v>
       </c>
       <c r="C42" s="3" t="n">
-        <v>0.04566220390052374</v>
+        <v>0.04325893001102249</v>
       </c>
       <c r="D42" s="2" t="n"/>
       <c r="E42" s="2" t="n"/>
@@ -2385,32 +2433,37 @@
       <c r="R42" s="2" t="n"/>
       <c r="S42" s="2" t="n"/>
       <c r="T42" s="2" t="n"/>
-      <c r="U42" s="2" t="n"/>
+      <c r="U42" s="3" t="n">
+        <v>0.04325893001102249</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>БОЛЬШОЙ МИХА</t>
+          <t>Rik_dds</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>42</v>
       </c>
       <c r="C43" s="4" t="n">
-        <v>0.04382359830122694</v>
+        <v>0.04151709312747816</v>
+      </c>
+      <c r="U43" s="4" t="n">
+        <v>0.04151709312747816</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Rik_dds</t>
+          <t>Davydovpussy</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
         <v>43</v>
       </c>
       <c r="C44" s="3" t="n">
-        <v>0.04201035480388823</v>
+        <v>0.03979928349842043</v>
       </c>
       <c r="D44" s="2" t="n"/>
       <c r="E44" s="2" t="n"/>
@@ -2429,7 +2482,9 @@
       <c r="R44" s="2" t="n"/>
       <c r="S44" s="2" t="n"/>
       <c r="T44" s="2" t="n"/>
-      <c r="U44" s="2" t="n"/>
+      <c r="U44" s="3" t="n">
+        <v>0.03979928349842043</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2441,7 +2496,10 @@
         <v>44</v>
       </c>
       <c r="C45" s="4" t="n">
-        <v>0.04022283324452903</v>
+        <v>0.03810584202113276</v>
+      </c>
+      <c r="U45" s="4" t="n">
+        <v>0.03810584202113276</v>
       </c>
     </row>
     <row r="46">
@@ -2454,7 +2512,7 @@
         <v>45</v>
       </c>
       <c r="C46" s="3" t="n">
-        <v>0.03846140922526767</v>
+        <v>0.03643712452920096</v>
       </c>
       <c r="D46" s="2" t="n"/>
       <c r="E46" s="2" t="n"/>
@@ -2473,7 +2531,9 @@
       <c r="R46" s="2" t="n"/>
       <c r="S46" s="2" t="n"/>
       <c r="T46" s="2" t="n"/>
-      <c r="U46" s="2" t="n"/>
+      <c r="U46" s="3" t="n">
+        <v>0.03643712452920096</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2485,7 +2545,10 @@
         <v>46</v>
       </c>
       <c r="C47" s="4" t="n">
-        <v>0.03672647530049522</v>
+        <v>0.03479350291625863</v>
+      </c>
+      <c r="U47" s="4" t="n">
+        <v>0.03479350291625863</v>
       </c>
     </row>
     <row r="48">
@@ -2498,7 +2561,7 @@
         <v>47</v>
       </c>
       <c r="C48" s="3" t="n">
-        <v>0.03501844229189371</v>
+        <v>0.03317536638179404</v>
       </c>
       <c r="D48" s="2" t="n"/>
       <c r="E48" s="2" t="n"/>
@@ -2517,7 +2580,9 @@
       <c r="R48" s="2" t="n"/>
       <c r="S48" s="2" t="n"/>
       <c r="T48" s="2" t="n"/>
-      <c r="U48" s="2" t="n"/>
+      <c r="U48" s="3" t="n">
+        <v>0.03317536638179404</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2529,7 +2594,10 @@
         <v>48</v>
       </c>
       <c r="C49" s="4" t="n">
-        <v>0.03333774075087094</v>
+        <v>0.03158312281661457</v>
+      </c>
+      <c r="U49" s="4" t="n">
+        <v>0.03158312281661457</v>
       </c>
     </row>
     <row r="50">
@@ -2542,7 +2610,7 @@
         <v>49</v>
       </c>
       <c r="C50" s="3" t="n">
-        <v>0.03168482259036684</v>
+        <v>0.03001720034876858</v>
       </c>
       <c r="D50" s="2" t="n"/>
       <c r="E50" s="2" t="n"/>
@@ -2561,32 +2629,37 @@
       <c r="R50" s="2" t="n"/>
       <c r="S50" s="2" t="n"/>
       <c r="T50" s="2" t="n"/>
-      <c r="U50" s="2" t="n"/>
+      <c r="U50" s="3" t="n">
+        <v>0.03001720034876858</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Бэндер</t>
+          <t>OlgaaGeorgieva</t>
         </is>
       </c>
       <c r="B51" t="n">
         <v>50</v>
       </c>
       <c r="C51" s="4" t="n">
-        <v>0.03006016291212127</v>
+        <v>0.0284780490746412</v>
+      </c>
+      <c r="U51" s="4" t="n">
+        <v>0.0284780490746412</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>OlgaaGeorgieva</t>
+          <t>Бэндер</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
         <v>51</v>
       </c>
       <c r="C52" s="3" t="n">
-        <v>0.02846426206058033</v>
+        <v>0.02696614300476031</v>
       </c>
       <c r="D52" s="2" t="n"/>
       <c r="E52" s="2" t="n"/>
@@ -2605,7 +2678,9 @@
       <c r="R52" s="2" t="n"/>
       <c r="S52" s="2" t="n"/>
       <c r="T52" s="2" t="n"/>
-      <c r="U52" s="2" t="n"/>
+      <c r="U52" s="3" t="n">
+        <v>0.02696614300476031</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2617,7 +2692,10 @@
         <v>52</v>
       </c>
       <c r="C53" s="4" t="n">
-        <v>0.02689764794092131</v>
+        <v>0.02548198225982019</v>
+      </c>
+      <c r="U53" s="4" t="n">
+        <v>0.02548198225982019</v>
       </c>
     </row>
     <row r="54">
@@ -2630,7 +2708,7 @@
         <v>53</v>
       </c>
       <c r="C54" s="3" t="n">
-        <v>0.02536087864654337</v>
+        <v>0.02402609555988319</v>
       </c>
       <c r="D54" s="2" t="n"/>
       <c r="E54" s="2" t="n"/>
@@ -2649,7 +2727,9 @@
       <c r="R54" s="2" t="n"/>
       <c r="S54" s="2" t="n"/>
       <c r="T54" s="2" t="n"/>
-      <c r="U54" s="2" t="n"/>
+      <c r="U54" s="3" t="n">
+        <v>0.02402609555988319</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2661,7 +2741,10 @@
         <v>54</v>
       </c>
       <c r="C55" s="4" t="n">
-        <v>0.02385454545126794</v>
+        <v>0.02259904305909594</v>
+      </c>
+      <c r="U55" s="4" t="n">
+        <v>0.02259904305909594</v>
       </c>
     </row>
     <row r="56">
@@ -2674,7 +2757,7 @@
         <v>55</v>
       </c>
       <c r="C56" s="3" t="n">
-        <v>0.0223792762340482</v>
+        <v>0.02120141959015093</v>
       </c>
       <c r="D56" s="2" t="n"/>
       <c r="E56" s="2" t="n"/>
@@ -2693,7 +2776,9 @@
       <c r="R56" s="2" t="n"/>
       <c r="S56" s="2" t="n"/>
       <c r="T56" s="2" t="n"/>
-      <c r="U56" s="2" t="n"/>
+      <c r="U56" s="3" t="n">
+        <v>0.02120141959015093</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2705,7 +2790,10 @@
         <v>56</v>
       </c>
       <c r="C57" s="4" t="n">
-        <v>0.02093573942006211</v>
+        <v>0.01983385839795358</v>
+      </c>
+      <c r="U57" s="4" t="n">
+        <v>0.01983385839795358</v>
       </c>
     </row>
     <row r="58">
@@ -2718,7 +2806,7 @@
         <v>57</v>
       </c>
       <c r="C58" s="3" t="n">
-        <v>0.01952464854284687</v>
+        <v>0.0184970354616444</v>
       </c>
       <c r="D58" s="2" t="n"/>
       <c r="E58" s="2" t="n"/>
@@ -2737,7 +2825,9 @@
       <c r="R58" s="2" t="n"/>
       <c r="S58" s="2" t="n"/>
       <c r="T58" s="2" t="n"/>
-      <c r="U58" s="2" t="n"/>
+      <c r="U58" s="3" t="n">
+        <v>0.0184970354616444</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2749,7 +2839,10 @@
         <v>58</v>
       </c>
       <c r="C59" s="4" t="n">
-        <v>0.01814676755929403</v>
+        <v>0.0171916745298575</v>
+      </c>
+      <c r="U59" s="4" t="n">
+        <v>0.0171916745298575</v>
       </c>
     </row>
     <row r="60">
@@ -2762,7 +2855,7 @@
         <v>59</v>
       </c>
       <c r="C60" s="3" t="n">
-        <v>0.01680291708523153</v>
+        <v>0.01591855302811408</v>
       </c>
       <c r="D60" s="2" t="n"/>
       <c r="E60" s="2" t="n"/>
@@ -2781,7 +2874,9 @@
       <c r="R60" s="2" t="n"/>
       <c r="S60" s="2" t="n"/>
       <c r="T60" s="2" t="n"/>
-      <c r="U60" s="2" t="n"/>
+      <c r="U60" s="3" t="n">
+        <v>0.01591855302811408</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2793,7 +2888,10 @@
         <v>60</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>0.01549398176739642</v>
+        <v>0.01467850904279661</v>
+      </c>
+      <c r="U61" s="4" t="n">
+        <v>0.01467850904279661</v>
       </c>
     </row>
     <row r="62">
@@ -2806,7 +2904,7 @@
         <v>61</v>
       </c>
       <c r="C62" s="3" t="n">
-        <v>0.01422091907287109</v>
+        <v>0.01347244964798314</v>
       </c>
       <c r="D62" s="2" t="n"/>
       <c r="E62" s="2" t="n"/>
@@ -2825,7 +2923,9 @@
       <c r="R62" s="2" t="n"/>
       <c r="S62" s="2" t="n"/>
       <c r="T62" s="2" t="n"/>
-      <c r="U62" s="2" t="n"/>
+      <c r="U62" s="3" t="n">
+        <v>0.01347244964798314</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2837,7 +2937,10 @@
         <v>62</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>0.01298476986703021</v>
+        <v>0.0123013609266602</v>
+      </c>
+      <c r="U63" s="4" t="n">
+        <v>0.0123013609266602</v>
       </c>
     </row>
     <row r="64">
@@ -2850,7 +2953,7 @@
         <v>63</v>
       </c>
       <c r="C64" s="3" t="n">
-        <v>0.01178667127718997</v>
+        <v>0.01116632015733787</v>
       </c>
       <c r="D64" s="2" t="n"/>
       <c r="E64" s="2" t="n"/>
@@ -2869,7 +2972,9 @@
       <c r="R64" s="2" t="n"/>
       <c r="S64" s="2" t="n"/>
       <c r="T64" s="2" t="n"/>
-      <c r="U64" s="2" t="n"/>
+      <c r="U64" s="3" t="n">
+        <v>0.01116632015733787</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2881,7 +2986,10 @@
         <v>64</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>0.01062787251936665</v>
+        <v>0.01006851080782104</v>
+      </c>
+      <c r="U65" s="4" t="n">
+        <v>0.01006851080782104</v>
       </c>
     </row>
     <row r="66">
@@ -2894,7 +3002,7 @@
         <v>65</v>
       </c>
       <c r="C66" s="3" t="n">
-        <v>0.009509754628496918</v>
+        <v>0.00900924122699708</v>
       </c>
       <c r="D66" s="2" t="n"/>
       <c r="E66" s="2" t="n"/>
@@ -2913,32 +3021,37 @@
       <c r="R66" s="2" t="n"/>
       <c r="S66" s="2" t="n"/>
       <c r="T66" s="2" t="n"/>
-      <c r="U66" s="2" t="n"/>
+      <c r="U66" s="3" t="n">
+        <v>0.00900924122699708</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Fara</t>
+          <t>Tim19</t>
         </is>
       </c>
       <c r="B67" t="n">
         <v>66</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>0.008433855425357134</v>
+        <v>0.007989968297706759</v>
+      </c>
+      <c r="U67" s="4" t="n">
+        <v>0.007989968297706759</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Tim19</t>
+          <t>Fara</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
         <v>67</v>
       </c>
       <c r="C68" s="3" t="n">
-        <v>0.007401901656540216</v>
+        <v>0.007012327885143364</v>
       </c>
       <c r="D68" s="2" t="n"/>
       <c r="E68" s="2" t="n"/>
@@ -2957,32 +3070,37 @@
       <c r="R68" s="2" t="n"/>
       <c r="S68" s="2" t="n"/>
       <c r="T68" s="2" t="n"/>
-      <c r="U68" s="2" t="n"/>
+      <c r="U68" s="3" t="n">
+        <v>0.007012327885143364</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>twewefe</t>
+          <t>edimerfi</t>
         </is>
       </c>
       <c r="B69" t="n">
         <v>68</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>0.006415851198896431</v>
+        <v>0.006078174820007144</v>
+      </c>
+      <c r="U69" s="4" t="n">
+        <v>0.006078174820007144</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>frida_hk</t>
+          <t>Shuricspinoza</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
         <v>69</v>
       </c>
       <c r="C70" s="3" t="n">
-        <v>0.005477949787653368</v>
+        <v>0.00518963664093477</v>
       </c>
       <c r="D70" s="2" t="n"/>
       <c r="E70" s="2" t="n"/>
@@ -3001,32 +3119,37 @@
       <c r="R70" s="2" t="n"/>
       <c r="S70" s="2" t="n"/>
       <c r="T70" s="2" t="n"/>
-      <c r="U70" s="2" t="n"/>
+      <c r="U70" s="3" t="n">
+        <v>0.00518963664093477</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Shuricspinoza</t>
+          <t>katerina_boc</t>
         </is>
       </c>
       <c r="B71" t="n">
         <v>70</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>0.004590809412561903</v>
+        <v>0.004349187864532329</v>
+      </c>
+      <c r="U71" s="4" t="n">
+        <v>0.004349187864532329</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>nsa</t>
+          <t>twewefe</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
         <v>71</v>
       </c>
       <c r="C72" s="3" t="n">
-        <v>0.003757520364015158</v>
+        <v>0.00355975613433015</v>
       </c>
       <c r="D72" s="2" t="n"/>
       <c r="E72" s="2" t="n"/>
@@ -3045,32 +3168,37 @@
       <c r="R72" s="2" t="n"/>
       <c r="S72" s="2" t="n"/>
       <c r="T72" s="2" t="n"/>
-      <c r="U72" s="2" t="n"/>
+      <c r="U72" s="3" t="n">
+        <v>0.00355975613433015</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>katerina_boc</t>
+          <t>Schwepp1S</t>
         </is>
       </c>
       <c r="B73" t="n">
         <v>72</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0.002981818181408492</v>
+        <v>0.002824880382386993</v>
+      </c>
+      <c r="U73" s="4" t="n">
+        <v>0.002824880382386993</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>rus210385</t>
+          <t>alinaadmv</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
         <v>73</v>
       </c>
       <c r="C74" s="3" t="n">
-        <v>0.002268345944911754</v>
+        <v>0.002148959316232187</v>
       </c>
       <c r="D74" s="2" t="n"/>
       <c r="E74" s="2" t="n"/>
@@ -3089,32 +3217,37 @@
       <c r="R74" s="2" t="n"/>
       <c r="S74" s="2" t="n"/>
       <c r="T74" s="2" t="n"/>
-      <c r="U74" s="2" t="n"/>
+      <c r="U74" s="3" t="n">
+        <v>0.002148959316232187</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Schwepp1S</t>
+          <t>rus210385</t>
         </is>
       </c>
       <c r="B75" t="n">
         <v>74</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>0.001623096233378776</v>
+        <v>0.001537670115832525</v>
+      </c>
+      <c r="U75" s="4" t="n">
+        <v>0.001537670115832525</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>DanilaOdinokov</t>
+          <t>frida_hk</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
         <v>75</v>
       </c>
       <c r="C76" s="3" t="n">
-        <v>0.001054231928169642</v>
+        <v>0.0009987460372133448</v>
       </c>
       <c r="D76" s="2" t="n"/>
       <c r="E76" s="2" t="n"/>
@@ -3133,25 +3266,30 @@
       <c r="R76" s="2" t="n"/>
       <c r="S76" s="2" t="n"/>
       <c r="T76" s="2" t="n"/>
-      <c r="U76" s="2" t="n"/>
+      <c r="U76" s="3" t="n">
+        <v>0.0009987460372133448</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>alinaadmv</t>
+          <t>nsa</t>
         </is>
       </c>
       <c r="B77" t="n">
         <v>76</v>
       </c>
       <c r="C77" s="4" t="n">
-        <v>0.0005738511765702378</v>
+        <v>0.0005436484830665411</v>
+      </c>
+      <c r="U77" s="4" t="n">
+        <v>0.0005436484830665411</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>edimerfi</t>
+          <t>DanilaOdinokov</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">

</xml_diff>

<commit_message>
NEW CALENDAR + added tournament metadata, bounty aggression index, attendance per player per type
</commit_message>
<xml_diff>
--- a/data/playoff_odds.xlsx
+++ b/data/playoff_odds.xlsx
@@ -591,7 +591,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Noize MC</t>
+          <t>Драйв</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -601,49 +601,49 @@
         <v>0.25</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.04175</v>
+        <v>0.03325</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.0335</v>
+        <v>0.02625</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.024</v>
+        <v>0.02725</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>0.02525</v>
+        <v>0.02325</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>0.0235</v>
+        <v>0.02225</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.0215</v>
+        <v>0.02225</v>
       </c>
       <c r="J2" s="3" t="n">
+        <v>0.0225</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>0.0155</v>
+      </c>
+      <c r="L2" s="3" t="n">
         <v>0.016</v>
       </c>
-      <c r="K2" s="3" t="n">
-        <v>0.01425</v>
-      </c>
-      <c r="L2" s="3" t="n">
-        <v>0.01675</v>
-      </c>
       <c r="M2" s="3" t="n">
-        <v>0.00975</v>
+        <v>0.01225</v>
       </c>
       <c r="N2" s="3" t="n">
+        <v>0.01275</v>
+      </c>
+      <c r="O2" s="3" t="n">
         <v>0.00725</v>
       </c>
-      <c r="O2" s="3" t="n">
-        <v>0.008500000000000001</v>
-      </c>
       <c r="P2" s="3" t="n">
-        <v>0.00375</v>
+        <v>0.0035</v>
       </c>
       <c r="Q2" s="3" t="n">
-        <v>0.002</v>
+        <v>0.00225</v>
       </c>
       <c r="R2" s="3" t="n">
-        <v>0.001</v>
+        <v>0.00225</v>
       </c>
       <c r="S2" s="3" t="n">
         <v>0.00075</v>
@@ -656,7 +656,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Гризли</t>
+          <t>long_2203</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -666,58 +666,64 @@
         <v>0.25</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>0.03825</v>
+        <v>0.02525</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0.027</v>
+        <v>0.02</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>0.03025</v>
+        <v>0.0205</v>
       </c>
       <c r="G3" s="4" t="n">
         <v>0.0235</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>0.02425</v>
+        <v>0.0245</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>0.02</v>
+        <v>0.0225</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>0.01875</v>
+        <v>0.017</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>0.01475</v>
+        <v>0.02625</v>
       </c>
       <c r="L3" s="4" t="n">
-        <v>0.012</v>
+        <v>0.01725</v>
       </c>
       <c r="M3" s="4" t="n">
-        <v>0.01175</v>
+        <v>0.015</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>0.0115</v>
+        <v>0.01375</v>
       </c>
       <c r="O3" s="4" t="n">
-        <v>0.0075</v>
+        <v>0.01</v>
       </c>
       <c r="P3" s="4" t="n">
-        <v>0.005</v>
+        <v>0.00775</v>
       </c>
       <c r="Q3" s="4" t="n">
-        <v>0.00325</v>
+        <v>0.004</v>
       </c>
       <c r="R3" s="4" t="n">
-        <v>0.00175</v>
+        <v>0.00075</v>
+      </c>
+      <c r="S3" s="4" t="n">
+        <v>0.0015</v>
       </c>
       <c r="T3" s="4" t="n">
-        <v>0.0005</v>
+        <v>0.00025</v>
+      </c>
+      <c r="U3" s="4" t="n">
+        <v>0.00025</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>кинчоч</t>
+          <t>Пассажир</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -727,55 +733,55 @@
         <v>0.25</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.01975</v>
+        <v>0.01875</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.0205</v>
+        <v>0.0245</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.02325</v>
+        <v>0.0225</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0.018</v>
+        <v>0.021</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>0.02175</v>
       </c>
       <c r="I4" s="3" t="n">
+        <v>0.02075</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0.0215</v>
+      </c>
+      <c r="K4" s="3" t="n">
         <v>0.022</v>
       </c>
-      <c r="J4" s="3" t="n">
-        <v>0.02175</v>
-      </c>
-      <c r="K4" s="3" t="n">
-        <v>0.02</v>
-      </c>
       <c r="L4" s="3" t="n">
-        <v>0.02175</v>
+        <v>0.01975</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>0.0175</v>
+        <v>0.016</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>0.01475</v>
+        <v>0.016</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>0.011</v>
+        <v>0.0095</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>0.00725</v>
+        <v>0.00775</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>0.00475</v>
+        <v>0.00325</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="S4" s="3" t="n">
-        <v>0.00125</v>
+        <v>0.00075</v>
       </c>
       <c r="T4" s="3" t="n">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="U4" s="3" t="n">
         <v>0.00025</v>
@@ -784,7 +790,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>G_rant_999</t>
+          <t>dolMy</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -794,13 +800,13 @@
         <v>0.25</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>0.01325</v>
+        <v>0.017</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0.018</v>
+        <v>0.0165</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>0.02025</v>
+        <v>0.01775</v>
       </c>
       <c r="G5" s="4" t="n">
         <v>0.0195</v>
@@ -809,43 +815,43 @@
         <v>0.01975</v>
       </c>
       <c r="I5" s="4" t="n">
+        <v>0.0185</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>0.02325</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>0.0185</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="N5" s="4" t="n">
         <v>0.0225</v>
       </c>
-      <c r="J5" s="4" t="n">
-        <v>0.0185</v>
-      </c>
-      <c r="K5" s="4" t="n">
-        <v>0.0205</v>
-      </c>
-      <c r="L5" s="4" t="n">
-        <v>0.019</v>
-      </c>
-      <c r="M5" s="4" t="n">
-        <v>0.01975</v>
-      </c>
-      <c r="N5" s="4" t="n">
-        <v>0.01825</v>
-      </c>
       <c r="O5" s="4" t="n">
-        <v>0.016</v>
+        <v>0.01525</v>
       </c>
       <c r="P5" s="4" t="n">
-        <v>0.01225</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="Q5" s="4" t="n">
-        <v>0.0065</v>
+        <v>0.005</v>
       </c>
       <c r="R5" s="4" t="n">
         <v>0.00325</v>
       </c>
       <c r="S5" s="4" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="T5" s="4" t="n">
         <v>0.00125</v>
       </c>
-      <c r="T5" s="4" t="n">
-        <v>0.0005</v>
-      </c>
       <c r="U5" s="4" t="n">
-        <v>0.001</v>
+        <v>0.0015</v>
       </c>
     </row>
     <row r="6">
@@ -861,131 +867,128 @@
         <v>0.24975</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0.01125</v>
+        <v>0.01275</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.013</v>
+        <v>0.016</v>
       </c>
       <c r="F6" s="3" t="n">
+        <v>0.01825</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0.01775</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>0.0225</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>0.0195</v>
+      </c>
+      <c r="J6" s="3" t="n">
         <v>0.0175</v>
       </c>
-      <c r="G6" s="3" t="n">
-        <v>0.01525</v>
-      </c>
-      <c r="H6" s="3" t="n">
-        <v>0.02025</v>
-      </c>
-      <c r="I6" s="3" t="n">
+      <c r="K6" s="3" t="n">
+        <v>0.01775</v>
+      </c>
+      <c r="L6" s="3" t="n">
         <v>0.01975</v>
       </c>
-      <c r="J6" s="3" t="n">
-        <v>0.01975</v>
-      </c>
-      <c r="K6" s="3" t="n">
-        <v>0.02025</v>
-      </c>
-      <c r="L6" s="3" t="n">
-        <v>0.02</v>
-      </c>
       <c r="M6" s="3" t="n">
-        <v>0.024</v>
+        <v>0.02275</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>0.01925</v>
+        <v>0.02125</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>0.016</v>
+        <v>0.0165</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>0.015</v>
+        <v>0.01375</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>0.008</v>
+        <v>0.0065</v>
       </c>
       <c r="R6" s="3" t="n">
-        <v>0.0055</v>
+        <v>0.00325</v>
       </c>
       <c r="S6" s="3" t="n">
         <v>0.0025</v>
       </c>
       <c r="T6" s="3" t="n">
-        <v>0.001</v>
+        <v>0.00125</v>
       </c>
       <c r="U6" s="3" t="n">
-        <v>0.0015</v>
+        <v>0.00025</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Сокол</t>
+          <t>Гризли</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>6</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>0.2495</v>
+        <v>0.24975</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>0.01325</v>
+        <v>0.0355</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0.01375</v>
+        <v>0.03225</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>0.02075</v>
+        <v>0.0295</v>
       </c>
       <c r="G7" s="4" t="n">
+        <v>0.0225</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>0.0215</v>
+      </c>
+      <c r="I7" s="4" t="n">
         <v>0.018</v>
       </c>
-      <c r="H7" s="4" t="n">
-        <v>0.0165</v>
-      </c>
-      <c r="I7" s="4" t="n">
+      <c r="J7" s="4" t="n">
         <v>0.01675</v>
       </c>
-      <c r="J7" s="4" t="n">
-        <v>0.02075</v>
-      </c>
       <c r="K7" s="4" t="n">
-        <v>0.0195</v>
+        <v>0.015</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>0.01875</v>
+        <v>0.017</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>0.02025</v>
+        <v>0.01475</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>0.02025</v>
+        <v>0.0105</v>
       </c>
       <c r="O7" s="4" t="n">
-        <v>0.01575</v>
+        <v>0.0075</v>
       </c>
       <c r="P7" s="4" t="n">
-        <v>0.01375</v>
+        <v>0.003</v>
       </c>
       <c r="Q7" s="4" t="n">
-        <v>0.0095</v>
+        <v>0.00375</v>
       </c>
       <c r="R7" s="4" t="n">
-        <v>0.0055</v>
+        <v>0.0015</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.00225</v>
+        <v>0.0005</v>
       </c>
       <c r="T7" s="4" t="n">
-        <v>0.00325</v>
-      </c>
-      <c r="U7" s="4" t="n">
-        <v>0.001</v>
+        <v>0.00025</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Драйв</t>
+          <t>Yanchik_250</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -995,62 +998,64 @@
         <v>0.2495</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0.03175</v>
+        <v>0.01025</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.0325</v>
+        <v>0.01375</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0.021</v>
+        <v>0.0155</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>0.02875</v>
+        <v>0.017</v>
       </c>
       <c r="H8" s="3" t="n">
+        <v>0.01875</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>0.0205</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>0.01875</v>
+      </c>
+      <c r="K8" s="3" t="n">
         <v>0.02275</v>
       </c>
-      <c r="I8" s="3" t="n">
-        <v>0.02175</v>
-      </c>
-      <c r="J8" s="3" t="n">
-        <v>0.0175</v>
-      </c>
-      <c r="K8" s="3" t="n">
-        <v>0.0175</v>
-      </c>
       <c r="L8" s="3" t="n">
-        <v>0.016</v>
+        <v>0.01875</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>0.0135</v>
+        <v>0.023</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>0.0105</v>
+        <v>0.0255</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>0.00475</v>
+        <v>0.01775</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>0.00575</v>
+        <v>0.01175</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>0.00275</v>
+        <v>0.00825</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>0.0015</v>
+        <v>0.00175</v>
       </c>
       <c r="S8" s="3" t="n">
-        <v>0.001</v>
+        <v>0.00175</v>
       </c>
       <c r="T8" s="3" t="n">
-        <v>0.00025</v>
-      </c>
-      <c r="U8" s="2" t="n"/>
+        <v>0.00325</v>
+      </c>
+      <c r="U8" s="3" t="n">
+        <v>0.0005</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>long_2203</t>
+          <t>Noize MC</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1060,122 +1065,116 @@
         <v>0.2495</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>0.02275</v>
+        <v>0.0405</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.02875</v>
+        <v>0.0335</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>0.02375</v>
+        <v>0.023</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.0235</v>
+        <v>0.0275</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>0.02075</v>
+        <v>0.01825</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>0.02025</v>
+        <v>0.02</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>0.022</v>
+        <v>0.018</v>
       </c>
       <c r="K9" s="4" t="n">
-        <v>0.01775</v>
+        <v>0.01475</v>
       </c>
       <c r="L9" s="4" t="n">
-        <v>0.0165</v>
+        <v>0.017</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>0.01675</v>
+        <v>0.012</v>
       </c>
       <c r="N9" s="4" t="n">
-        <v>0.012</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="O9" s="4" t="n">
-        <v>0.0095</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="P9" s="4" t="n">
-        <v>0.0065</v>
+        <v>0.0045</v>
       </c>
       <c r="Q9" s="4" t="n">
-        <v>0.00425</v>
+        <v>0.00175</v>
       </c>
       <c r="R9" s="4" t="n">
-        <v>0.0025</v>
+        <v>0.00025</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.0015</v>
-      </c>
-      <c r="T9" s="4" t="n">
-        <v>0.00025</v>
-      </c>
-      <c r="U9" s="4" t="n">
-        <v>0.00025</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Пассажир</t>
+          <t>G_rant_999</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
         <v>9</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.2495</v>
+        <v>0.24925</v>
       </c>
       <c r="D10" s="3" t="n">
+        <v>0.01175</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>0.0155</v>
+      </c>
+      <c r="F10" s="3" t="n">
         <v>0.01825</v>
       </c>
-      <c r="E10" s="3" t="n">
+      <c r="G10" s="3" t="n">
+        <v>0.01925</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>0.02225</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>0.0195</v>
+      </c>
+      <c r="K10" s="3" t="n">
         <v>0.01875</v>
       </c>
-      <c r="F10" s="3" t="n">
-        <v>0.02225</v>
-      </c>
-      <c r="G10" s="3" t="n">
-        <v>0.02375</v>
-      </c>
-      <c r="H10" s="3" t="n">
-        <v>0.022</v>
-      </c>
-      <c r="I10" s="3" t="n">
-        <v>0.0225</v>
-      </c>
-      <c r="J10" s="3" t="n">
-        <v>0.0215</v>
-      </c>
-      <c r="K10" s="3" t="n">
-        <v>0.02175</v>
-      </c>
       <c r="L10" s="3" t="n">
-        <v>0.01725</v>
+        <v>0.02325</v>
       </c>
       <c r="M10" s="3" t="n">
+        <v>0.02125</v>
+      </c>
+      <c r="N10" s="3" t="n">
         <v>0.0155</v>
       </c>
-      <c r="N10" s="3" t="n">
-        <v>0.016</v>
-      </c>
       <c r="O10" s="3" t="n">
-        <v>0.0125</v>
+        <v>0.01925</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>0.00775</v>
+        <v>0.01275</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>0.0045</v>
+        <v>0.006</v>
       </c>
       <c r="R10" s="3" t="n">
-        <v>0.0015</v>
+        <v>0.00375</v>
       </c>
       <c r="S10" s="3" t="n">
         <v>0.00175</v>
       </c>
       <c r="T10" s="3" t="n">
-        <v>0.001</v>
+        <v>0.0015</v>
       </c>
       <c r="U10" s="3" t="n">
         <v>0.001</v>
@@ -1184,74 +1183,74 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yanchik_250</t>
+          <t>кинчоч</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>10</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>0.2495</v>
+        <v>0.24925</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>0.0115</v>
+        <v>0.02225</v>
       </c>
       <c r="E11" s="4" t="n">
+        <v>0.02225</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>0.02275</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>0.02125</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>0.02375</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>0.0195</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>0.02125</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>0.0185</v>
+      </c>
+      <c r="M11" s="4" t="n">
         <v>0.0155</v>
       </c>
-      <c r="F11" s="4" t="n">
-        <v>0.0145</v>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>0.01425</v>
-      </c>
-      <c r="H11" s="4" t="n">
-        <v>0.01825</v>
-      </c>
-      <c r="I11" s="4" t="n">
-        <v>0.02025</v>
-      </c>
-      <c r="J11" s="4" t="n">
-        <v>0.02225</v>
-      </c>
-      <c r="K11" s="4" t="n">
-        <v>0.021</v>
-      </c>
-      <c r="L11" s="4" t="n">
-        <v>0.0215</v>
-      </c>
-      <c r="M11" s="4" t="n">
-        <v>0.0205</v>
-      </c>
       <c r="N11" s="4" t="n">
-        <v>0.017</v>
+        <v>0.01625</v>
       </c>
       <c r="O11" s="4" t="n">
-        <v>0.01675</v>
+        <v>0.011</v>
       </c>
       <c r="P11" s="4" t="n">
-        <v>0.01325</v>
+        <v>0.00625</v>
       </c>
       <c r="Q11" s="4" t="n">
-        <v>0.008750000000000001</v>
+        <v>0.00275</v>
       </c>
       <c r="R11" s="4" t="n">
-        <v>0.00625</v>
+        <v>0.002</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.00375</v>
+        <v>0.001</v>
       </c>
       <c r="T11" s="4" t="n">
-        <v>0.0025</v>
+        <v>0.00075</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.00175</v>
+        <v>0.00025</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>dolMy</t>
+          <t>Сокол</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1261,58 +1260,58 @@
         <v>0.249</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0.01325</v>
+        <v>0.01175</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.01475</v>
+        <v>0.0145</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.014</v>
+        <v>0.01775</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0.0205</v>
+        <v>0.01725</v>
       </c>
       <c r="H12" s="3" t="n">
+        <v>0.0185</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>0.02025</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>0.02175</v>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>0.02125</v>
+      </c>
+      <c r="L12" s="3" t="n">
+        <v>0.02275</v>
+      </c>
+      <c r="M12" s="3" t="n">
         <v>0.0215</v>
       </c>
-      <c r="I12" s="3" t="n">
-        <v>0.02075</v>
-      </c>
-      <c r="J12" s="3" t="n">
-        <v>0.02075</v>
-      </c>
-      <c r="K12" s="3" t="n">
-        <v>0.02075</v>
-      </c>
-      <c r="L12" s="3" t="n">
-        <v>0.0235</v>
-      </c>
-      <c r="M12" s="3" t="n">
-        <v>0.02025</v>
-      </c>
       <c r="N12" s="3" t="n">
-        <v>0.01775</v>
+        <v>0.01575</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.01775</v>
+        <v>0.0185</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>0.00775</v>
+        <v>0.01175</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>0.00475</v>
+        <v>0.00675</v>
       </c>
       <c r="R12" s="3" t="n">
-        <v>0.006</v>
+        <v>0.0055</v>
       </c>
       <c r="S12" s="3" t="n">
-        <v>0.0025</v>
+        <v>0.002</v>
       </c>
       <c r="T12" s="3" t="n">
-        <v>0.001</v>
+        <v>0.00075</v>
       </c>
       <c r="U12" s="3" t="n">
-        <v>0.0015</v>
+        <v>0.00075</v>
       </c>
     </row>
     <row r="13">
@@ -1325,61 +1324,61 @@
         <v>12</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>0.2485</v>
+        <v>0.24825</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>0.0145</v>
+        <v>0.011</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.01325</v>
+        <v>0.01425</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0.01675</v>
+        <v>0.01575</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.01725</v>
+        <v>0.0185</v>
       </c>
       <c r="H13" s="4" t="n">
         <v>0.01575</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>0.0155</v>
+        <v>0.01875</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>0.021</v>
+        <v>0.025</v>
       </c>
       <c r="K13" s="4" t="n">
-        <v>0.02275</v>
+        <v>0.022</v>
       </c>
       <c r="L13" s="4" t="n">
-        <v>0.02225</v>
+        <v>0.0195</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>0.01825</v>
+        <v>0.023</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>0.0215</v>
+        <v>0.01925</v>
       </c>
       <c r="O13" s="4" t="n">
-        <v>0.0165</v>
+        <v>0.01725</v>
       </c>
       <c r="P13" s="4" t="n">
-        <v>0.015</v>
+        <v>0.01</v>
       </c>
       <c r="Q13" s="4" t="n">
-        <v>0.00625</v>
+        <v>0.008</v>
       </c>
       <c r="R13" s="4" t="n">
-        <v>0.00525</v>
+        <v>0.00575</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.00175</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.001</v>
+        <v>0.00075</v>
       </c>
     </row>
     <row r="14">
@@ -1392,61 +1391,57 @@
         <v>13</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>0.21525</v>
-      </c>
-      <c r="D14" s="3" t="n">
-        <v>0.00025</v>
-      </c>
-      <c r="E14" s="3" t="n">
-        <v>0.00025</v>
-      </c>
+        <v>0.20925</v>
+      </c>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
       <c r="F14" s="3" t="n">
-        <v>0.00025</v>
+        <v>0.00075</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>0.00075</v>
+        <v>0.0005</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0.00125</v>
+        <v>0.0015</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>0.00175</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0.00275</v>
+        <v>0.00225</v>
       </c>
       <c r="K14" s="3" t="n">
         <v>0.00325</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>0.00675</v>
+        <v>0.00425</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0.00925</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>0.0115</v>
+        <v>0.01</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>0.021</v>
+        <v>0.01825</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>0.028</v>
+        <v>0.02825</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>0.02925</v>
+        <v>0.0285</v>
       </c>
       <c r="R14" s="3" t="n">
-        <v>0.0295</v>
+        <v>0.03225</v>
       </c>
       <c r="S14" s="3" t="n">
-        <v>0.031</v>
+        <v>0.0265</v>
       </c>
       <c r="T14" s="3" t="n">
-        <v>0.019</v>
+        <v>0.02125</v>
       </c>
       <c r="U14" s="3" t="n">
-        <v>0.0195</v>
+        <v>0.02075</v>
       </c>
     </row>
     <row r="15">
@@ -1459,55 +1454,55 @@
         <v>14</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>0.19825</v>
-      </c>
-      <c r="F15" s="4" t="n">
+        <v>0.20075</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="G15" s="4" t="n">
         <v>0.00025</v>
       </c>
-      <c r="G15" s="4" t="n">
-        <v>0.0005</v>
-      </c>
       <c r="H15" s="4" t="n">
-        <v>0.0005</v>
+        <v>0.00125</v>
       </c>
       <c r="I15" s="4" t="n">
-        <v>0.00075</v>
+        <v>0.003</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>0.00225</v>
+        <v>0.0015</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>0.00475</v>
+        <v>0.0015</v>
       </c>
       <c r="L15" s="4" t="n">
-        <v>0.0045</v>
+        <v>0.00275</v>
       </c>
       <c r="M15" s="4" t="n">
         <v>0.0075</v>
       </c>
       <c r="N15" s="4" t="n">
-        <v>0.014</v>
+        <v>0.0095</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>0.01375</v>
+        <v>0.0135</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>0.01475</v>
+        <v>0.0225</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>0.02975</v>
+        <v>0.0235</v>
       </c>
       <c r="R15" s="4" t="n">
         <v>0.03325</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.02525</v>
+        <v>0.031</v>
       </c>
       <c r="T15" s="4" t="n">
-        <v>0.02525</v>
+        <v>0.02575</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.02125</v>
+        <v>0.0235</v>
       </c>
     </row>
     <row r="16">
@@ -1520,121 +1515,114 @@
         <v>15</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>0.19025</v>
+        <v>0.18925</v>
       </c>
       <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
+      <c r="E16" s="3" t="n">
+        <v>0.00025</v>
+      </c>
       <c r="F16" s="3" t="n">
-        <v>0.00025</v>
+        <v>0.0005</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>0.00025</v>
+        <v>0.0005</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>0.00075</v>
+        <v>0.001</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>0.00175</v>
+        <v>0.0005</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>0.00225</v>
+        <v>0.00325</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>0.002</v>
+        <v>0.00375</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0.0055</v>
+        <v>0.0045</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0.0105</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>0.013</v>
+        <v>0.012</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>0.019</v>
+        <v>0.0205</v>
       </c>
       <c r="Q16" s="3" t="n">
-        <v>0.024</v>
+        <v>0.026</v>
       </c>
       <c r="R16" s="3" t="n">
-        <v>0.02625</v>
+        <v>0.0285</v>
       </c>
       <c r="S16" s="3" t="n">
-        <v>0.02775</v>
+        <v>0.02525</v>
       </c>
       <c r="T16" s="3" t="n">
-        <v>0.02975</v>
+        <v>0.0255</v>
       </c>
       <c r="U16" s="3" t="n">
-        <v>0.02675</v>
+        <v>0.02725</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Lock</t>
+          <t>ksuhony</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>16</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>0.18975</v>
-      </c>
-      <c r="E17" s="4" t="n">
+        <v>0.1725</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="H17" s="4" t="n">
         <v>0.0005</v>
       </c>
-      <c r="F17" s="4" t="n">
-        <v>0.00025</v>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="H17" s="4" t="n">
-        <v>0.00025</v>
-      </c>
       <c r="I17" s="4" t="n">
-        <v>0.00025</v>
-      </c>
-      <c r="J17" s="4" t="n">
         <v>0.00075</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>0.00325</v>
+        <v>0.00075</v>
       </c>
       <c r="L17" s="4" t="n">
-        <v>0.00425</v>
+        <v>0.002</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>0.00675</v>
+        <v>0.00225</v>
       </c>
       <c r="N17" s="4" t="n">
-        <v>0.00675</v>
+        <v>0.0055</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>0.0145</v>
+        <v>0.00925</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>0.01925</v>
+        <v>0.014</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>0.02725</v>
+        <v>0.02225</v>
       </c>
       <c r="R17" s="4" t="n">
-        <v>0.02575</v>
+        <v>0.027</v>
       </c>
       <c r="S17" s="4" t="n">
         <v>0.02625</v>
       </c>
       <c r="T17" s="4" t="n">
-        <v>0.0275</v>
+        <v>0.03175</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.02575</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="18">
@@ -1647,188 +1635,176 @@
         <v>17</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>0.178</v>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>0.00025</v>
-      </c>
+        <v>0.1705</v>
+      </c>
+      <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="n"/>
-      <c r="F18" s="3" t="n">
-        <v>0.00025</v>
-      </c>
+      <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="n"/>
       <c r="H18" s="3" t="n">
         <v>0.00025</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>0.00075</v>
+        <v>0.0005</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>0.00125</v>
+        <v>0.0005</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>0.00275</v>
+        <v>0.0015</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>0.00225</v>
+        <v>0.00175</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>0.0035</v>
+        <v>0.004</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>0.008</v>
+        <v>0.00525</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>0.01</v>
+        <v>0.01325</v>
       </c>
       <c r="P18" s="3" t="n">
-        <v>0.0165</v>
+        <v>0.019</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>0.021</v>
+        <v>0.02</v>
       </c>
       <c r="R18" s="3" t="n">
-        <v>0.02925</v>
+        <v>0.02425</v>
       </c>
       <c r="S18" s="3" t="n">
-        <v>0.02725</v>
+        <v>0.028</v>
       </c>
       <c r="T18" s="3" t="n">
-        <v>0.02875</v>
+        <v>0.0275</v>
       </c>
       <c r="U18" s="3" t="n">
-        <v>0.026</v>
+        <v>0.02475</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>ksuhony</t>
+          <t>Lock</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
         <v>18</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.1685</v>
+        <v>0.16175</v>
       </c>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
-      <c r="F19" s="6" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="G19" s="6" t="n">
-        <v>0.00025</v>
-      </c>
+      <c r="F19" s="5" t="n"/>
+      <c r="G19" s="5" t="n"/>
       <c r="H19" s="5" t="n"/>
       <c r="I19" s="6" t="n">
-        <v>0.00075</v>
-      </c>
-      <c r="J19" s="6" t="n">
-        <v>0.00075</v>
-      </c>
+        <v>0.00025</v>
+      </c>
+      <c r="J19" s="5" t="n"/>
       <c r="K19" s="6" t="n">
         <v>0.0015</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>0.00175</v>
+        <v>0.00225</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>0.0055</v>
+        <v>0.00325</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>0.00525</v>
+        <v>0.005</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>0.01</v>
+        <v>0.008750000000000001</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>0.015</v>
+        <v>0.0155</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>0.01925</v>
+        <v>0.02475</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>0.01775</v>
+        <v>0.022</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>0.0285</v>
+        <v>0.0245</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>0.02875</v>
+        <v>0.02675</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>0.033</v>
+        <v>0.02725</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Rabie</t>
+          <t>gvrdkn</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
         <v>19</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>0.1495</v>
+        <v>0.1485</v>
       </c>
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="n"/>
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="n"/>
       <c r="H20" s="2" t="n"/>
-      <c r="I20" s="3" t="n">
-        <v>0.00025</v>
-      </c>
+      <c r="I20" s="2" t="n"/>
       <c r="J20" s="3" t="n">
         <v>0.0005</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>0.0015</v>
+        <v>0.0005</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>0.00225</v>
+        <v>0.001</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0.002</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>0.00425</v>
+        <v>0.00225</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>0.008750000000000001</v>
+        <v>0.006</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>0.012</v>
+        <v>0.01075</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>0.017</v>
+        <v>0.018</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>0.02</v>
+        <v>0.01725</v>
       </c>
       <c r="S20" s="3" t="n">
-        <v>0.02475</v>
+        <v>0.0295</v>
       </c>
       <c r="T20" s="3" t="n">
-        <v>0.0275</v>
+        <v>0.02625</v>
       </c>
       <c r="U20" s="3" t="n">
-        <v>0.02875</v>
+        <v>0.0345</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>gvrdkn</t>
+          <t>Rabie</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>20</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>0.134</v>
+        <v>0.147</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>0.00025</v>
@@ -1839,35 +1815,38 @@
       <c r="J21" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="K21" s="4" t="n">
+        <v>0.002</v>
+      </c>
       <c r="L21" s="4" t="n">
-        <v>0.001</v>
+        <v>0.00075</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>0.00225</v>
+        <v>0.002</v>
       </c>
       <c r="N21" s="4" t="n">
-        <v>0.00275</v>
+        <v>0.00425</v>
       </c>
       <c r="O21" s="4" t="n">
-        <v>0.005</v>
+        <v>0.007</v>
       </c>
       <c r="P21" s="4" t="n">
-        <v>0.01</v>
+        <v>0.01175</v>
       </c>
       <c r="Q21" s="4" t="n">
-        <v>0.01275</v>
+        <v>0.021</v>
       </c>
       <c r="R21" s="4" t="n">
-        <v>0.01375</v>
+        <v>0.01825</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.02175</v>
+        <v>0.02525</v>
       </c>
       <c r="T21" s="4" t="n">
-        <v>0.0325</v>
+        <v>0.03</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.03125</v>
+        <v>0.02375</v>
       </c>
     </row>
     <row r="22">
@@ -1880,43 +1859,49 @@
         <v>21</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>0.08271522788301899</v>
+        <v>0.09399999999999999</v>
       </c>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
       <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="n"/>
-      <c r="H22" s="2" t="n"/>
-      <c r="I22" s="2" t="n"/>
+      <c r="H22" s="3" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>0.00025</v>
+      </c>
       <c r="J22" s="3" t="n">
-        <v>0.0003121329354076188</v>
+        <v>0.00025</v>
       </c>
       <c r="K22" s="2" t="n"/>
       <c r="L22" s="2" t="n"/>
-      <c r="M22" s="2" t="n"/>
+      <c r="M22" s="3" t="n">
+        <v>0.00025</v>
+      </c>
       <c r="N22" s="3" t="n">
-        <v>0.001248531741630475</v>
+        <v>0.00125</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>0.001872797612445713</v>
+        <v>0.00375</v>
       </c>
       <c r="P22" s="3" t="n">
-        <v>0.002809196418668569</v>
+        <v>0.00575</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>0.00530625990192952</v>
+        <v>0.00725</v>
       </c>
       <c r="R22" s="3" t="n">
-        <v>0.0115489186100819</v>
+        <v>0.01375</v>
       </c>
       <c r="S22" s="3" t="n">
-        <v>0.01591877970578856</v>
+        <v>0.0155</v>
       </c>
       <c r="T22" s="3" t="n">
-        <v>0.01841584318904951</v>
+        <v>0.01875</v>
       </c>
       <c r="U22" s="3" t="n">
-        <v>0.02528276776801713</v>
+        <v>0.027</v>
       </c>
     </row>
     <row r="23">
@@ -1932,28 +1917,28 @@
         <v>0.08054808646256829</v>
       </c>
       <c r="P23" s="4" t="n">
-        <v>0.002301373898930523</v>
+        <v>0.002684936215418943</v>
       </c>
       <c r="Q23" s="4" t="n">
-        <v>0.002301373898930523</v>
+        <v>0.005369872430837886</v>
       </c>
       <c r="R23" s="4" t="n">
-        <v>0.009205495595722091</v>
+        <v>0.002684936215418943</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01380824339358314</v>
+        <v>0.008054808646256828</v>
       </c>
       <c r="T23" s="4" t="n">
-        <v>0.01380824339358314</v>
+        <v>0.02147948972335154</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.03912335628181889</v>
+        <v>0.04027404323128414</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>sfv</t>
+          <t>emilian_s</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1978,19 +1963,19 @@
       <c r="Q24" s="2" t="n"/>
       <c r="R24" s="2" t="n"/>
       <c r="S24" s="3" t="n">
-        <v>0.0156800418316979</v>
+        <v>0.007840020915848948</v>
       </c>
       <c r="T24" s="3" t="n">
+        <v>0.04704012549509369</v>
+      </c>
+      <c r="U24" s="3" t="n">
         <v>0.02352006274754685</v>
-      </c>
-      <c r="U24" s="3" t="n">
-        <v>0.03920010457924474</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>emilian_s</t>
+          <t>sfv</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -2000,16 +1985,16 @@
         <v>0.07627177032444879</v>
       </c>
       <c r="R25" s="4" t="n">
-        <v>0.005867059255726829</v>
+        <v>0.01271196172074147</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>0.005867059255726829</v>
+        <v>0.01271196172074147</v>
       </c>
       <c r="T25" s="4" t="n">
-        <v>0.02346823702290732</v>
+        <v>0.02542392344148293</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.04106941479008781</v>
+        <v>0.02542392344148293</v>
       </c>
     </row>
     <row r="26">
@@ -2260,7 +2245,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Suruchik</t>
+          <t>Ryumon_Hozukimaruu</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -2293,7 +2278,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Настя дай стек</t>
+          <t>Retbin</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2309,7 +2294,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Yars</t>
+          <t>Suruchik</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -2342,7 +2327,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Ryumon_Hozukimaruu</t>
+          <t>Yars</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2358,7 +2343,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Retbin</t>
+          <t>Davydovpussy</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2391,7 +2376,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>springbulk</t>
+          <t>Настя дай стек</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2407,7 +2392,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>БОЛЬШОЙ МИХА</t>
+          <t>Rik_dds</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2440,7 +2425,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Rik_dds</t>
+          <t>springbulk</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2456,7 +2441,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Davydovpussy</t>
+          <t>БОЛЬШОЙ МИХА</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2636,7 +2621,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>OlgaaGeorgieva</t>
+          <t>Бэндер</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2652,7 +2637,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Бэндер</t>
+          <t>OlgaaGeorgieva</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -2701,7 +2686,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>DARI</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -2734,7 +2719,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>DARI</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2848,7 +2833,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>elli</t>
+          <t>He3hAy</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -2881,7 +2866,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>He3hAy</t>
+          <t>elli</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -2930,7 +2915,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Mar_u_shka</t>
+          <t>repe_kate</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -2946,7 +2931,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>repe_kate</t>
+          <t>Mar_u_shka</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -3044,7 +3029,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Fara</t>
+          <t>Shuricspinoza</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -3077,7 +3062,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>edimerfi</t>
+          <t>twewefe</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3093,7 +3078,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Shuricspinoza</t>
+          <t>katerina_boc</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -3126,7 +3111,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>katerina_boc</t>
+          <t>edimerfi</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3142,7 +3127,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>twewefe</t>
+          <t>Schwepp1S</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -3175,7 +3160,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Schwepp1S</t>
+          <t>Fara</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3191,7 +3176,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>alinaadmv</t>
+          <t>nsa</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -3224,7 +3209,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>rus210385</t>
+          <t>frida_hk</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3240,7 +3225,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>frida_hk</t>
+          <t>alinaadmv</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -3273,7 +3258,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>nsa</t>
+          <t>DanilaOdinokov</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3289,7 +3274,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>DanilaOdinokov</t>
+          <t>rus210385</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">

</xml_diff>

<commit_message>
dynamic state update, advanced attendance model, improved forecasting
</commit_message>
<xml_diff>
--- a/data/playoff_odds.xlsx
+++ b/data/playoff_odds.xlsx
@@ -591,7 +591,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Noize MC</t>
+          <t>Драйв</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -601,583 +601,929 @@
         <v>0.25</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.17025</v>
+        <v>0.02875</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.065</v>
+        <v>0.03075</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.01425</v>
+        <v>0.0255</v>
       </c>
       <c r="G2" s="3" t="n">
+        <v>0.02025</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>0.01875</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>0.01525</v>
+      </c>
+      <c r="L2" s="3" t="n">
+        <v>0.01125</v>
+      </c>
+      <c r="M2" s="3" t="n">
+        <v>0.0135</v>
+      </c>
+      <c r="N2" s="3" t="n">
+        <v>0.0115</v>
+      </c>
+      <c r="O2" s="3" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="P2" s="3" t="n">
+        <v>0.008750000000000001</v>
+      </c>
+      <c r="Q2" s="3" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="R2" s="3" t="n">
+        <v>0.0045</v>
+      </c>
+      <c r="S2" s="3" t="n">
         <v>0.0005</v>
       </c>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="n"/>
-      <c r="O2" s="2" t="n"/>
-      <c r="P2" s="2" t="n"/>
-      <c r="Q2" s="2" t="n"/>
-      <c r="R2" s="2" t="n"/>
-      <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="n"/>
-      <c r="U2" s="2" t="n"/>
+      <c r="T2" s="3" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="U2" s="3" t="n">
+        <v>0.00075</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Драйв</t>
+          <t>Гризли</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>0.25</v>
+        <v>0.24975</v>
       </c>
       <c r="D3" s="4" t="n">
+        <v>0.0365</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>0.02775</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>0.02025</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>0.02525</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>0.02125</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>0.01925</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>0.0175</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>0.01725</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="M3" s="4" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="N3" s="4" t="n">
+        <v>0.01225</v>
+      </c>
+      <c r="O3" s="4" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="P3" s="4" t="n">
         <v>0.008</v>
       </c>
-      <c r="E3" s="4" t="n">
-        <v>0.04425</v>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>0.18675</v>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>0.01075</v>
-      </c>
-      <c r="H3" s="4" t="n">
-        <v>0.00025</v>
+      <c r="Q3" s="4" t="n">
+        <v>0.00425</v>
+      </c>
+      <c r="R3" s="4" t="n">
+        <v>0.00325</v>
+      </c>
+      <c r="S3" s="4" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="T3" s="4" t="n">
+        <v>0.00075</v>
+      </c>
+      <c r="U3" s="4" t="n">
+        <v>0.00075</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>long_2203</t>
+          <t>Noize MC</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
+        <v>0.24975</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0.0355</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.0285</v>
+      </c>
       <c r="F4" s="3" t="n">
-        <v>0.01225</v>
+        <v>0.03075</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0.20375</v>
+        <v>0.0205</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.03025</v>
+        <v>0.0185</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.00375</v>
-      </c>
-      <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="n"/>
-      <c r="L4" s="2" t="n"/>
-      <c r="M4" s="2" t="n"/>
-      <c r="N4" s="2" t="n"/>
-      <c r="O4" s="2" t="n"/>
-      <c r="P4" s="2" t="n"/>
-      <c r="Q4" s="2" t="n"/>
-      <c r="R4" s="2" t="n"/>
-      <c r="S4" s="2" t="n"/>
-      <c r="T4" s="2" t="n"/>
-      <c r="U4" s="2" t="n"/>
+        <v>0.0165</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0.01575</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>0.01125</v>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>0.01275</v>
+      </c>
+      <c r="N4" s="3" t="n">
+        <v>0.0115</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>0.008750000000000001</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>0.00775</v>
+      </c>
+      <c r="Q4" s="3" t="n">
+        <v>0.00925</v>
+      </c>
+      <c r="R4" s="3" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="S4" s="3" t="n">
+        <v>0.00325</v>
+      </c>
+      <c r="T4" s="3" t="n">
+        <v>0.00125</v>
+      </c>
+      <c r="U4" s="3" t="n">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>кинчоч</t>
+          <t>long_2203</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>0.25</v>
+        <v>0.24925</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>0.0235</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>0.02025</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>0.02375</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.0315</v>
+        <v>0.01875</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0.17625</v>
+        <v>0.022</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>0.042</v>
+        <v>0.0175</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>0.00025</v>
+        <v>0.019</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>0.01925</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="N5" s="4" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="O5" s="4" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>0.0115</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <v>0.00525</v>
+      </c>
+      <c r="R5" s="4" t="n">
+        <v>0.0035</v>
+      </c>
+      <c r="S5" s="4" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="T5" s="4" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="U5" s="4" t="n">
+        <v>0.0015</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Пассажир</t>
+          <t>terzzzzzzzzz</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
+        <v>0.24825</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.017</v>
+      </c>
       <c r="G6" s="3" t="n">
-        <v>0.003</v>
+        <v>0.01575</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.043</v>
+        <v>0.01375</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.196</v>
+        <v>0.0145</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.007</v>
+        <v>0.0175</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="L6" s="2" t="n"/>
-      <c r="M6" s="2" t="n"/>
-      <c r="N6" s="2" t="n"/>
-      <c r="O6" s="2" t="n"/>
-      <c r="P6" s="2" t="n"/>
-      <c r="Q6" s="2" t="n"/>
-      <c r="R6" s="2" t="n"/>
-      <c r="S6" s="2" t="n"/>
-      <c r="T6" s="2" t="n"/>
-      <c r="U6" s="2" t="n"/>
+        <v>0.01725</v>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>0.02125</v>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="N6" s="3" t="n">
+        <v>0.0195</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>0.0195</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>0.01675</v>
+      </c>
+      <c r="Q6" s="3" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="R6" s="3" t="n">
+        <v>0.0105</v>
+      </c>
+      <c r="S6" s="3" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="T6" s="3" t="n">
+        <v>0.0035</v>
+      </c>
+      <c r="U6" s="3" t="n">
+        <v>0.0025</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>лучший игрок</t>
+          <t>Пассажир</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>6</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>0.25</v>
+        <v>0.248</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>0.01925</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>0.02125</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>0.01925</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>0.02125</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>0.007</v>
+        <v>0.01875</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>0.15375</v>
+        <v>0.01825</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>0.066</v>
+        <v>0.0195</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>0.0175</v>
+        <v>0.014</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>0.00475</v>
+        <v>0.01425</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>0.00075</v>
+        <v>0.01375</v>
       </c>
       <c r="O7" s="4" t="n">
-        <v>0.00025</v>
+        <v>0.0165</v>
+      </c>
+      <c r="P7" s="4" t="n">
+        <v>0.0095</v>
+      </c>
+      <c r="Q7" s="4" t="n">
+        <v>0.008500000000000001</v>
+      </c>
+      <c r="R7" s="4" t="n">
+        <v>0.0045</v>
+      </c>
+      <c r="S7" s="4" t="n">
+        <v>0.0045</v>
+      </c>
+      <c r="T7" s="4" t="n">
+        <v>0.00125</v>
+      </c>
+      <c r="U7" s="4" t="n">
+        <v>0.00175</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>G_rant_999</t>
+          <t>Yanchik_250</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
         <v>7</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n"/>
+        <v>0.248</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0.00925</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0.0155</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>0.0145</v>
+      </c>
       <c r="I8" s="3" t="n">
-        <v>0.00125</v>
+        <v>0.0185</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.07124999999999999</v>
+        <v>0.01775</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>0.11275</v>
+        <v>0.01825</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>0.04275</v>
+        <v>0.02225</v>
       </c>
       <c r="M8" s="3" t="n">
+        <v>0.01875</v>
+      </c>
+      <c r="N8" s="3" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="O8" s="3" t="n">
+        <v>0.01775</v>
+      </c>
+      <c r="P8" s="3" t="n">
         <v>0.016</v>
       </c>
-      <c r="N8" s="3" t="n">
-        <v>0.0035</v>
-      </c>
-      <c r="O8" s="3" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="P8" s="2" t="n"/>
       <c r="Q8" s="3" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="R8" s="2" t="n"/>
-      <c r="S8" s="2" t="n"/>
-      <c r="T8" s="2" t="n"/>
-      <c r="U8" s="2" t="n"/>
+        <v>0.01225</v>
+      </c>
+      <c r="R8" s="3" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="S8" s="3" t="n">
+        <v>0.00475</v>
+      </c>
+      <c r="T8" s="3" t="n">
+        <v>0.00525</v>
+      </c>
+      <c r="U8" s="3" t="n">
+        <v>0.00275</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>dolMy</t>
+          <t>кинчоч</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>8</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>0.25</v>
+        <v>0.24775</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>0.0205</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>0.0215</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>0.02025</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>0.02325</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>0.0205</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>0.01925</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>0.0145</v>
+        <v>0.01675</v>
       </c>
       <c r="K9" s="4" t="n">
-        <v>0.044</v>
+        <v>0.01825</v>
       </c>
       <c r="L9" s="4" t="n">
-        <v>0.08925</v>
+        <v>0.0195</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>0.05525</v>
+        <v>0.01575</v>
       </c>
       <c r="N9" s="4" t="n">
-        <v>0.0215</v>
+        <v>0.014</v>
       </c>
       <c r="O9" s="4" t="n">
-        <v>0.01375</v>
+        <v>0.01075</v>
       </c>
       <c r="P9" s="4" t="n">
-        <v>0.00575</v>
+        <v>0.01075</v>
       </c>
       <c r="Q9" s="4" t="n">
-        <v>0.003</v>
+        <v>0.00775</v>
       </c>
       <c r="R9" s="4" t="n">
+        <v>0.00475</v>
+      </c>
+      <c r="S9" s="4" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="T9" s="4" t="n">
         <v>0.00125</v>
       </c>
-      <c r="S9" s="4" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="T9" s="4" t="n">
-        <v>0.00075</v>
+      <c r="U9" s="4" t="n">
+        <v>0.0005</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Гризли</t>
+          <t>Laches1</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
         <v>9</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.25</v>
+        <v>0.24775</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.07174999999999999</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.14075</v>
+        <v>0.014</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.03675</v>
+        <v>0.0125</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>0.0005</v>
+        <v>0.017</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.00025</v>
-      </c>
-      <c r="I10" s="2" t="n"/>
-      <c r="J10" s="2" t="n"/>
-      <c r="K10" s="2" t="n"/>
-      <c r="L10" s="2" t="n"/>
-      <c r="M10" s="2" t="n"/>
-      <c r="N10" s="2" t="n"/>
-      <c r="O10" s="2" t="n"/>
-      <c r="P10" s="2" t="n"/>
-      <c r="Q10" s="2" t="n"/>
-      <c r="R10" s="2" t="n"/>
-      <c r="S10" s="2" t="n"/>
-      <c r="T10" s="2" t="n"/>
-      <c r="U10" s="2" t="n"/>
+        <v>0.01725</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>0.01825</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>0.01675</v>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="M10" s="3" t="n">
+        <v>0.01725</v>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>0.01675</v>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>0.01825</v>
+      </c>
+      <c r="P10" s="3" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="Q10" s="3" t="n">
+        <v>0.01725</v>
+      </c>
+      <c r="R10" s="3" t="n">
+        <v>0.0095</v>
+      </c>
+      <c r="S10" s="3" t="n">
+        <v>0.00725</v>
+      </c>
+      <c r="T10" s="3" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="U10" s="3" t="n">
+        <v>0.00075</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Пиковая Дама</t>
+          <t>G_rant_999</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>10</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>0.24925</v>
+        <v>0.24725</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>0.0155</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>0.01625</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>0.01475</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>0.02025</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>0.018</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>0.00275</v>
+        <v>0.019</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>0.017</v>
+        <v>0.0165</v>
       </c>
       <c r="L11" s="4" t="n">
-        <v>0.047</v>
+        <v>0.021</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>0.067</v>
+        <v>0.01575</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>0.04575</v>
+        <v>0.02025</v>
       </c>
       <c r="O11" s="4" t="n">
-        <v>0.02825</v>
+        <v>0.0165</v>
       </c>
       <c r="P11" s="4" t="n">
-        <v>0.0165</v>
+        <v>0.01525</v>
       </c>
       <c r="Q11" s="4" t="n">
-        <v>0.01225</v>
+        <v>0.01</v>
       </c>
       <c r="R11" s="4" t="n">
-        <v>0.006</v>
+        <v>0.0065</v>
       </c>
       <c r="S11" s="4" t="n">
         <v>0.00425</v>
       </c>
       <c r="T11" s="4" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="U11" s="4" t="n">
         <v>0.0015</v>
-      </c>
-      <c r="U11" s="4" t="n">
-        <v>0.001</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Сокол</t>
+          <t>dolMy</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
         <v>11</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>0.2445</v>
-      </c>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n"/>
+        <v>0.24725</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>0.01375</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>0.0155</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>0.0195</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>0.01475</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>0.02075</v>
+      </c>
       <c r="J12" s="3" t="n">
-        <v>0.00025</v>
+        <v>0.01775</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0.0055</v>
+        <v>0.01775</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>0.0225</v>
+        <v>0.01675</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0.03</v>
+        <v>0.0165</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.049</v>
+        <v>0.01625</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.0355</v>
+        <v>0.01475</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>0.03575</v>
+        <v>0.01225</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>0.02675</v>
+        <v>0.01325</v>
       </c>
       <c r="R12" s="3" t="n">
-        <v>0.01625</v>
+        <v>0.00975</v>
       </c>
       <c r="S12" s="3" t="n">
-        <v>0.013</v>
+        <v>0.005</v>
       </c>
       <c r="T12" s="3" t="n">
-        <v>0.008</v>
+        <v>0.00425</v>
       </c>
       <c r="U12" s="3" t="n">
-        <v>0.002</v>
+        <v>0.00175</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>terzzzzzzzzz</t>
+          <t>Сокол</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>12</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>0.241</v>
+        <v>0.24725</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>0.0115</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>0.0155</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>0.01675</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>0.01625</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>0.00025</v>
+        <v>0.02325</v>
       </c>
       <c r="K13" s="4" t="n">
+        <v>0.02175</v>
+      </c>
+      <c r="L13" s="4" t="n">
+        <v>0.01625</v>
+      </c>
+      <c r="M13" s="4" t="n">
+        <v>0.0185</v>
+      </c>
+      <c r="N13" s="4" t="n">
+        <v>0.0175</v>
+      </c>
+      <c r="O13" s="4" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="P13" s="4" t="n">
+        <v>0.0135</v>
+      </c>
+      <c r="Q13" s="4" t="n">
+        <v>0.01075</v>
+      </c>
+      <c r="R13" s="4" t="n">
+        <v>0.00925</v>
+      </c>
+      <c r="S13" s="4" t="n">
+        <v>0.00625</v>
+      </c>
+      <c r="T13" s="4" t="n">
+        <v>0.0035</v>
+      </c>
+      <c r="U13" s="4" t="n">
         <v>0.00125</v>
-      </c>
-      <c r="L13" s="4" t="n">
-        <v>0.00975</v>
-      </c>
-      <c r="M13" s="4" t="n">
-        <v>0.0205</v>
-      </c>
-      <c r="N13" s="4" t="n">
-        <v>0.03275</v>
-      </c>
-      <c r="O13" s="4" t="n">
-        <v>0.03575</v>
-      </c>
-      <c r="P13" s="4" t="n">
-        <v>0.037</v>
-      </c>
-      <c r="Q13" s="4" t="n">
-        <v>0.032</v>
-      </c>
-      <c r="R13" s="4" t="n">
-        <v>0.02875</v>
-      </c>
-      <c r="S13" s="4" t="n">
-        <v>0.0205</v>
-      </c>
-      <c r="T13" s="4" t="n">
-        <v>0.0145</v>
-      </c>
-      <c r="U13" s="4" t="n">
-        <v>0.008</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>cheremsha</t>
+          <t>Lock</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
         <v>13</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>0.2355</v>
-      </c>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
-      <c r="J14" s="2" t="n"/>
+        <v>0.245</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>0.008500000000000001</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>0.0105</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0.01425</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>0.01325</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>0.01925</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>0.016</v>
+      </c>
       <c r="K14" s="3" t="n">
-        <v>0.001</v>
+        <v>0.01875</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.02</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0.01825</v>
+        <v>0.02125</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>0.02875</v>
+        <v>0.016</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>0.0365</v>
+        <v>0.016</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>0.03725</v>
+        <v>0.01925</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>0.03275</v>
+        <v>0.0115</v>
       </c>
       <c r="R14" s="3" t="n">
-        <v>0.02925</v>
+        <v>0.01125</v>
       </c>
       <c r="S14" s="3" t="n">
-        <v>0.02025</v>
+        <v>0.0065</v>
       </c>
       <c r="T14" s="3" t="n">
-        <v>0.01325</v>
+        <v>0.00425</v>
       </c>
       <c r="U14" s="3" t="n">
-        <v>0.00975</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Yanchik_250</t>
+          <t>Rabie</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>14</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>0.235</v>
+        <v>0.23775</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>0.00275</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>0.00525</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>0.00975</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>0.01175</v>
+      </c>
+      <c r="J15" s="4" t="n">
+        <v>0.01075</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>0.00075</v>
+        <v>0.0135</v>
       </c>
       <c r="L15" s="4" t="n">
-        <v>0.00675</v>
+        <v>0.016</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>0.01625</v>
+        <v>0.017</v>
       </c>
       <c r="N15" s="4" t="n">
-        <v>0.03325</v>
+        <v>0.0195</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>0.036</v>
+        <v>0.0205</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>0.034</v>
+        <v>0.025</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>0.033</v>
+        <v>0.023</v>
       </c>
       <c r="R15" s="4" t="n">
-        <v>0.02925</v>
+        <v>0.0165</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.02075</v>
+        <v>0.01325</v>
       </c>
       <c r="T15" s="4" t="n">
-        <v>0.0145</v>
+        <v>0.0105</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.0105</v>
+        <v>0.00825</v>
       </c>
     </row>
     <row r="16">
@@ -1190,282 +1536,342 @@
         <v>15</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>0.22</v>
+        <v>0.17125</v>
       </c>
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
-      <c r="G16" s="2" t="n"/>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
-      <c r="J16" s="2" t="n"/>
+      <c r="F16" s="3" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>0.00075</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>0.00125</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>0.0015</v>
+      </c>
       <c r="K16" s="3" t="n">
-        <v>0.0005</v>
+        <v>0.00275</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>0.003</v>
+        <v>0.00375</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0.011</v>
+        <v>0.00475</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0.0155</v>
+        <v>0.00625</v>
       </c>
       <c r="O16" s="3" t="n">
+        <v>0.00975</v>
+      </c>
+      <c r="P16" s="3" t="n">
+        <v>0.01225</v>
+      </c>
+      <c r="Q16" s="3" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="R16" s="3" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="S16" s="3" t="n">
+        <v>0.02875</v>
+      </c>
+      <c r="T16" s="3" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="U16" s="3" t="n">
         <v>0.02575</v>
-      </c>
-      <c r="P16" s="3" t="n">
-        <v>0.0235</v>
-      </c>
-      <c r="Q16" s="3" t="n">
-        <v>0.03325</v>
-      </c>
-      <c r="R16" s="3" t="n">
-        <v>0.0365</v>
-      </c>
-      <c r="S16" s="3" t="n">
-        <v>0.028</v>
-      </c>
-      <c r="T16" s="3" t="n">
-        <v>0.0255</v>
-      </c>
-      <c r="U16" s="3" t="n">
-        <v>0.0175</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Laches1</t>
+          <t>лучший игрок</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>16</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>0.211</v>
+        <v>0.153</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>0.00075</v>
+      </c>
+      <c r="J17" s="4" t="n">
+        <v>0.00125</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>0.00025</v>
+        <v>0.002</v>
       </c>
       <c r="L17" s="4" t="n">
-        <v>0.00275</v>
+        <v>0.0015</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>0.00725</v>
+        <v>0.00425</v>
       </c>
       <c r="N17" s="4" t="n">
-        <v>0.011</v>
+        <v>0.0065</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>0.02175</v>
+        <v>0.008</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>0.0285</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="Q17" s="4" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="R17" s="4" t="n">
+        <v>0.02425</v>
+      </c>
+      <c r="S17" s="4" t="n">
         <v>0.0305</v>
       </c>
-      <c r="R17" s="4" t="n">
-        <v>0.03075</v>
-      </c>
-      <c r="S17" s="4" t="n">
-        <v>0.033</v>
-      </c>
       <c r="T17" s="4" t="n">
-        <v>0.0285</v>
+        <v>0.02675</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.01675</v>
+        <v>0.02375</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>ksuhony</t>
+          <t>Пиковая Дама</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
         <v>17</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>0.16175</v>
+        <v>0.1315</v>
       </c>
       <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="n"/>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="n"/>
-      <c r="J18" s="2" t="n"/>
-      <c r="K18" s="2" t="n"/>
+      <c r="H18" s="3" t="n">
+        <v>0.00075</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="K18" s="3" t="n">
+        <v>0.00075</v>
+      </c>
       <c r="L18" s="3" t="n">
-        <v>0.00025</v>
+        <v>0.002</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>0.00225</v>
+        <v>0.00275</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>0.00375</v>
+        <v>0.00175</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>0.00675</v>
+        <v>0.00825</v>
       </c>
       <c r="P18" s="3" t="n">
-        <v>0.0145</v>
+        <v>0.00725</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>0.0155</v>
+        <v>0.011</v>
       </c>
       <c r="R18" s="3" t="n">
-        <v>0.02575</v>
+        <v>0.0185</v>
       </c>
       <c r="S18" s="3" t="n">
-        <v>0.0305</v>
+        <v>0.02175</v>
       </c>
       <c r="T18" s="3" t="n">
-        <v>0.03125</v>
+        <v>0.027</v>
       </c>
       <c r="U18" s="3" t="n">
-        <v>0.03125</v>
+        <v>0.029</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Lock</t>
+          <t>cheremsha</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
         <v>18</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.12</v>
+        <v>0.1175</v>
       </c>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
       <c r="F19" s="5" t="n"/>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="5" t="n"/>
+      <c r="G19" s="6" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="H19" s="6" t="n">
+        <v>0.00075</v>
+      </c>
       <c r="I19" s="5" t="n"/>
-      <c r="J19" s="5" t="n"/>
-      <c r="K19" s="5" t="n"/>
-      <c r="L19" s="5" t="n"/>
+      <c r="J19" s="6" t="n">
+        <v>0.00075</v>
+      </c>
+      <c r="K19" s="6" t="n">
+        <v>0.00075</v>
+      </c>
+      <c r="L19" s="6" t="n">
+        <v>0.00025</v>
+      </c>
       <c r="M19" s="6" t="n">
-        <v>0.0005</v>
+        <v>0.00275</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>0.00225</v>
+        <v>0.003</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>0.0025</v>
+        <v>0.0035</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>0.006</v>
+        <v>0.00625</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>0.00975</v>
+        <v>0.0095</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>0.01375</v>
+        <v>0.01775</v>
       </c>
       <c r="S19" s="6" t="n">
         <v>0.0185</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>0.03325</v>
+        <v>0.02425</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>0.0335</v>
+        <v>0.02925</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>gvrdkn</t>
+          <t>ksuhony</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
         <v>19</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>0.11375</v>
+        <v>0.115</v>
       </c>
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="n"/>
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="n"/>
       <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
-      <c r="J20" s="2" t="n"/>
-      <c r="K20" s="2" t="n"/>
-      <c r="L20" s="2" t="n"/>
+      <c r="I20" s="3" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="J20" s="3" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="K20" s="3" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="L20" s="3" t="n">
+        <v>0.00125</v>
+      </c>
       <c r="M20" s="3" t="n">
-        <v>0.00075</v>
+        <v>0.00175</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>0.00075</v>
+        <v>0.0025</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>0.002</v>
+        <v>0.0045</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>0.0065</v>
+        <v>0.00725</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>0.0095</v>
+        <v>0.012</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>0.01525</v>
+        <v>0.0145</v>
       </c>
       <c r="S20" s="3" t="n">
-        <v>0.02225</v>
+        <v>0.02125</v>
       </c>
       <c r="T20" s="3" t="n">
-        <v>0.02775</v>
+        <v>0.02175</v>
       </c>
       <c r="U20" s="3" t="n">
-        <v>0.029</v>
+        <v>0.027</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Rabie</t>
+          <t>nesmotri_v_shelll1</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>20</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>0.08490146367539786</v>
+        <v>0.1145</v>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>0.00125</v>
+      </c>
+      <c r="K21" s="4" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="L21" s="4" t="n">
+        <v>0.00075</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>0.0002858635140585786</v>
+        <v>0.0015</v>
       </c>
       <c r="N21" s="4" t="n">
-        <v>0.001715181084351472</v>
+        <v>0.00225</v>
       </c>
       <c r="O21" s="4" t="n">
-        <v>0.002572771626527207</v>
+        <v>0.00425</v>
       </c>
       <c r="P21" s="4" t="n">
-        <v>0.001715181084351472</v>
+        <v>0.005</v>
       </c>
       <c r="Q21" s="4" t="n">
-        <v>0.005145543253054415</v>
+        <v>0.01275</v>
       </c>
       <c r="R21" s="4" t="n">
-        <v>0.007718314879581623</v>
+        <v>0.016</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.01658008381539756</v>
+        <v>0.0195</v>
       </c>
       <c r="T21" s="4" t="n">
-        <v>0.02029630949815908</v>
+        <v>0.0245</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.02887221491991644</v>
+        <v>0.02625</v>
       </c>
     </row>
     <row r="22">
@@ -1478,76 +1884,107 @@
         <v>21</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>0.08271522788301899</v>
+        <v>0.104</v>
       </c>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
       <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="n"/>
       <c r="H22" s="2" t="n"/>
-      <c r="I22" s="2" t="n"/>
-      <c r="J22" s="2" t="n"/>
-      <c r="K22" s="2" t="n"/>
+      <c r="I22" s="3" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="J22" s="3" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="K22" s="3" t="n">
+        <v>0.00075</v>
+      </c>
       <c r="L22" s="2" t="n"/>
-      <c r="M22" s="2" t="n"/>
-      <c r="N22" s="2" t="n"/>
+      <c r="M22" s="3" t="n">
+        <v>0.00175</v>
+      </c>
+      <c r="N22" s="3" t="n">
+        <v>0.00125</v>
+      </c>
       <c r="O22" s="3" t="n">
-        <v>0.001434368113578364</v>
+        <v>0.00525</v>
       </c>
       <c r="P22" s="3" t="n">
-        <v>0.002390613522630607</v>
+        <v>0.00475</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>0.004303104340735092</v>
+        <v>0.0105</v>
       </c>
       <c r="R22" s="3" t="n">
-        <v>0.008128085976944064</v>
+        <v>0.013</v>
       </c>
       <c r="S22" s="3" t="n">
-        <v>0.01434368113578364</v>
+        <v>0.01975</v>
       </c>
       <c r="T22" s="3" t="n">
-        <v>0.01673429465841425</v>
+        <v>0.02275</v>
       </c>
       <c r="U22" s="3" t="n">
-        <v>0.03538108013493298</v>
+        <v>0.02375</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>sfv</t>
+          <t>gvrdkn</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>22</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>0.08054808646256829</v>
+        <v>0.08875</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="K23" s="4" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="L23" s="4" t="n">
+        <v>0.00125</v>
+      </c>
+      <c r="M23" s="4" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="N23" s="4" t="n">
+        <v>0.00225</v>
+      </c>
+      <c r="O23" s="4" t="n">
+        <v>0.00225</v>
       </c>
       <c r="P23" s="4" t="n">
-        <v>0.001776796024909595</v>
+        <v>0.00575</v>
       </c>
       <c r="Q23" s="4" t="n">
-        <v>0.004145857391455722</v>
+        <v>0.00625</v>
       </c>
       <c r="R23" s="4" t="n">
-        <v>0.00355359204981919</v>
+        <v>0.012</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01184530683273063</v>
+        <v>0.0165</v>
       </c>
       <c r="T23" s="4" t="n">
-        <v>0.02369061366546127</v>
+        <v>0.01725</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.0355359204981919</v>
+        <v>0.02225</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>nesmotri_v_shelll1</t>
+          <t>Julia_2499</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1563,28 +2000,34 @@
       <c r="H24" s="2" t="n"/>
       <c r="I24" s="2" t="n"/>
       <c r="J24" s="2" t="n"/>
-      <c r="K24" s="2" t="n"/>
+      <c r="K24" s="3" t="n">
+        <v>0.0008711134350943276</v>
+      </c>
       <c r="L24" s="2" t="n"/>
-      <c r="M24" s="2" t="n"/>
+      <c r="M24" s="3" t="n">
+        <v>0.0008711134350943276</v>
+      </c>
       <c r="N24" s="2" t="n"/>
-      <c r="O24" s="2" t="n"/>
+      <c r="O24" s="3" t="n">
+        <v>0.0008711134350943276</v>
+      </c>
       <c r="P24" s="3" t="n">
-        <v>0.002657634208762355</v>
+        <v>0.004355567175471638</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>0.003986451313143533</v>
+        <v>0.00348445374037731</v>
       </c>
       <c r="R24" s="3" t="n">
-        <v>0.005315268417524711</v>
+        <v>0.007840020915848948</v>
       </c>
       <c r="S24" s="3" t="n">
-        <v>0.01661021380476472</v>
+        <v>0.008711134350943277</v>
       </c>
       <c r="T24" s="3" t="n">
-        <v>0.01594580525257413</v>
+        <v>0.02439117618264117</v>
       </c>
       <c r="U24" s="3" t="n">
-        <v>0.03388483616172003</v>
+        <v>0.02700451648792416</v>
       </c>
     </row>
     <row r="25">
@@ -1599,26 +2042,32 @@
       <c r="C25" s="4" t="n">
         <v>0.07627177032444879</v>
       </c>
+      <c r="N25" s="4" t="n">
+        <v>0.002276769263416382</v>
+      </c>
+      <c r="P25" s="4" t="n">
+        <v>0.002276769263416382</v>
+      </c>
       <c r="Q25" s="4" t="n">
-        <v>0.003720574162168234</v>
+        <v>0.002276769263416382</v>
       </c>
       <c r="R25" s="4" t="n">
-        <v>0.0111617224865047</v>
+        <v>0.005691923158540954</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>0.007441148324336468</v>
+        <v>0.01593738484391467</v>
       </c>
       <c r="T25" s="4" t="n">
-        <v>0.01674258372975705</v>
+        <v>0.01593738484391467</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.03720574162168234</v>
+        <v>0.03187476968782935</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>1С</t>
+          <t>Davit</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1638,26 +2087,20 @@
       <c r="L26" s="2" t="n"/>
       <c r="M26" s="2" t="n"/>
       <c r="N26" s="2" t="n"/>
-      <c r="O26" s="3" t="n">
-        <v>0.00200440403069711</v>
-      </c>
+      <c r="O26" s="2" t="n"/>
       <c r="P26" s="2" t="n"/>
       <c r="Q26" s="2" t="n"/>
       <c r="R26" s="2" t="n"/>
-      <c r="S26" s="3" t="n">
-        <v>0.008017616122788439</v>
-      </c>
-      <c r="T26" s="3" t="n">
-        <v>0.02405284836836532</v>
-      </c>
+      <c r="S26" s="2" t="n"/>
+      <c r="T26" s="2" t="n"/>
       <c r="U26" s="3" t="n">
-        <v>0.04008808061394219</v>
+        <v>0.07416294913579306</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Julia_2499</t>
+          <t>bogdanov</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1666,29 +2109,23 @@
       <c r="C27" s="4" t="n">
         <v>0.07207392981597664</v>
       </c>
-      <c r="P27" s="4" t="n">
-        <v>0.002059255137599333</v>
-      </c>
-      <c r="Q27" s="4" t="n">
-        <v>0.002059255137599333</v>
+      <c r="O27" s="4" t="n">
+        <v>0.01201232163599611</v>
       </c>
       <c r="R27" s="4" t="n">
-        <v>0.004118510275198666</v>
-      </c>
-      <c r="S27" s="4" t="n">
-        <v>0.006177765412797998</v>
+        <v>0.01201232163599611</v>
       </c>
       <c r="T27" s="4" t="n">
-        <v>0.01647404110079466</v>
+        <v>0.02402464327199222</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.04118510275198665</v>
+        <v>0.02402464327199222</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>TryFraiz</t>
+          <t>sfv</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1710,26 +2147,18 @@
       <c r="N28" s="2" t="n"/>
       <c r="O28" s="2" t="n"/>
       <c r="P28" s="2" t="n"/>
-      <c r="Q28" s="3" t="n">
-        <v>0.005384992452166209</v>
-      </c>
-      <c r="R28" s="3" t="n">
-        <v>0.01076998490433242</v>
-      </c>
-      <c r="S28" s="3" t="n">
-        <v>0.01615497735649863</v>
-      </c>
-      <c r="T28" s="3" t="n">
-        <v>0.005384992452166209</v>
-      </c>
+      <c r="Q28" s="2" t="n"/>
+      <c r="R28" s="2" t="n"/>
+      <c r="S28" s="2" t="n"/>
+      <c r="T28" s="2" t="n"/>
       <c r="U28" s="3" t="n">
-        <v>0.03230995471299725</v>
+        <v>0.07000490187816071</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>bogdanov</t>
+          <t>.</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1738,26 +2167,14 @@
       <c r="C29" s="4" t="n">
         <v>0.06795606038331763</v>
       </c>
-      <c r="Q29" s="4" t="n">
-        <v>0.004530404025554508</v>
-      </c>
-      <c r="R29" s="4" t="n">
-        <v>0.004530404025554508</v>
-      </c>
-      <c r="S29" s="4" t="n">
-        <v>0.009060808051109016</v>
-      </c>
-      <c r="T29" s="4" t="n">
-        <v>0.009060808051109016</v>
-      </c>
       <c r="U29" s="4" t="n">
-        <v>0.04077363622999057</v>
+        <v>0.06795606038331763</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Davit</t>
+          <t>TryFraiz</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1781,20 +2198,16 @@
       <c r="P30" s="2" t="n"/>
       <c r="Q30" s="2" t="n"/>
       <c r="R30" s="2" t="n"/>
-      <c r="S30" s="3" t="n">
-        <v>0.02197586873877316</v>
-      </c>
-      <c r="T30" s="3" t="n">
-        <v>0.03296380310815974</v>
-      </c>
+      <c r="S30" s="2" t="n"/>
+      <c r="T30" s="2" t="n"/>
       <c r="U30" s="3" t="n">
-        <v>0.01098793436938658</v>
+        <v>0.06592760621631949</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Настя дай стек</t>
+          <t>1С</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1810,7 +2223,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>БОЛЬШОЙ МИХА</t>
+          <t>Suruchik</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1843,7 +2256,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Suruchik</t>
+          <t>Rik_dds</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1859,7 +2272,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>Son_Ton</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1901,14 +2314,14 @@
       <c r="C35" s="4" t="n">
         <v>0.05609862308114691</v>
       </c>
-      <c r="S35" s="4" t="n">
-        <v>0.05609862308114692</v>
+      <c r="U35" s="4" t="n">
+        <v>0.05609862308114691</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Son_Ton</t>
+          <t>Alina_97</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -1941,7 +2354,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Alina_97</t>
+          <t>БОЛЬШОЙ МИХА</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1957,7 +2370,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>springbulk</t>
+          <t>Аннэтт</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -1990,7 +2403,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Yars</t>
+          <t>springbulk</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2006,7 +2419,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Ryumon_Hozukimaruu</t>
+          <t>mflameee</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2039,7 +2452,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Аннэтт</t>
+          <t>Ryumon_Hozukimaruu</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2055,7 +2468,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rik_dds</t>
+          <t>Retbin</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2088,7 +2501,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>mflameee</t>
+          <t>Davydovpussy</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2104,7 +2517,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Retbin</t>
+          <t>Yars</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2137,7 +2550,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Davydovpussy</t>
+          <t>Настя дай стек</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2186,7 +2599,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>mrCelviano</t>
+          <t>Gur4an</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2202,7 +2615,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Gur4an</t>
+          <t>mrCelviano</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2235,7 +2648,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Qrexi</t>
+          <t>Бэндер</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2251,7 +2664,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Бэндер</t>
+          <t>Qrexi</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2431,7 +2844,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Vitos2049</t>
+          <t>He3hAy</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2447,7 +2860,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>He3hAy</t>
+          <t>elli</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -2480,7 +2893,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>elli</t>
+          <t>Vitos2049</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -2496,7 +2909,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>dance_with_vlad</t>
+          <t>imt360_ATDK</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -2529,7 +2942,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>imt360_ATDK</t>
+          <t>dance_with_vlad</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -2692,7 +3105,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Shuricspinoza</t>
+          <t>twewefe</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -2725,7 +3138,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>katerina_boc</t>
+          <t>Shuricspinoza</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -2741,7 +3154,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>twewefe</t>
+          <t>frida_hk</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -2774,7 +3187,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Fara</t>
+          <t>katerina_boc</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -2790,7 +3203,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Schwepp1S</t>
+          <t>edimerfi</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -2823,7 +3236,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>frida_hk</t>
+          <t>Fara</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -2839,7 +3252,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>edimerfi</t>
+          <t>Schwepp1S</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">

</xml_diff>